<commit_message>
📊 V9.2.1 daily run 2026-05-07_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -650,17 +650,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>4146</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -669,19 +669,19 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>14.82</v>
+        <v>43.19</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>14.05</v>
+        <v>41.21</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>15.64</v>
+        <v>44.99</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>16.28</v>
+        <v>46.41</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>28.95</v>
+        <v>32.16</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -692,7 +692,7 @@
         <v>0</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>14.82</v>
+        <v>43.19</v>
       </c>
       <c r="N4" s="7" t="n">
         <v>0</v>
@@ -717,17 +717,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -736,19 +736,19 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>126.35</v>
+        <v>137.37</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>119.79</v>
+        <v>130.48</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>132.8</v>
+        <v>143.72</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>137.82</v>
+        <v>148.68</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>22.11</v>
+        <v>30.86</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -759,7 +759,7 @@
         <v>0</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>126.35</v>
+        <v>137.37</v>
       </c>
       <c r="N5" s="7" t="n">
         <v>0</v>
@@ -784,17 +784,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2040</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -803,19 +803,19 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>30.86</v>
+        <v>27.31</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>29.38</v>
+        <v>25.97</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>32.22</v>
+        <v>28.55</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>33.28</v>
+        <v>29.51</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>21.92</v>
+        <v>26.27</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -826,7 +826,7 @@
         <v>0</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>30.86</v>
+        <v>27.31</v>
       </c>
       <c r="N6" s="7" t="n">
         <v>0</v>
@@ -851,38 +851,38 @@
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>198.4</v>
+        <v>37.25</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>188.1</v>
+        <v>35.32</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>211.52</v>
+        <v>39.15</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>221.65</v>
+        <v>40.63</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>21.42</v>
+        <v>23.8</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
@@ -893,7 +893,7 @@
         <v>0</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>198.4</v>
+        <v>37.25</v>
       </c>
       <c r="N7" s="7" t="n">
         <v>0</v>
@@ -918,38 +918,38 @@
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2190</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>34.61</v>
+        <v>26.25</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>32.81</v>
+        <v>24.89</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>36.49</v>
+        <v>28.16</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>37.96</v>
+        <v>29.62</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>20.64</v>
+        <v>16.26</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -960,7 +960,7 @@
         <v>0</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>34.61</v>
+        <v>26.25</v>
       </c>
       <c r="N8" s="7" t="n">
         <v>0</v>
@@ -985,38 +985,38 @@
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>4030</t>
+          <t>8280</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>37.03</v>
+        <v>10.7</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>35.11</v>
+        <v>10.15</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>38.99</v>
+        <v>11.29</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>40.52</v>
+        <v>11.75</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>19.54</v>
+        <v>12.8</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1027,7 +1027,7 @@
         <v>0</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>37.03</v>
+        <v>10.7</v>
       </c>
       <c r="N9" s="7" t="n">
         <v>0</v>
@@ -1052,38 +1052,38 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>1304</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>42</v>
+        <v>11.92</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>39.82</v>
+        <v>11.3</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>44.58</v>
+        <v>12.66</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>46.57</v>
+        <v>13.24</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>19.53</v>
+        <v>12</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1094,7 +1094,7 @@
         <v>0</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>42</v>
+        <v>11.92</v>
       </c>
       <c r="N10" s="7" t="n">
         <v>0</v>
@@ -1119,12 +1119,12 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2240</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1134,23 +1134,23 @@
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>39.68</v>
+        <v>26.89</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>37.62</v>
+        <v>25.86</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>42.02</v>
+        <v>27.82</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>43.83</v>
+        <v>28.55</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>19.07</v>
+        <v>10.63</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1161,7 +1161,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>39.68</v>
+        <v>26.89</v>
       </c>
       <c r="N11" s="7" t="n">
         <v>0</v>
@@ -1186,38 +1186,38 @@
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>31.46</v>
+        <v>105.01</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>29.83</v>
+        <v>99.56</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>33.48</v>
+        <v>110.66</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>35.04</v>
+        <v>115.06</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>16.42</v>
+        <v>10.01</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>31.46</v>
+        <v>105.01</v>
       </c>
       <c r="N12" s="7" t="n">
         <v>0</v>
@@ -1253,38 +1253,38 @@
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-01</t>
+          <t>2026-05-07</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>38.08</v>
+        <v>14.64</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>36.37</v>
+        <v>13.88</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>39.63</v>
+        <v>15.34</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>40.86</v>
+        <v>15.89</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>14.44</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1295,7 +1295,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>38.08</v>
+        <v>14.64</v>
       </c>
       <c r="N13" s="7" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-08_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -43,6 +43,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="001F4E78"/>
       <sz val="16"/>
     </font>
@@ -50,9 +53,6 @@
       <i val="1"/>
       <color rgb="00666666"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -147,17 +147,22 @@
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -689,19 +694,19 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>43.19</v>
+        <v>43.9</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O4" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P4" s="7" t="n">
-        <v>0</v>
+        <v>1.64</v>
+      </c>
+      <c r="O4" s="8" t="n">
+        <v>1.78</v>
+      </c>
+      <c r="P4" s="8" t="n">
+        <v>-0.16</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -756,19 +761,19 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>137.37</v>
+        <v>141.8</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O5" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P5" s="7" t="n">
-        <v>0</v>
+        <v>3.22</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="P5" s="8" t="n">
+        <v>-0.2</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -823,19 +828,19 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>27.31</v>
+        <v>27.9</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O6" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="7" t="n">
-        <v>0</v>
+        <v>2.16</v>
+      </c>
+      <c r="O6" s="8" t="n">
+        <v>3.92</v>
+      </c>
+      <c r="P6" s="8" t="n">
+        <v>-1.14</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -890,19 +895,19 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>37.25</v>
+        <v>38.48</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O7" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="7" t="n">
-        <v>0</v>
+        <v>3.3</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>3.36</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>-2.12</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -957,19 +962,19 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>26.25</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O8" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P8" s="7" t="n">
-        <v>0</v>
+        <v>25.8</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>-1.71</v>
+      </c>
+      <c r="O8" s="8" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="P8" s="8" t="n">
+        <v>-2.63</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -1024,19 +1029,19 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>10.7</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O9" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P9" s="7" t="n">
-        <v>0</v>
+        <v>10.6</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>-0.93</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>-0.93</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1047,7 +1052,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1057,33 +1062,33 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>11.3</v>
+        <v>99.56</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>12.66</v>
+        <v>110.66</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>13.24</v>
+        <v>115.06</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1091,19 +1096,19 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>11.92</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O10" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P10" s="7" t="n">
-        <v>0</v>
+        <v>102.9</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>-2.01</v>
+      </c>
+      <c r="O10" s="8" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="P10" s="8" t="n">
+        <v>-2.2</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1114,7 +1119,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0008</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1124,33 +1129,33 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>26.89</v>
+        <v>14.64</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>25.86</v>
+        <v>13.88</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>27.82</v>
+        <v>15.34</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>28.55</v>
+        <v>15.89</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10.63</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1158,19 +1163,19 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>26.89</v>
-      </c>
-      <c r="N11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="O11" s="7" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="7" t="n">
-        <v>0</v>
+        <v>14.63</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>-0.07000000000000001</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>0.34</v>
+      </c>
+      <c r="P11" s="8" t="n">
+        <v>-0.89</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1181,22 +1186,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1205,19 +1210,19 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>105.01</v>
+        <v>70.64</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>99.56</v>
+        <v>66.97</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>110.66</v>
+        <v>74.7</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>115.06</v>
+        <v>77.86</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>10.01</v>
+        <v>24.18</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1228,15 +1233,15 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>105.01</v>
-      </c>
-      <c r="N12" s="7" t="n">
+        <v>70.64</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O12" s="7" t="n">
+      <c r="O12" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="P12" s="7" t="n">
+      <c r="P12" s="8" t="n">
         <v>0</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
@@ -1248,43 +1253,43 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>13.88</v>
+        <v>173</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>15.34</v>
+        <v>191.75</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>15.89</v>
+        <v>198.98</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1295,15 +1300,15 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>14.64</v>
-      </c>
-      <c r="N13" s="7" t="n">
+        <v>182.46</v>
+      </c>
+      <c r="N13" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="O13" s="7" t="n">
+      <c r="O13" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="P13" s="7" t="n">
+      <c r="P13" s="8" t="n">
         <v>0</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
@@ -1326,7 +1331,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1420,6 +1425,138 @@
         <is>
           <t>ADX</t>
         </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K4" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M4" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O4" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P4" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>T0008</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G5" s="5" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>-0.0431</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>-0.08550000000000001</v>
+      </c>
+      <c r="O5" s="6" t="n">
+        <v>10.63</v>
+      </c>
+      <c r="P5" s="6" t="n">
+        <v>30.3</v>
       </c>
     </row>
   </sheetData>
@@ -1436,7 +1573,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E34"/>
+  <dimension ref="A1:E38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1444,44 +1581,44 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="8" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>📊 إحصاءات الأداء الإجمالي</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">محسوب في: </t>
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>محسوب في: 2026-05-08T02:02:46</t>
         </is>
       </c>
     </row>
     <row r="3"/>
     <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+      <c r="A4" s="13" t="inlineStr">
         <is>
           <t>المقياس</t>
         </is>
       </c>
-      <c r="B4" s="10" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>القيمة</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>إجمالي الصفقات</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="14" t="inlineStr">
         <is>
           <t>الصفقات النشطة</t>
         </is>
@@ -1491,7 +1628,7 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="14" t="inlineStr">
         <is>
           <t>الفائزة</t>
         </is>
@@ -1501,78 +1638,76 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="14" t="inlineStr">
         <is>
           <t>الخاسرة</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="14" t="inlineStr">
+        <is>
+          <t>Win Rate</t>
+        </is>
+      </c>
+      <c r="B9" s="15" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="14" t="inlineStr">
+        <is>
+          <t>متوسط الربح</t>
+        </is>
+      </c>
+      <c r="B10" s="15" t="inlineStr">
+        <is>
+          <t>+0%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="14" t="inlineStr">
+        <is>
+          <t>متوسط الخسارة</t>
+        </is>
+      </c>
+      <c r="B11" s="16" t="inlineStr">
+        <is>
+          <t>-4.99%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="14" t="inlineStr">
+        <is>
+          <t>Profit Factor</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="11" t="inlineStr">
-        <is>
-          <t>Win Rate</t>
-        </is>
-      </c>
-      <c r="B9" s="12" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="11" t="inlineStr">
-        <is>
-          <t>متوسط الربح</t>
-        </is>
-      </c>
-      <c r="B10" s="12" t="inlineStr">
-        <is>
-          <t>+0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="11" t="inlineStr">
-        <is>
-          <t>متوسط الخسارة</t>
-        </is>
-      </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>0%</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="11" t="inlineStr">
-        <is>
-          <t>Profit Factor</t>
-        </is>
-      </c>
-      <c r="B12" s="14" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-    </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>إجمالي P&amp;L%</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>0%</t>
+      <c r="B13" s="16" t="inlineStr">
+        <is>
+          <t>-9.99%</t>
         </is>
       </c>
     </row>
     <row r="14"/>
     <row r="15">
-      <c r="A15" s="15" t="inlineStr">
+      <c r="A15" s="18" t="inlineStr">
         <is>
           <t>🏆 أفضل صفقة</t>
         </is>
@@ -1581,18 +1716,18 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>- (-)</t>
-        </is>
-      </c>
-      <c r="B16" s="16" t="inlineStr">
-        <is>
-          <t>+0.00%</t>
+          <t>2050 (2026-05-08)</t>
+        </is>
+      </c>
+      <c r="B16" s="19" t="inlineStr">
+        <is>
+          <t>+-4.31%</t>
         </is>
       </c>
     </row>
     <row r="17"/>
     <row r="18">
-      <c r="A18" s="15" t="inlineStr">
+      <c r="A18" s="18" t="inlineStr">
         <is>
           <t>📉 أسوأ صفقة</t>
         </is>
@@ -1601,19 +1736,19 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>- (-)</t>
-        </is>
-      </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>0.00%</t>
+          <t>4040 (2026-05-08)</t>
+        </is>
+      </c>
+      <c r="B19" s="20" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="20"/>
     <row r="21"/>
     <row r="22">
-      <c r="A22" s="18" t="inlineStr">
+      <c r="A22" s="21" t="inlineStr">
         <is>
           <t>📈 الأداء حسب نوع الإشارة</t>
         </is>
@@ -1621,81 +1756,173 @@
     </row>
     <row r="23"/>
     <row r="24">
-      <c r="A24" s="19" t="inlineStr">
+      <c r="A24" s="22" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B24" s="19" t="inlineStr">
+      <c r="B24" s="22" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C24" s="19" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D24" s="19" t="inlineStr">
+      <c r="D24" s="22" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E24" s="19" t="inlineStr">
+      <c r="E24" s="22" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="25"/>
-    <row r="26"/>
-    <row r="27">
-      <c r="A27" s="18" t="inlineStr">
-        <is>
-          <t>🏢 الأداء حسب القطاع</t>
-        </is>
-      </c>
-    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="16" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E25" s="16" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="16" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27"/>
     <row r="28"/>
     <row r="29">
-      <c r="A29" s="19" t="inlineStr">
+      <c r="A29" s="21" t="inlineStr">
+        <is>
+          <t>🏢 الأداء حسب القطاع</t>
+        </is>
+      </c>
+    </row>
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B29" s="19" t="inlineStr">
+      <c r="B31" s="22" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C29" s="19" t="inlineStr">
+      <c r="C31" s="22" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D29" s="19" t="inlineStr">
+      <c r="D31" s="22" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E29" s="19" t="inlineStr">
+      <c r="E31" s="22" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31"/>
     <row r="32">
-      <c r="A32" s="20" t="inlineStr">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="16" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="16" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34"/>
+    <row r="35"/>
+    <row r="36">
+      <c r="A36" s="23" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34">
-      <c r="A34" s="21" t="inlineStr">
+    <row r="37"/>
+    <row r="38">
+      <c r="A38" s="24" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -1716,11 +1943,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
-    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1775,6 +2002,88 @@
       <c r="I3" s="2" t="inlineStr">
         <is>
           <t>Worst</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-10_08:28
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -694,16 +694,16 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>43.9</v>
+        <v>43.5</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>1.64</v>
+        <v>0.72</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1.78</v>
+        <v>1.88</v>
       </c>
       <c r="P4" s="8" t="n">
         <v>-0.16</v>
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>141.8</v>
+        <v>141.7</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>3.22</v>
+        <v>3.15</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>3.37</v>
+        <v>3.59</v>
       </c>
       <c r="P5" s="8" t="n">
         <v>-0.2</v>
@@ -828,13 +828,13 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>27.9</v>
+        <v>27.82</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>2.16</v>
+        <v>1.87</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>3.92</v>
@@ -895,16 +895,16 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>38.48</v>
+        <v>37.84</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>3.3</v>
+        <v>1.58</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>3.36</v>
+        <v>3.79</v>
       </c>
       <c r="P7" s="8" t="n">
         <v>-2.12</v>
@@ -962,13 +962,13 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>25.8</v>
+        <v>25.7</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-1.71</v>
+        <v>-2.1</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0.11</v>
@@ -1029,13 +1029,13 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>10.6</v>
-      </c>
-      <c r="N9" s="9" t="n">
-        <v>-0.93</v>
+        <v>10.73</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>0.28</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>1.68</v>
@@ -1096,13 +1096,13 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>102.9</v>
+        <v>104.4</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-2.01</v>
+        <v>-0.58</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0.75</v>
@@ -1163,19 +1163,19 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>14.63</v>
+        <v>14.54</v>
       </c>
       <c r="N11" s="9" t="n">
-        <v>-0.07000000000000001</v>
+        <v>-0.68</v>
       </c>
       <c r="O11" s="8" t="n">
         <v>0.34</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-0.89</v>
+        <v>-2.94</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1230,19 +1230,19 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>70.64</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>0</v>
+        <v>71.5</v>
+      </c>
+      <c r="N12" s="7" t="n">
+        <v>1.22</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>0</v>
+        <v>1.71</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0</v>
+        <v>-1.47</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1297,19 +1297,19 @@
         </is>
       </c>
       <c r="L13" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>182.46</v>
-      </c>
-      <c r="N13" s="8" t="n">
-        <v>0</v>
+        <v>185.2</v>
+      </c>
+      <c r="N13" s="7" t="n">
+        <v>1.5</v>
       </c>
       <c r="O13" s="8" t="n">
-        <v>0</v>
+        <v>3.15</v>
       </c>
       <c r="P13" s="8" t="n">
-        <v>0</v>
+        <v>-0.36</v>
       </c>
       <c r="Q13" s="3" t="inlineStr">
         <is>
@@ -1590,7 +1590,7 @@
     <row r="2">
       <c r="A2" s="12" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-08T02:02:46</t>
+          <t>محسوب في: 2026-05-10T08:28:40</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-11_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -166,18 +166,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -653,7 +653,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -663,33 +663,33 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>43.19</v>
+        <v>14.64</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>41.21</v>
+        <v>13.88</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>44.99</v>
+        <v>15.34</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>46.41</v>
+        <v>15.89</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>32.16</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -697,19 +697,19 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>43.64</v>
+        <v>14.58</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>1.04</v>
+        <v>-0.41</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1.88</v>
+        <v>0.34</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-0.16</v>
+        <v>-2.94</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -720,22 +720,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,19 +744,19 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>137.37</v>
+        <v>70.64</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>130.48</v>
+        <v>66.97</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>143.72</v>
+        <v>74.7</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>148.68</v>
+        <v>77.86</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>30.86</v>
+        <v>24.18</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -767,16 +767,16 @@
         <v>4</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>143.1</v>
+        <v>69.15000000000001</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>4.17</v>
+        <v>-2.11</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>4.32</v>
+        <v>1.78</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-0.2</v>
+        <v>-3.03</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -811,19 +811,19 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>27.31</v>
+        <v>182.46</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>25.97</v>
+        <v>173</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>28.55</v>
+        <v>191.75</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>29.51</v>
+        <v>198.98</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>26.27</v>
+        <v>23.45</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -834,16 +834,16 @@
         <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>28</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>2.53</v>
+        <v>185.1</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>1.45</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>3.92</v>
+        <v>3.15</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-1.14</v>
+        <v>-0.36</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -854,63 +854,63 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>37.25</v>
+        <v>14.05</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>35.32</v>
+        <v>13.32</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>39.15</v>
+        <v>15.09</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>40.63</v>
+        <v>15.89</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>23.8</v>
+        <v>14.88</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>36.94</v>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>-0.83</v>
+        <v>14</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>-0.36</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>3.79</v>
+        <v>0.36</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-2.12</v>
+        <v>-4.84</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -921,22 +921,22 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -945,39 +945,39 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>105.01</v>
+        <v>15.01</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>99.56</v>
+        <v>14.23</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>110.66</v>
+        <v>15.74</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>115.06</v>
+        <v>16.31</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.01</v>
+        <v>11.78</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>104.2</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>-0.77</v>
+        <v>14.66</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>-2.33</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.75</v>
+        <v>1.27</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.2</v>
+        <v>-3.06</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -988,63 +988,63 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>14.64</v>
+        <v>12.24</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>13.88</v>
+        <v>11.61</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>15.34</v>
+        <v>13.07</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>15.89</v>
+        <v>13.7</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>16.08</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>14.52</v>
-      </c>
-      <c r="N9" s="9" t="n">
-        <v>-0.82</v>
+        <v>12.24</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.34</v>
+        <v>0</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-2.94</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1055,22 +1055,22 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1079,39 +1079,39 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>70.64</v>
+        <v>25.85</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>66.97</v>
+        <v>24.88</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>74.7</v>
+        <v>26.72</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>77.86</v>
+        <v>27.41</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>24.18</v>
+        <v>14.35</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>70.2</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>-0.62</v>
+        <v>25.85</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>1.78</v>
+        <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-1.47</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,22 +1122,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,39 +1146,39 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>182.46</v>
+        <v>90.63</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>173</v>
+        <v>86.5</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>191.75</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>198.98</v>
+        <v>97.36</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>23.45</v>
+        <v>14.18</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>184.8</v>
-      </c>
-      <c r="N11" s="7" t="n">
-        <v>1.28</v>
+        <v>90.63</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>3.15</v>
+        <v>0</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-0.36</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1189,54 +1189,54 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>14.05</v>
+        <v>15.53</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>13.32</v>
+        <v>14.99</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>15.09</v>
+        <v>16.01</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>15.89</v>
+        <v>16.39</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>14.88</v>
+        <v>11.78</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>14.05</v>
+        <v>15.53</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1256,22 +1256,22 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1280,30 +1280,30 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>15.01</v>
+        <v>694.39</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>14.23</v>
+        <v>658.35</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>15.74</v>
+        <v>742</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>16.31</v>
+        <v>778.75</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>11.78</v>
+        <v>10.02</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>15.01</v>
+        <v>694.39</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P7"/>
+  <dimension ref="A1:P12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1433,7 +1433,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1443,39 +1443,39 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>26.25</v>
+        <v>43.19</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>25.64</v>
+        <v>43.88</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0232</v>
+        <v>0.016</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -1484,22 +1484,22 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0188</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0016</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>16.26</v>
+        <v>32.16</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>31.4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1509,12 +1509,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
@@ -1524,22 +1524,22 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>10.7</v>
+        <v>137.37</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>10.73</v>
+        <v>143</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -1550,22 +1550,22 @@
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0432</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.002</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>12.8</v>
+        <v>30.86</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>14.8</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1575,122 +1575,452 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>11.92</v>
+        <v>27.31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>11.24</v>
+        <v>27.86</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.0568</v>
+        <v>0.0201</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0</v>
+        <v>0.0392</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0114</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>12</v>
+        <v>26.27</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>33.5</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>T0004</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>2083</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
+          <t>مرافق</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>38.14</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>0.0379</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="O7" s="6" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="P7" s="6" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>T0009</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>105.01</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M8" s="8" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="N8" s="8" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="O8" s="6" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="P8" s="6" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E9" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L9" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O9" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P9" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M10" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O10" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P10" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O11" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P11" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D7" s="3" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
+      <c r="E12" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="F12" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G7" s="5" t="n">
+      <c r="G12" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H7" s="5" t="n">
+      <c r="H12" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="9" t="n">
+      <c r="I12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J12" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K7" s="10" t="inlineStr">
+      <c r="K12" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L7" s="4" t="inlineStr">
+      <c r="L12" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="8" t="n">
+      <c r="M12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N12" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="O12" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P7" s="6" t="n">
+      <c r="P12" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -1708,7 +2038,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1725,7 +2055,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-10T09:57:32</t>
+          <t>محسوب في: 2026-05-11T02:02:11</t>
         </is>
       </c>
     </row>
@@ -1749,7 +2079,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6">
@@ -1769,7 +2099,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
@@ -1779,7 +2109,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="9">
@@ -1790,7 +2120,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>55.6%</t>
         </is>
       </c>
     </row>
@@ -1802,7 +2132,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>+0.28%</t>
+          <t>+2.08%</t>
         </is>
       </c>
     </row>
@@ -1814,7 +2144,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-4.1%</t>
+          <t>-3.08%</t>
         </is>
       </c>
     </row>
@@ -1825,7 +2155,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.02</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="13">
@@ -1836,7 +2166,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-12.03%</t>
+          <t>-1.94%</t>
         </is>
       </c>
     </row>
@@ -1851,12 +2181,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8280 (2026-05-10)</t>
+          <t>8010 (2026-05-11)</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>+0.28%</t>
+          <t>+4.10%</t>
         </is>
       </c>
     </row>
@@ -1963,70 +2293,70 @@
         </is>
       </c>
     </row>
-    <row r="27"/>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>80.0%</t>
+        </is>
+      </c>
+      <c r="E27" s="16" t="inlineStr">
+        <is>
+          <t>+2.02%</t>
+        </is>
+      </c>
+    </row>
     <row r="28"/>
-    <row r="29">
-      <c r="A29" s="22" t="inlineStr">
+    <row r="29"/>
+    <row r="30">
+      <c r="A30" s="22" t="inlineStr">
         <is>
           <t>🏢 الأداء حسب القطاع</t>
         </is>
       </c>
     </row>
-    <row r="30"/>
-    <row r="31">
-      <c r="A31" s="23" t="inlineStr">
+    <row r="31"/>
+    <row r="32">
+      <c r="A32" s="23" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B31" s="23" t="inlineStr">
+      <c r="B32" s="23" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C31" s="23" t="inlineStr">
+      <c r="C32" s="23" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D31" s="23" t="inlineStr">
+      <c r="D32" s="23" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E31" s="23" t="inlineStr">
+      <c r="E32" s="23" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="32">
-      <c r="A32" t="inlineStr">
-        <is>
-          <t>نقل</t>
-        </is>
-      </c>
-      <c r="B32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C32" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D32" s="17" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E32" s="3" t="inlineStr">
-        <is>
-          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="B33" s="3" t="n">
@@ -2042,14 +2372,14 @@
       </c>
       <c r="E33" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
@@ -2065,45 +2395,137 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>تأمين</t>
         </is>
       </c>
-      <c r="B35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D35" s="16" t="inlineStr">
+      <c r="B36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="D36" s="16" t="inlineStr">
         <is>
           <t>100.0%</t>
         </is>
       </c>
-      <c r="E35" s="3" t="inlineStr">
-        <is>
-          <t>+0.28%</t>
-        </is>
-      </c>
-    </row>
-    <row r="36"/>
-    <row r="37"/>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>+2.13%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>زراعة وأغذية</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>+1.60%</t>
+        </is>
+      </c>
+    </row>
     <row r="38">
-      <c r="A38" s="24" t="inlineStr">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>مرافق</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>+2.39%</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C39" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>-0.01%</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41"/>
+    <row r="42">
+      <c r="A42" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="39"/>
-    <row r="40">
-      <c r="A40" s="25" t="inlineStr">
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="25" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -2124,7 +2546,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2230,123 +2652,328 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C5" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F5" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>0</v>
+      </c>
+      <c r="F5" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+1.60%</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+1.60%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+1.60%</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C6" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E6" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>0</v>
+      </c>
+      <c r="F6" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.10%</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.10%</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.10%</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
+          <t>8250</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>+2.01%</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>+2.01%</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>+2.01%</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>2083</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>مرافق</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>+2.39%</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>+2.39%</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>+2.39%</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>-5.68%</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>-4.31%</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>4145</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B11" s="4" t="inlineStr">
         <is>
           <t>صناعية</t>
         </is>
       </c>
-      <c r="C7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D7" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="3" t="inlineStr">
+      <c r="C11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>-2.32%</t>
         </is>
       </c>
-      <c r="H7" s="3" t="inlineStr">
+      <c r="H11" s="3" t="inlineStr">
         <is>
           <t>-2.32%</t>
         </is>
       </c>
-      <c r="I7" s="3" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr">
+        <is>
+          <t>-0.01%</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>-0.01%</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-12_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -150,10 +150,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -697,16 +697,16 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>14.58</v>
+        <v>14.51</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-0.41</v>
+        <v>-0.89</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>0.34</v>
+        <v>0.89</v>
       </c>
       <c r="P4" s="8" t="n">
         <v>-2.94</v>
@@ -720,22 +720,22 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,39 +744,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>70.64</v>
+        <v>15.01</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>66.97</v>
+        <v>14.23</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>74.7</v>
+        <v>15.74</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>77.86</v>
+        <v>16.31</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>53%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>69.15000000000001</v>
+        <v>14.68</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>-2.11</v>
+        <v>-2.2</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>1.78</v>
+        <v>1.27</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-3.03</v>
+        <v>-3.06</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -811,39 +811,39 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>182.46</v>
+        <v>12.24</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>173</v>
+        <v>11.61</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>191.75</v>
+        <v>13.07</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>198.98</v>
+        <v>13.7</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>23.45</v>
+        <v>16.08</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>185.1</v>
+        <v>12.72</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>1.45</v>
+        <v>3.92</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>3.15</v>
+        <v>6.62</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-0.36</v>
+        <v>-1.55</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -854,63 +854,63 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>14.05</v>
+        <v>25.85</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>13.32</v>
+        <v>24.88</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>15.09</v>
+        <v>26.72</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>15.89</v>
+        <v>27.41</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14.88</v>
+        <v>14.35</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>14</v>
+        <v>25.52</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>-0.36</v>
+        <v>-1.28</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>0.36</v>
+        <v>0</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-4.84</v>
+        <v>-1.97</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -921,22 +921,22 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -945,50 +945,50 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>15.01</v>
+        <v>90.63</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>14.23</v>
+        <v>86.5</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>15.74</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>16.31</v>
+        <v>97.36</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>14.66</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>-2.33</v>
+        <v>92.84999999999999</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>2.45</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>1.27</v>
+        <v>5.7</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-3.06</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -998,12 +998,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1012,50 +1012,50 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>12.24</v>
+        <v>15.53</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>11.61</v>
+        <v>14.99</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>13.07</v>
+        <v>16.01</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>13.7</v>
+        <v>16.39</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>16.08</v>
+        <v>11.78</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>12.24</v>
-      </c>
-      <c r="N9" s="8" t="n">
-        <v>0</v>
+        <v>15.99</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>2.96</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0</v>
+        <v>3.8</v>
       </c>
       <c r="P9" s="8" t="n">
         <v>0</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1065,12 +1065,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1079,39 +1079,39 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>25.85</v>
+        <v>694.39</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>24.88</v>
+        <v>658.35</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>26.72</v>
+        <v>742</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>27.41</v>
+        <v>778.75</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>14.35</v>
+        <v>10.02</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>25.85</v>
-      </c>
-      <c r="N10" s="8" t="n">
-        <v>0</v>
+        <v>698.5</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>0.59</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0</v>
+        <v>2.54</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0</v>
+        <v>-0.34</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,22 +1122,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,30 +1146,30 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>90.63</v>
+        <v>32.56</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>86.5</v>
+        <v>30.88</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>34.52</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>97.36</v>
+        <v>36.04</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>14.18</v>
+        <v>15.98</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>90.63</v>
+        <v>32.56</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1189,22 +1189,22 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
@@ -1213,30 +1213,30 @@
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>15.53</v>
+        <v>45.31</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>14.99</v>
+        <v>43.36</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>16.01</v>
+        <v>47.08</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>16.39</v>
+        <v>48.47</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>11.78</v>
+        <v>13.05</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>15.53</v>
+        <v>45.31</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1256,54 +1256,54 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>694.39</v>
+        <v>28.9</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>658.35</v>
+        <v>27.4</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>742</v>
+        <v>30.89</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>778.75</v>
+        <v>32.42</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>10.02</v>
+        <v>12.9</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>14%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>694.39</v>
+        <v>28.9</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P12"/>
+  <dimension ref="A1:P15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1433,27 +1433,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1462,20 +1462,20 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>43.19</v>
+        <v>70.64</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>43.88</v>
+        <v>69</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="9" t="n">
-        <v>0.016</v>
+      <c r="J4" s="7" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -1484,42 +1484,42 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0178</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0331</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>32.16</v>
+        <v>24.18</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>13</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1528,110 +1528,110 @@
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>137.37</v>
+        <v>182.46</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>143</v>
+        <v>198.78</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.106</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0036</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>30.86</v>
+        <v>23.45</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>22.9</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>27.31</v>
+        <v>14.05</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>27.86</v>
+        <v>13.25</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="9" t="n">
-        <v>0.0201</v>
+        <v>2</v>
+      </c>
+      <c r="J6" s="7" t="n">
+        <v>-0.0567</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0036</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.079</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>26.27</v>
+        <v>14.88</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>23.9</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1646,12 +1646,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1660,18 +1660,18 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>37.25</v>
+        <v>43.19</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>38.14</v>
+        <v>43.88</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
+        <v>0.016</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -1682,22 +1682,22 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0188</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0016</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>23.8</v>
+        <v>32.16</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>27.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1712,12 +1712,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1726,20 +1726,20 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>105.01</v>
+        <v>137.37</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>-0.0001</v>
+      <c r="J8" s="9" t="n">
+        <v>0.04099999999999999</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1748,22 +1748,22 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0432</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.002</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>10.01</v>
+        <v>30.86</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>17.6</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1773,39 +1773,39 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>26.25</v>
+        <v>27.31</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>25.64</v>
+        <v>27.86</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>-0.0232</v>
+        <v>5</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>0.0201</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -1814,22 +1814,22 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0392</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0114</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.26</v>
+        <v>26.27</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1839,37 +1839,37 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>10.7</v>
+        <v>37.25</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>10.73</v>
+        <v>38.14</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
+        <v>0.0239</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0379</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>14.8</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1905,122 +1905,320 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>11.24</v>
+        <v>105</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>-0.0568</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0001</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.022</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>33.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M12" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O12" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P12" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L13" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M14" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N14" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P14" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E12" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G12" s="5" t="n">
+      <c r="G15" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H12" s="5" t="n">
+      <c r="H15" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J12" s="7" t="n">
+      <c r="I15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L12" s="4" t="inlineStr">
+      <c r="L15" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M12" s="8" t="n">
+      <c r="M15" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N12" s="8" t="n">
+      <c r="N15" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O12" s="6" t="n">
+      <c r="O15" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P12" s="6" t="n">
+      <c r="P15" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2055,7 +2253,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-11T02:02:11</t>
+          <t>محسوب في: 2026-05-12T02:02:25</t>
         </is>
       </c>
     </row>
@@ -2079,7 +2277,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6">
@@ -2099,7 +2297,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="8">
@@ -2109,7 +2307,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="9">
@@ -2120,7 +2318,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>55.6%</t>
+          <t>50.0%</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2330,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>+2.08%</t>
+          <t>+3.22%</t>
         </is>
       </c>
     </row>
@@ -2144,7 +2342,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.08%</t>
+          <t>-3.38%</t>
         </is>
       </c>
     </row>
@@ -2155,7 +2353,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.84</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="13">
@@ -2166,7 +2364,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-1.94%</t>
+          <t>-0.99%</t>
         </is>
       </c>
     </row>
@@ -2181,12 +2379,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>8010 (2026-05-11)</t>
+          <t>2082 (2026-05-12)</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>+4.10%</t>
+          <t>+8.94%</t>
         </is>
       </c>
     </row>
@@ -2254,7 +2452,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0</v>
@@ -2266,7 +2464,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>
@@ -2300,19 +2498,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="C27" s="3" t="n">
-        <v>4</v>
-      </c>
       <c r="D27" s="16" t="inlineStr">
         <is>
-          <t>80.0%</t>
+          <t>71.4%</t>
         </is>
       </c>
       <c r="E27" s="16" t="inlineStr">
         <is>
-          <t>+2.02%</t>
+          <t>+2.39%</t>
         </is>
       </c>
     </row>
@@ -2383,7 +2581,7 @@
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0</v>
@@ -2395,7 +2593,7 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-3.31%</t>
         </is>
       </c>
     </row>
@@ -2452,19 +2650,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>+1.60%</t>
+          <t>-2.04%</t>
         </is>
       </c>
     </row>
@@ -2475,10 +2673,10 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="16" t="inlineStr">
         <is>
@@ -2487,7 +2685,7 @@
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>+2.39%</t>
+          <t>+5.67%</t>
         </is>
       </c>
     </row>
@@ -2546,7 +2744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -2816,53 +3014,53 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="C9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F9" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G9" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+8.94%</t>
         </is>
       </c>
       <c r="H9" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+8.94%</t>
         </is>
       </c>
       <c r="I9" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+8.94%</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
@@ -2881,29 +3079,29 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
@@ -2922,29 +3120,29 @@
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
@@ -2963,17 +3161,140 @@
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
+        <is>
           <t>-0.01%</t>
         </is>
       </c>
-      <c r="H12" s="3" t="inlineStr">
+      <c r="H13" s="3" t="inlineStr">
         <is>
           <t>-0.01%</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
+      <c r="I13" s="3" t="inlineStr">
         <is>
           <t>-0.01%</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>2320</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>6017</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>زراعة وأغذية</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G15" s="3" t="inlineStr">
+        <is>
+          <t>-5.67%</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>-5.67%</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-13_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -150,10 +150,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -166,18 +166,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -653,22 +653,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -677,50 +677,50 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>15.01</v>
+        <v>12.24</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>14.23</v>
+        <v>11.61</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>15.74</v>
+        <v>13.07</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>16.31</v>
+        <v>13.7</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>53%</t>
+          <t>69%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
         <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>14.68</v>
+        <v>13.02</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-2.2</v>
+        <v>6.37</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1.27</v>
+        <v>8.74</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-3.06</v>
+        <v>-1.55</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -730,12 +730,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,39 +744,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>12.24</v>
+        <v>25.85</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>11.61</v>
+        <v>24.88</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>13.07</v>
+        <v>26.72</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>13.7</v>
+        <v>27.41</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>16.08</v>
+        <v>14.35</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>67%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>12.72</v>
+        <v>25.28</v>
       </c>
       <c r="N5" s="9" t="n">
-        <v>3.92</v>
+        <v>-2.21</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>6.62</v>
+        <v>0</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-1.55</v>
+        <v>-2.21</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -787,7 +787,7 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -797,12 +797,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -811,50 +811,50 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>25.85</v>
+        <v>90.63</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>24.88</v>
+        <v>86.5</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>26.72</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>27.41</v>
+        <v>97.36</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>14.35</v>
+        <v>14.18</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>5%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>25.52</v>
+        <v>93.09999999999999</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>-1.28</v>
+        <v>2.73</v>
       </c>
       <c r="O6" s="8" t="n">
+        <v>5.7</v>
+      </c>
+      <c r="P6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="P6" s="8" t="n">
-        <v>-1.97</v>
-      </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -864,12 +864,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -878,36 +878,36 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>90.63</v>
+        <v>15.53</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>86.5</v>
+        <v>14.99</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>16.01</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>97.36</v>
+        <v>16.39</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14.18</v>
+        <v>11.78</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>94%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>92.84999999999999</v>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>2.45</v>
+        <v>15.82</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>1.87</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>5.7</v>
+        <v>3.8</v>
       </c>
       <c r="P7" s="8" t="n">
         <v>0</v>
@@ -921,7 +921,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -931,12 +931,12 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -945,65 +945,65 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>15.53</v>
+        <v>694.39</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>14.99</v>
+        <v>658.35</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>16.01</v>
+        <v>742</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>16.39</v>
+        <v>778.75</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>11.78</v>
+        <v>10.02</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>25%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>15.99</v>
+        <v>677</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>2.96</v>
+        <v>-2.5</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>3.8</v>
+        <v>2.54</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0</v>
+        <v>-2.86</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1012,39 +1012,39 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>694.39</v>
+        <v>100.3</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>658.35</v>
+        <v>95.5</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>742</v>
+        <v>104.7</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>778.75</v>
+        <v>108.16</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>10.02</v>
+        <v>9.9</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>698.5</v>
+        <v>96.5</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>0.59</v>
+        <v>-3.79</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>2.54</v>
+        <v>0.6</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-0.34</v>
+        <v>-4.19</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1055,7 +1055,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1065,53 +1065,53 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>28.9</v>
+        <v>45.31</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>27.4</v>
+        <v>43.36</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>30.89</v>
+        <v>47.08</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>32.42</v>
+        <v>48.47</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>12.9</v>
+        <v>12.84</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>14%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>28.84</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>-0.21</v>
+        <v>44.34</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>-2.14</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-4.36</v>
+        <v>-2.41</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,7 +1122,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1132,12 +1132,12 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,97 +1146,97 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>100.3</v>
+        <v>32.56</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>95.5</v>
+        <v>30.88</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>104.7</v>
+        <v>34.52</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>108.16</v>
+        <v>36.04</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>9.9</v>
+        <v>12.52</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>100.1</v>
+        <v>34.44</v>
       </c>
       <c r="N11" s="7" t="n">
-        <v>-0.2</v>
+        <v>5.77</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0.6</v>
+        <v>6.63</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-2.49</v>
+        <v>-0.12</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>45.31</v>
+        <v>15.33</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>43.36</v>
+        <v>14.54</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>47.08</v>
+        <v>16.61</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>48.47</v>
+        <v>17.6</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>12.84</v>
+        <v>9.57</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>45.31</v>
+        <v>15.33</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1256,17 +1256,17 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1276,34 +1276,34 @@
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>32.56</v>
+        <v>195.39</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>30.88</v>
+        <v>185.25</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>34.52</v>
+        <v>209.15</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>36.04</v>
+        <v>219.76</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>12.52</v>
+        <v>8.51</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="L13" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>32.56</v>
+        <v>195.39</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1334,7 +1334,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1433,27 +1433,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1462,16 +1462,16 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>70.64</v>
+        <v>15.01</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>69</v>
+        <v>14.34</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J4" s="7" t="n">
-        <v>-0.0232</v>
+      <c r="J4" s="9" t="n">
+        <v>-0.0446</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
@@ -1484,93 +1484,93 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0127</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0466</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>13.3</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>182.46</v>
+        <v>28.9</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>198.78</v>
+        <v>28.16</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+        <v>-0.0256</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0436</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>23.45</v>
+        <v>12.9</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>12.1</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1580,63 +1580,63 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>14.05</v>
+        <v>70.64</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>13.25</v>
+        <v>69</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>-0.0567</v>
+        <v>5</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0178</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0331</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>14.88</v>
+        <v>24.18</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>35.5</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1646,96 +1646,96 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>14.51</v>
+        <v>198.78</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.106</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0036</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>20.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>32.56</v>
+        <v>14.05</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>30.73</v>
+        <v>13.25</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>-0.0563</v>
+        <v>2</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>-0.0567</v>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
@@ -1748,88 +1748,88 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0036</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.079</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>15.98</v>
+        <v>14.88</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>43.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>-0.0478</v>
+        <v>7</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>-0.0089</v>
       </c>
       <c r="K9" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>13.05</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1844,12 +1844,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1858,16 +1858,16 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>-0.0478</v>
+      <c r="J10" s="9" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K10" s="10" t="inlineStr">
         <is>
@@ -1880,22 +1880,22 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.93</v>
+        <v>15.98</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1910,12 +1910,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1924,16 +1924,16 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>-0.0563</v>
+      <c r="J11" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
@@ -1946,37 +1946,37 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>12.53</v>
+        <v>13.05</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1990,64 +1990,64 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0478</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>32.16</v>
+        <v>12.93</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2056,44 +2056,44 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0563</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>30.86</v>
+        <v>12.53</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2108,12 +2108,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2122,16 +2122,16 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>27.31</v>
+        <v>43.19</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>27.86</v>
+        <v>43.88</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J14" s="9" t="n">
-        <v>0.0201</v>
+      <c r="J14" s="7" t="n">
+        <v>0.016</v>
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
@@ -2144,22 +2144,22 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0188</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0016</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>26.27</v>
+        <v>32.16</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>23.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2174,12 +2174,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2188,16 +2188,16 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>37.25</v>
+        <v>137.37</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>38.14</v>
+        <v>143</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J15" s="9" t="n">
-        <v>0.0239</v>
+      <c r="J15" s="7" t="n">
+        <v>0.04099999999999999</v>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
@@ -2210,22 +2210,22 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0432</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.002</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>23.8</v>
+        <v>30.86</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>27.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2240,12 +2240,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2254,20 +2254,20 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>105.01</v>
+        <v>27.31</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>105</v>
+        <v>27.86</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K16" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0201</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -2276,22 +2276,22 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0392</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0114</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>10.01</v>
+        <v>26.27</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>17.6</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2301,39 +2301,39 @@
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>26.25</v>
+        <v>37.25</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>25.64</v>
+        <v>38.14</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0239</v>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -2342,22 +2342,22 @@
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0379</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0212</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>16.26</v>
+        <v>23.8</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2367,39 +2367,39 @@
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>10.7</v>
+        <v>105.01</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>10.73</v>
+        <v>105</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0001</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -2408,22 +2408,22 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0075</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.022</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>12.8</v>
+        <v>10.01</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2433,122 +2433,254 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>-0.0568</v>
+        <v>4</v>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E20" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M20" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N20" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O20" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P20" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L21" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B22" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C22" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D22" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E20" s="4" t="inlineStr">
+      <c r="E22" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G20" s="5" t="n">
+      <c r="G22" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H20" s="5" t="n">
+      <c r="H22" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J20" s="7" t="n">
+      <c r="I22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K20" s="10" t="inlineStr">
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L20" s="4" t="inlineStr">
+      <c r="L22" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M20" s="8" t="n">
+      <c r="M22" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N20" s="8" t="n">
+      <c r="N22" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O20" s="6" t="n">
+      <c r="O22" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P20" s="6" t="n">
+      <c r="P22" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2566,7 +2698,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E45"/>
+  <dimension ref="A1:E46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2583,7 +2715,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-12T05:31:52</t>
+          <t>محسوب في: 2026-05-13T02:02:55</t>
         </is>
       </c>
     </row>
@@ -2607,7 +2739,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
@@ -2637,7 +2769,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
@@ -2648,7 +2780,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>35.3%</t>
+          <t>31.6%</t>
         </is>
       </c>
     </row>
@@ -2672,7 +2804,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.82%</t>
+          <t>-3.77%</t>
         </is>
       </c>
     </row>
@@ -2683,7 +2815,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.46</v>
+        <v>0.39</v>
       </c>
     </row>
     <row r="13">
@@ -2694,7 +2826,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-22.7%</t>
+          <t>-29.72%</t>
         </is>
       </c>
     </row>
@@ -2828,90 +2960,90 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>5</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>45.5%</t>
+          <t>41.7%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.37%</t>
-        </is>
-      </c>
-    </row>
-    <row r="28"/>
+          <t>-0.71%</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>mean_reversion</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E28" s="17" t="inlineStr">
+        <is>
+          <t>-2.56%</t>
+        </is>
+      </c>
+    </row>
     <row r="29"/>
-    <row r="30">
-      <c r="A30" s="22" t="inlineStr">
+    <row r="30"/>
+    <row r="31">
+      <c r="A31" s="22" t="inlineStr">
         <is>
           <t>🏢 الأداء حسب القطاع</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32">
-      <c r="A32" s="23" t="inlineStr">
+    <row r="32"/>
+    <row r="33">
+      <c r="A33" s="23" t="inlineStr">
         <is>
           <t>Signal Type</t>
         </is>
       </c>
-      <c r="B32" s="23" t="inlineStr">
+      <c r="B33" s="23" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="C32" s="23" t="inlineStr">
+      <c r="C33" s="23" t="inlineStr">
         <is>
           <t>Wins</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D33" s="23" t="inlineStr">
         <is>
           <t>Win Rate</t>
         </is>
       </c>
-      <c r="E32" s="23" t="inlineStr">
+      <c r="E33" s="23" t="inlineStr">
         <is>
           <t>Avg P&amp;L</t>
-        </is>
-      </c>
-    </row>
-    <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t>نقل</t>
-        </is>
-      </c>
-      <c r="B33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="C33" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D33" s="17" t="inlineStr">
-        <is>
-          <t>0.0%</t>
-        </is>
-      </c>
-      <c r="E33" s="3" t="inlineStr">
-        <is>
-          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="B34" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="C34" s="3" t="n">
         <v>0</v>
@@ -2923,18 +3055,18 @@
       </c>
       <c r="E34" s="3" t="inlineStr">
         <is>
-          <t>-4.47%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>0</v>
@@ -2946,106 +3078,106 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.09%</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+        <v>0</v>
+      </c>
+      <c r="D36" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>+2.13%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
         <v>4</v>
       </c>
       <c r="C37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D37" s="17" t="inlineStr">
-        <is>
-          <t>25.0%</t>
+        <v>3</v>
+      </c>
+      <c r="D37" s="16" t="inlineStr">
+        <is>
+          <t>75.0%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>+0.48%</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="D38" s="16" t="inlineStr">
-        <is>
-          <t>100.0%</t>
+        <v>1</v>
+      </c>
+      <c r="D38" s="17" t="inlineStr">
+        <is>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>+5.67%</t>
+          <t>-3.41%</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="B39" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C39" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D39" s="17" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>2</v>
+      </c>
+      <c r="D39" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>+5.67%</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="B40" s="3" t="n">
@@ -3061,22 +3193,45 @@
       </c>
       <c r="E40" s="3" t="inlineStr">
         <is>
+          <t>-0.01%</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>تجزئة</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C41" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D41" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
           <t>-0.89%</t>
         </is>
       </c>
     </row>
-    <row r="41"/>
     <row r="42"/>
-    <row r="43">
-      <c r="A43" s="24" t="inlineStr">
+    <row r="43"/>
+    <row r="44">
+      <c r="A44" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="44"/>
-    <row r="45">
-      <c r="A45" s="25" t="inlineStr">
+    <row r="45"/>
+    <row r="46">
+      <c r="A46" s="25" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -3097,7 +3252,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3774,6 +3929,88 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>8030</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>2170</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>-2.56%</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>-2.56%</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>-2.56%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-14_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -86,12 +86,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -166,18 +166,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -549,7 +549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:Q11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -653,22 +653,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -677,65 +677,65 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>12.24</v>
+        <v>100.3</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>11.61</v>
+        <v>95.5</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>13.07</v>
+        <v>104.7</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>13.7</v>
+        <v>108.16</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>16.08</v>
+        <v>9.9</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>69%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>13.02</v>
+        <v>97.34999999999999</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>6.37</v>
+        <v>-2.94</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>8.74</v>
+        <v>0.6</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-1.55</v>
+        <v>-4.19</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,39 +744,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>25.85</v>
+        <v>45.31</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>24.88</v>
+        <v>43.36</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>26.72</v>
+        <v>47.08</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>27.41</v>
+        <v>48.47</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>14.35</v>
+        <v>12.84</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>67%</t>
+          <t>52%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>25.28</v>
-      </c>
-      <c r="N5" s="9" t="n">
-        <v>-2.21</v>
+        <v>43.68</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>-3.6</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-2.21</v>
+        <v>-3.6</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -787,22 +787,22 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -811,39 +811,39 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>90.63</v>
+        <v>32.56</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>86.5</v>
+        <v>30.88</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>34.52</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>97.36</v>
+        <v>36.04</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>14.18</v>
+        <v>12.52</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>5%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>93.09999999999999</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>2.73</v>
+        <v>34</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>4.42</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>5.7</v>
+        <v>6.63</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>0</v>
+        <v>-0.12</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -854,130 +854,130 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>15.53</v>
+        <v>15.33</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>14.99</v>
+        <v>14.54</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>16.01</v>
+        <v>16.61</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>16.39</v>
+        <v>17.6</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>11.78</v>
+        <v>9.57</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>94%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>15.82</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>1.87</v>
+        <v>16</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>4.37</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>3.8</v>
+        <v>5.15</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>0</v>
+        <v>-0.33</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>694.39</v>
+        <v>195.39</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>658.35</v>
+        <v>185.25</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>742</v>
+        <v>209.15</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>778.75</v>
+        <v>219.76</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.02</v>
+        <v>8.51</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>25%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>677</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>-2.5</v>
+        <v>192.1</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>-1.68</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>2.54</v>
+        <v>0.21</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.86</v>
+        <v>-2.66</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -988,63 +988,63 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>100.3</v>
+        <v>128.16</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>95.5</v>
+        <v>121.51</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>104.7</v>
+        <v>135.22</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>108.16</v>
+        <v>140.71</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>9.9</v>
+        <v>5.12</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>96.5</v>
-      </c>
-      <c r="N9" s="9" t="n">
-        <v>-3.79</v>
+        <v>128.16</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.6</v>
+        <v>0</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-4.19</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1055,63 +1055,63 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>43.36</v>
+        <v>13.88</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>47.08</v>
+        <v>15.47</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>48.47</v>
+        <v>16.12</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>12.84</v>
+        <v>3.78</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>44.34</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>-2.14</v>
+        <v>14.64</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-2.41</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,17 +1122,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1146,175 +1146,41 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>32.56</v>
+        <v>158.92</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>30.88</v>
+        <v>150.69</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>34.52</v>
+        <v>166.51</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>36.04</v>
+        <v>172.44</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>12.52</v>
+        <v>3.46</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>34.44</v>
-      </c>
-      <c r="N11" s="7" t="n">
-        <v>5.77</v>
+        <v>158.92</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>6.63</v>
+        <v>0</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-0.12</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
-        <is>
-          <t>🟡 Partial</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="3" t="inlineStr">
-        <is>
-          <t>T0028</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>2380</t>
-        </is>
-      </c>
-      <c r="D12" s="4" t="inlineStr">
-        <is>
-          <t>بتروكيماويات</t>
-        </is>
-      </c>
-      <c r="E12" s="3" t="inlineStr">
-        <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>15.33</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>14.54</v>
-      </c>
-      <c r="H12" s="5" t="n">
-        <v>16.61</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>17.6</v>
-      </c>
-      <c r="J12" s="6" t="n">
-        <v>9.57</v>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>44%</t>
-        </is>
-      </c>
-      <c r="L12" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>15.33</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="3" t="inlineStr">
-        <is>
-          <t>🟢 Active</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>T0029</t>
-        </is>
-      </c>
-      <c r="B13" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-13</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>1321</t>
-        </is>
-      </c>
-      <c r="D13" s="4" t="inlineStr">
-        <is>
-          <t>بتروكيماويات</t>
-        </is>
-      </c>
-      <c r="E13" s="3" t="inlineStr">
-        <is>
-          <t>default</t>
-        </is>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>195.39</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>185.25</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>209.15</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>219.76</v>
-      </c>
-      <c r="J13" s="6" t="n">
-        <v>8.51</v>
-      </c>
-      <c r="K13" s="3" t="inlineStr">
-        <is>
-          <t>29%</t>
-        </is>
-      </c>
-      <c r="L13" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>195.39</v>
-      </c>
-      <c r="N13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="O13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>🟢 Active</t>
         </is>
@@ -1334,7 +1200,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P22"/>
+  <dimension ref="A1:P27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1433,27 +1299,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1462,20 +1328,20 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>15.01</v>
+        <v>12.24</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>14.34</v>
+        <v>12.9</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0446</v>
+        <v>0.0609</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -1484,62 +1350,62 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0466</v>
+        <v>-0.0155</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>11.8</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>28.9</v>
+        <v>25.85</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>28.16</v>
+        <v>25.22</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>-0.0256</v>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1553,39 +1419,39 @@
         <v>0</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0352</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>12.9</v>
+        <v>14.35</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>32.8</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1594,20 +1460,20 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>70.64</v>
+        <v>90.63</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>69</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.0232</v>
+        <v>0.0416</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -1616,42 +1482,42 @@
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.057</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0331</v>
+        <v>0</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>24.18</v>
+        <v>14.18</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>13.3</v>
+        <v>23</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1660,150 +1526,150 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>182.46</v>
+        <v>15.53</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>198.78</v>
+        <v>15.88</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J7" s="7" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+      <c r="J7" s="9" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.106</v>
+        <v>0.038</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0036</v>
+        <v>0</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>23.45</v>
+        <v>11.78</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>12.1</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>14.05</v>
+        <v>694.39</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>13.25</v>
+        <v>680</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0254</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0517</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>14.88</v>
+        <v>10.02</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>35.5</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>14.64</v>
+        <v>15.01</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>14.51</v>
+        <v>14.34</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>-0.0446</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1814,22 +1680,22 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0127</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0466</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>11.78</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>20.2</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1839,12 +1705,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1854,68 +1720,68 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>32.56</v>
+        <v>28.9</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>30.73</v>
+        <v>28.16</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>3</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0436</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>15.98</v>
+        <v>12.9</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>43.3</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1924,64 +1790,64 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>45.31</v>
+        <v>70.64</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>43.14</v>
+        <v>69</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J11" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0</v>
+        <v>0.0178</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0331</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>13.05</v>
+        <v>24.18</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>28.7</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C12" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1990,84 +1856,84 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>45.31</v>
+        <v>182.46</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>43.14</v>
+        <v>198.78</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>-0.0478</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0</v>
+        <v>0.106</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0036</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>12.93</v>
+        <v>23.45</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>28.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>32.56</v>
+        <v>14.05</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>30.73</v>
+        <v>13.25</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J13" s="9" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>-0.0567</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2078,22 +1944,22 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0036</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.079</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>12.53</v>
+        <v>14.88</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>43.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2103,39 +1969,39 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>43.19</v>
+        <v>14.64</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>43.88</v>
+        <v>14.51</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>0.016</v>
+        <v>-0.0089</v>
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -2144,42 +2010,42 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0089</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0294</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>32.16</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>13</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2188,64 +2054,64 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>0.04099999999999999</v>
+        <v>-0.0563</v>
       </c>
       <c r="K15" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>30.86</v>
+        <v>15.98</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2254,64 +2120,64 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>27.31</v>
+        <v>45.31</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>27.86</v>
+        <v>43.14</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>0.0201</v>
+        <v>-0.0478</v>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0392</v>
+        <v>0</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0925</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>26.27</v>
+        <v>13.05</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>23.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2320,64 +2186,64 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>37.25</v>
+        <v>45.31</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>38.14</v>
+        <v>43.14</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>0.0239</v>
+        <v>-0.0478</v>
       </c>
       <c r="K17" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.0379</v>
+        <v>0</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0925</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>23.8</v>
+        <v>12.93</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>27.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2386,44 +2252,44 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>105.01</v>
+        <v>32.56</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>105</v>
+        <v>30.73</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J18" s="9" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>1</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0608</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>10.01</v>
+        <v>12.53</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>17.6</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2433,39 +2299,39 @@
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>26.25</v>
+        <v>43.19</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>25.64</v>
+        <v>43.88</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-0.0232</v>
+        <v>0.016</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -2474,22 +2340,22 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0188</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0016</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>16.26</v>
+        <v>32.16</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>31.4</v>
+        <v>13</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2499,12 +2365,12 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2514,22 +2380,22 @@
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>10.7</v>
+        <v>137.37</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>10.73</v>
+        <v>143</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -2540,22 +2406,22 @@
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0432</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.002</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>12.8</v>
+        <v>30.86</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>14.8</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2565,122 +2431,452 @@
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>11.92</v>
+        <v>27.31</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>11.24</v>
+        <v>27.86</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>-0.0568</v>
+        <v>0.0201</v>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0</v>
+        <v>0.0392</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0114</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>12</v>
+        <v>26.27</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>33.5</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
+          <t>T0004</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>2083</t>
+        </is>
+      </c>
+      <c r="E22" s="4" t="inlineStr">
+        <is>
+          <t>مرافق</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>37.25</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>38.14</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J22" s="9" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M22" s="8" t="n">
+        <v>0.0379</v>
+      </c>
+      <c r="N22" s="8" t="n">
+        <v>-0.0212</v>
+      </c>
+      <c r="O22" s="6" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="P22" s="6" t="n">
+        <v>27.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>T0009</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="E23" s="4" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>105.01</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J23" s="7" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L23" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="P23" s="6" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E24" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M24" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N24" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P24" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E25" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L25" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P25" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M26" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N26" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P26" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B27" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C27" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E22" s="4" t="inlineStr">
+      <c r="E27" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
+      <c r="F27" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G22" s="5" t="n">
+      <c r="G27" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H22" s="5" t="n">
+      <c r="H27" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J22" s="9" t="n">
+      <c r="I27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K22" s="10" t="inlineStr">
+      <c r="K27" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L22" s="4" t="inlineStr">
+      <c r="L27" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M22" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N22" s="8" t="n">
+      <c r="M27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N27" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O22" s="6" t="n">
+      <c r="O27" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P22" s="6" t="n">
+      <c r="P27" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2698,7 +2894,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E46"/>
+  <dimension ref="A1:E49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2715,7 +2911,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-13T02:02:55</t>
+          <t>محسوب في: 2026-05-14T02:02:56</t>
         </is>
       </c>
     </row>
@@ -2739,7 +2935,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
     </row>
     <row r="6">
@@ -2749,7 +2945,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="7">
@@ -2759,7 +2955,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -2769,7 +2965,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>13</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
@@ -2780,7 +2976,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>31.6%</t>
+          <t>37.5%</t>
         </is>
       </c>
     </row>
@@ -2792,7 +2988,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>+3.22%</t>
+          <t>+3.58%</t>
         </is>
       </c>
     </row>
@@ -2804,7 +3000,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.77%</t>
+          <t>-3.57%</t>
         </is>
       </c>
     </row>
@@ -2815,7 +3011,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.39</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="13">
@@ -2826,7 +3022,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-29.72%</t>
+          <t>-21.31%</t>
         </is>
       </c>
     </row>
@@ -2960,19 +3156,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>41.7%</t>
+          <t>47.1%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.71%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
@@ -3089,19 +3285,19 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C36" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D36" s="17" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>+1.89%</t>
         </is>
       </c>
     </row>
@@ -3220,18 +3416,87 @@
         </is>
       </c>
     </row>
-    <row r="42"/>
-    <row r="43"/>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>أسمنت</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>+0.11%</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>فنادق</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C43" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D43" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>+4.16%</t>
+        </is>
+      </c>
+    </row>
     <row r="44">
-      <c r="A44" s="24" t="inlineStr">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>تقنية</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C44" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>-2.07%</t>
+        </is>
+      </c>
+    </row>
+    <row r="45"/>
+    <row r="46"/>
+    <row r="47">
+      <c r="A47" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="45"/>
-    <row r="46">
-      <c r="A46" s="25" t="inlineStr">
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="25" t="inlineStr">
         <is>
           <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
         </is>
@@ -3252,7 +3517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I20"/>
+  <dimension ref="A1:I25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -3563,135 +3828,135 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>0</v>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+6.09%</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+6.09%</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+6.09%</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="C11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F11" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>0</v>
+      </c>
+      <c r="F11" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G11" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.16%</t>
         </is>
       </c>
       <c r="H11" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.16%</t>
         </is>
       </c>
       <c r="I11" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>+4.16%</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="C12" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E12" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>0</v>
+      </c>
+      <c r="F12" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>+2.67%</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>+2.67%</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>+2.67%</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C13" s="3" t="n">
@@ -3710,24 +3975,24 @@
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
@@ -3751,29 +4016,29 @@
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -3792,29 +4057,29 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -3833,24 +4098,24 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
@@ -3859,13 +4124,13 @@
         </is>
       </c>
       <c r="C17" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D17" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E17" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
@@ -3874,24 +4139,24 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
@@ -3900,13 +4165,13 @@
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D18" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E18" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
@@ -3915,29 +4180,29 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -3956,58 +4221,263 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-0.89%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
+          <t>2370</t>
+        </is>
+      </c>
+      <c r="B20" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>-5.63%</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>2280</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t>زراعة وأغذية</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>-4.78%</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>8030</t>
+        </is>
+      </c>
+      <c r="B22" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>-4.46%</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
           <t>2170</t>
         </is>
       </c>
-      <c r="B20" s="4" t="inlineStr">
+      <c r="B23" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="C20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D20" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E20" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F20" s="3" t="inlineStr">
+      <c r="C23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>-2.56%</t>
         </is>
       </c>
-      <c r="H20" s="3" t="inlineStr">
+      <c r="H23" s="3" t="inlineStr">
         <is>
           <t>-2.56%</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
+      <c r="I23" s="3" t="inlineStr">
         <is>
           <t>-2.56%</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>3080</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>أسمنت</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>-2.44%</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>-2.44%</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>-2.44%</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>7203</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="inlineStr">
+        <is>
+          <t>تقنية</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>-2.07%</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>-2.07%</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>-2.07%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-15_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -23,7 +23,7 @@
     <numFmt numFmtId="164" formatCode="0.0"/>
     <numFmt numFmtId="165" formatCode="+0.00%;-0.00%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -66,10 +66,6 @@
       <b val="1"/>
       <color rgb="00C00000"/>
       <sz val="12"/>
-    </font>
-    <font>
-      <i val="1"/>
-      <color rgb="00666666"/>
     </font>
   </fonts>
   <fills count="7">
@@ -131,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -150,10 +146,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -183,7 +179,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -549,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q11"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -697,13 +692,13 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>97.34999999999999</v>
+        <v>98</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-2.94</v>
+        <v>-2.29</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>0.6</v>
@@ -720,7 +715,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -730,12 +725,12 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
@@ -744,60 +739,60 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>43.36</v>
+        <v>30.88</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>47.08</v>
+        <v>34.52</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>48.47</v>
+        <v>36.04</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>12.84</v>
+        <v>12.52</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>52%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>43.68</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>-3.6</v>
+        <v>33.22</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>2.03</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>0</v>
+        <v>6.63</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-3.6</v>
+        <v>-0.12</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -807,54 +802,54 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>32.56</v>
+        <v>15.33</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>30.88</v>
+        <v>14.54</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>34.52</v>
+        <v>16.61</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>36.04</v>
+        <v>17.6</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>12.52</v>
+        <v>9.57</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>34</v>
+        <v>15.99</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>4.42</v>
+        <v>4.31</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>6.63</v>
+        <v>6.33</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-0.12</v>
+        <v>-0.33</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -864,7 +859,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -878,39 +873,39 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>15.33</v>
+        <v>195.39</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>14.54</v>
+        <v>185.25</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>16.61</v>
+        <v>209.15</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>17.6</v>
+        <v>219.76</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>9.57</v>
+        <v>8.51</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>29%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>16</v>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>4.37</v>
+        <v>189</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>-3.27</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>5.15</v>
+        <v>5.43</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-0.33</v>
+        <v>-3.42</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -921,17 +916,17 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -945,39 +940,39 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>195.39</v>
+        <v>128.16</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>185.25</v>
+        <v>121.51</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>209.15</v>
+        <v>135.22</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>219.76</v>
+        <v>140.71</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>8.51</v>
+        <v>5.12</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>192.1</v>
+        <v>127.5</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>-1.68</v>
+        <v>-0.51</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.21</v>
+        <v>1.12</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.66</v>
+        <v>-1.69</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -988,7 +983,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -998,7 +993,7 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -1012,39 +1007,39 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>128.16</v>
+        <v>14.64</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>121.51</v>
+        <v>13.88</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>135.22</v>
+        <v>15.47</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>140.71</v>
+        <v>16.12</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>5.12</v>
+        <v>3.78</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>128.16</v>
-      </c>
-      <c r="N9" s="8" t="n">
-        <v>0</v>
+        <v>14.4</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>-1.64</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>0</v>
+        <v>-1.84</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1055,7 +1050,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1065,7 +1060,7 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1075,43 +1070,43 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>14.64</v>
+        <v>158.92</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>13.88</v>
+        <v>150.69</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>15.47</v>
+        <v>166.51</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>16.12</v>
+        <v>172.44</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>3.78</v>
+        <v>3.46</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>14.64</v>
-      </c>
-      <c r="N10" s="8" t="n">
-        <v>0</v>
+        <v>155</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>-2.47</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>0</v>
+        <v>-2.84</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1122,22 +1117,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1146,30 +1141,30 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>158.92</v>
+        <v>14.6</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>150.69</v>
+        <v>13.84</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>166.51</v>
+        <v>15.39</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>172.44</v>
+        <v>16.01</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>3.46</v>
+        <v>3.63</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>158.92</v>
+        <v>14.6</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1181,6 +1176,73 @@
         <v>0</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>T0034</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-15</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>2170</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>28.94</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>27.44</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>30.84</v>
+      </c>
+      <c r="I12" s="5" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>7%</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M12" s="5" t="n">
+        <v>28.94</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
         <is>
           <t>🟢 Active</t>
         </is>
@@ -1200,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P27"/>
+  <dimension ref="A1:P28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1299,27 +1361,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1328,44 +1390,44 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>12.24</v>
+        <v>45.31</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>12.9</v>
+        <v>43.14</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J4" s="9" t="n">
-        <v>0.0609</v>
+        <v>3</v>
+      </c>
+      <c r="J4" s="7" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0461</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>16.08</v>
+        <v>12.84</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>36.7</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -1380,12 +1442,12 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1394,20 +1456,20 @@
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>25.85</v>
+        <v>12.24</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>25.22</v>
+        <v>12.9</v>
       </c>
       <c r="I5" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J5" s="7" t="n">
-        <v>-0.0244</v>
+      <c r="J5" s="9" t="n">
+        <v>0.0609</v>
       </c>
       <c r="K5" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
@@ -1416,22 +1478,22 @@
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0155</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>14.35</v>
+        <v>16.08</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>26.1</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1446,12 +1508,12 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1460,20 +1522,20 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>90.63</v>
+        <v>25.85</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>25.22</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J6" s="9" t="n">
-        <v>0.0416</v>
+      <c r="J6" s="7" t="n">
+        <v>-0.0244</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
@@ -1482,22 +1544,22 @@
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>0</v>
+        <v>-0.0352</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>14.18</v>
+        <v>14.35</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>23</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1512,12 +1574,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1526,18 +1588,18 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>15.53</v>
+        <v>90.63</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>15.88</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J7" s="9" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
+        <v>0.0416</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -1548,22 +1610,22 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.038</v>
+        <v>0.057</v>
       </c>
       <c r="N7" s="8" t="n">
         <v>0</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>19.9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1578,12 +1640,12 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1592,20 +1654,20 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>694.39</v>
+        <v>15.53</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>680</v>
+        <v>15.88</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J8" s="7" t="n">
-        <v>-0.0207</v>
+      <c r="J8" s="9" t="n">
+        <v>0.0267</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1614,42 +1676,42 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.038</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0517</v>
+        <v>0</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>10.02</v>
+        <v>11.78</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>23.7</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1658,18 +1720,18 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>15.01</v>
+        <v>694.39</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>14.34</v>
+        <v>680</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>-0.0446</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
+        <v>-0.0207</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1680,27 +1742,27 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.0254</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0466</v>
+        <v>-0.0517</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>11.78</v>
+        <v>10.02</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>11.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1710,32 +1772,32 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>28.9</v>
+        <v>15.01</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>28.16</v>
+        <v>14.34</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>-0.0256</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
+        <v>-0.0446</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1746,37 +1808,37 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0</v>
+        <v>0.0127</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0466</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.9</v>
+        <v>11.78</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>32.8</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1786,22 +1848,22 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>70.64</v>
+        <v>28.9</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>69</v>
+        <v>28.16</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
+        <v>-0.0256</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1812,22 +1874,22 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0178</v>
+        <v>0</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0436</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>24.18</v>
+        <v>12.9</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>13.3</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1842,12 +1904,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1856,49 +1918,49 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>182.46</v>
+        <v>70.64</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>198.78</v>
+        <v>69</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="9" t="n">
-        <v>0.08939999999999999</v>
+      <c r="J12" s="7" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0178</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0331</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>23.45</v>
+        <v>24.18</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1908,63 +1970,63 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>14.05</v>
+        <v>182.46</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>13.25</v>
+        <v>198.78</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J13" s="7" t="n">
-        <v>-0.0567</v>
+        <v>5</v>
+      </c>
+      <c r="J13" s="9" t="n">
+        <v>0.08939999999999999</v>
       </c>
       <c r="K13" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.106</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0036</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>14.88</v>
+        <v>23.45</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>35.5</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -1974,12 +2036,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -1988,110 +2050,110 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>14.64</v>
+        <v>14.05</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>14.51</v>
+        <v>13.25</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>-0.0567</v>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0036</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.079</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>14.88</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>20.2</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>32.56</v>
+        <v>14.64</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>30.73</v>
+        <v>14.51</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0089</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0294</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>15.98</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>43.3</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2106,12 +2168,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2120,18 +2182,18 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J16" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
+        <v>-0.0563</v>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2142,22 +2204,22 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>13.05</v>
+        <v>15.98</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2197,7 +2259,7 @@
       <c r="J17" s="7" t="n">
         <v>-0.0478</v>
       </c>
-      <c r="K17" s="11" t="inlineStr">
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2214,7 +2276,7 @@
         <v>-0.0925</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>12.93</v>
+        <v>13.05</v>
       </c>
       <c r="P17" s="6" t="n">
         <v>28.7</v>
@@ -2223,7 +2285,7 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2238,12 +2300,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2252,18 +2314,18 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
+        <v>-0.0478</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2274,42 +2336,42 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>12.53</v>
+        <v>12.93</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2318,44 +2380,44 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>43.19</v>
+        <v>32.56</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>43.88</v>
+        <v>30.73</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J19" s="9" t="n">
-        <v>0.016</v>
+        <v>1</v>
+      </c>
+      <c r="J19" s="7" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0608</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>32.16</v>
+        <v>12.53</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>13</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2370,12 +2432,12 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2384,18 +2446,18 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>137.37</v>
+        <v>43.19</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>143</v>
+        <v>43.88</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K20" s="10" t="inlineStr">
+        <v>0.016</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -2406,22 +2468,22 @@
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0188</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0016</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>30.86</v>
+        <v>32.16</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>22.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2436,7 +2498,7 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
@@ -2450,18 +2512,18 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>27.31</v>
+        <v>137.37</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>27.86</v>
+        <v>143</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.0201</v>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
+        <v>0.04099999999999999</v>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -2472,22 +2534,22 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0432</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.002</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>26.27</v>
+        <v>30.86</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>23.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2502,12 +2564,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2516,18 +2578,18 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>37.25</v>
+        <v>27.31</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>38.14</v>
+        <v>27.86</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
+        <v>0.0201</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -2538,22 +2600,22 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0392</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0114</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>23.8</v>
+        <v>26.27</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>27.9</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2568,12 +2630,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2582,20 +2644,20 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>105.01</v>
+        <v>37.25</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>105</v>
+        <v>38.14</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J23" s="7" t="n">
-        <v>-0.0001</v>
+      <c r="J23" s="9" t="n">
+        <v>0.0239</v>
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
@@ -2604,22 +2666,22 @@
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0379</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0212</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>10.01</v>
+        <v>23.8</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>17.6</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2629,37 +2691,37 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>26.25</v>
+        <v>105.01</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>25.64</v>
+        <v>105</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
+        <v>-0.0001</v>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2670,22 +2732,22 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0075</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.022</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>16.26</v>
+        <v>10.01</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>31.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2700,12 +2762,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2714,20 +2776,20 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>10.7</v>
+        <v>26.25</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>10.73</v>
+        <v>25.64</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J25" s="9" t="n">
-        <v>0.0028</v>
+      <c r="J25" s="7" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K25" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2736,22 +2798,22 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0011</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0316</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>12.8</v>
+        <v>16.26</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>14.8</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0006</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2761,63 +2823,63 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>8280</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>11.92</v>
+        <v>10.7</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>11.24</v>
+        <v>10.73</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J26" s="7" t="n">
-        <v>-0.0568</v>
+        <v>4</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>0.0028</v>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0</v>
+        <v>0.0168</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.009300000000000001</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>12</v>
+        <v>12.8</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>33.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0008</t>
+          <t>T0007</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2832,32 +2894,32 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>26.89</v>
+        <v>11.92</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>25.73</v>
+        <v>11.24</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>-0.0431</v>
-      </c>
-      <c r="K27" s="11" t="inlineStr">
+        <v>-0.0568</v>
+      </c>
+      <c r="K27" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2871,12 +2933,78 @@
         <v>0</v>
       </c>
       <c r="N27" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P27" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>T0008</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>-0.0431</v>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N28" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O27" s="6" t="n">
+      <c r="O28" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P27" s="6" t="n">
+      <c r="P28" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -2894,7 +3022,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E49"/>
+  <dimension ref="A1:E50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -2911,7 +3039,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-14T02:02:56</t>
+          <t>محسوب في: 2026-05-15T02:02:45</t>
         </is>
       </c>
     </row>
@@ -2935,7 +3063,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="6">
@@ -2945,7 +3073,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -2965,7 +3093,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9">
@@ -2976,7 +3104,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>36.0%</t>
         </is>
       </c>
     </row>
@@ -3000,7 +3128,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.57%</t>
+          <t>-3.65%</t>
         </is>
       </c>
     </row>
@@ -3011,7 +3139,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.6</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="13">
@@ -3022,7 +3150,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-21.31%</t>
+          <t>-26.09%</t>
         </is>
       </c>
     </row>
@@ -3156,19 +3284,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>47.1%</t>
+          <t>44.4%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-0.27%</t>
         </is>
       </c>
     </row>
@@ -3331,19 +3459,19 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C38" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>-3.41%</t>
+          <t>-3.68%</t>
         </is>
       </c>
     </row>
@@ -3495,10 +3623,11 @@
       </c>
     </row>
     <row r="48"/>
-    <row r="49">
-      <c r="A49" s="25" t="inlineStr">
-        <is>
-          <t>(لا توجد بعد - يحتاج 3+ صفقات لكل سهم)</t>
+    <row r="49"/>
+    <row r="50">
+      <c r="A50" s="21" t="inlineStr">
+        <is>
+          <t>2280: 0/3 = 0.0%</t>
         </is>
       </c>
     </row>
@@ -4288,15 +4417,15 @@
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F21" s="3" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="F21" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-18_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -82,12 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -146,10 +146,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -162,18 +162,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -544,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q12"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -648,7 +648,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -658,12 +658,12 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -672,60 +672,60 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>100.3</v>
+        <v>32.56</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>95.5</v>
+        <v>30.88</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>104.7</v>
+        <v>34.52</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>108.16</v>
+        <v>36.04</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>9.9</v>
+        <v>12.52</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>97%</t>
+          <t>76%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
         <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>98</v>
+        <v>32.9</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-2.29</v>
+        <v>1.04</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>0.6</v>
+        <v>6.63</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-4.19</v>
+        <v>-0.12</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -735,64 +735,64 @@
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>32.56</v>
+        <v>15.33</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>30.88</v>
+        <v>14.54</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>34.52</v>
+        <v>16.61</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>36.04</v>
+        <v>17.6</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>12.52</v>
+        <v>9.57</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>76%</t>
+          <t>44%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
         <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>33.22</v>
-      </c>
-      <c r="N5" s="9" t="n">
-        <v>2.03</v>
+        <v>15.84</v>
+      </c>
+      <c r="N5" s="7" t="n">
+        <v>3.33</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>6.63</v>
+        <v>6.33</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-0.12</v>
+        <v>-0.33</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
-          <t>🟡 Partial</t>
+          <t>🟢 Active</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -806,39 +806,39 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>15.33</v>
+        <v>128.16</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>14.54</v>
+        <v>121.51</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>16.61</v>
+        <v>135.22</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>17.6</v>
+        <v>140.71</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>9.57</v>
+        <v>5.12</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>15.99</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>4.31</v>
+        <v>128.9</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.58</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>6.33</v>
+        <v>1.12</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-0.33</v>
+        <v>-1.69</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,17 +849,17 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -873,39 +873,39 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>195.39</v>
+        <v>14.64</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>185.25</v>
+        <v>13.88</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>209.15</v>
+        <v>15.47</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>219.76</v>
+        <v>16.12</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>8.51</v>
+        <v>3.78</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>29%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>189</v>
-      </c>
-      <c r="N7" s="7" t="n">
-        <v>-3.27</v>
+        <v>14.25</v>
+      </c>
+      <c r="N7" s="9" t="n">
+        <v>-2.66</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>5.43</v>
+        <v>0.55</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-3.42</v>
+        <v>-3.21</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -926,7 +926,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -936,43 +936,43 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>128.16</v>
+        <v>158.92</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>121.51</v>
+        <v>150.69</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>135.22</v>
+        <v>166.51</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>140.71</v>
+        <v>172.44</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>5.12</v>
+        <v>3.46</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>24%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>127.5</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>-0.51</v>
+        <v>154.1</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>-3.03</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>1.12</v>
+        <v>0</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-1.69</v>
+        <v>-3.41</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,63 +983,63 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>14.64</v>
+        <v>14.6</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>13.88</v>
+        <v>13.84</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>15.47</v>
+        <v>15.39</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>16.12</v>
+        <v>16.01</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3.78</v>
+        <v>3.63</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>14.4</v>
+        <v>14.95</v>
       </c>
       <c r="N9" s="7" t="n">
-        <v>-1.64</v>
+        <v>2.4</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.55</v>
+        <v>4.45</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-1.84</v>
+        <v>0</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,17 +1050,17 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -1070,43 +1070,43 @@
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>158.92</v>
+        <v>28.94</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>150.69</v>
+        <v>27.44</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>166.51</v>
+        <v>30.84</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>172.44</v>
+        <v>32.3</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>3.46</v>
+        <v>3</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>155</v>
-      </c>
-      <c r="N10" s="7" t="n">
-        <v>-2.47</v>
+        <v>28.6</v>
+      </c>
+      <c r="N10" s="9" t="n">
+        <v>-1.17</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0</v>
+        <v>0.48</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-2.84</v>
+        <v>-2.28</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,17 +1117,17 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -1141,30 +1141,30 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>14.6</v>
+        <v>11.82</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>13.84</v>
+        <v>11.21</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>15.39</v>
+        <v>12.43</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>16.01</v>
+        <v>12.91</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>3.63</v>
+        <v>16.94</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>14.6</v>
+        <v>11.82</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1184,54 +1184,54 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>28.94</v>
+        <v>11.35</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>27.44</v>
+        <v>10.76</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>30.84</v>
+        <v>12.01</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>32.3</v>
+        <v>12.51</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>3</v>
+        <v>16.05</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="L12" s="3" t="n">
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>28.94</v>
+        <v>11.35</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1243,6 +1243,73 @@
         <v>0</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>🟢 Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>T0037</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-18</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>7202</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>تقنية</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>230.06</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>220.32</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>238.88</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>245.84</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>12.77</v>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>50%</t>
+        </is>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M13" s="5" t="n">
+        <v>230.06</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="3" t="inlineStr">
         <is>
           <t>🟢 Active</t>
         </is>
@@ -1262,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P28"/>
+  <dimension ref="A1:P30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1361,7 +1428,7 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
@@ -1371,17 +1438,17 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1390,130 +1457,130 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>45.31</v>
+        <v>100.3</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>43.14</v>
+        <v>97</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>-0.0478</v>
+        <v>5</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>-0.0329</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>12.84</v>
+        <v>9.9</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>28.7</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>12.24</v>
+        <v>195.39</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>12.9</v>
+        <v>184.32</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>-0.0566</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0634</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>16.08</v>
+        <v>8.51</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>36.7</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1522,44 +1589,44 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>25.85</v>
+        <v>45.31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>25.22</v>
+        <v>43.14</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>-0.0244</v>
+        <v>3</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0461</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>14.35</v>
+        <v>12.84</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>26.1</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1574,12 +1641,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1588,16 +1655,16 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>90.63</v>
+        <v>12.24</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>12.9</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J7" s="9" t="n">
-        <v>0.0416</v>
+      <c r="J7" s="7" t="n">
+        <v>0.0609</v>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
@@ -1610,22 +1677,22 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.057</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>14.18</v>
+        <v>16.08</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>23</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -1640,7 +1707,7 @@
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1654,20 +1721,20 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>15.53</v>
+        <v>25.85</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>15.88</v>
+        <v>25.22</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K8" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>-0.0244</v>
+      </c>
+      <c r="K8" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1676,22 +1743,22 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>0</v>
+        <v>-0.0352</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>11.78</v>
+        <v>14.35</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>19.9</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1706,12 +1773,12 @@
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1720,20 +1787,20 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>694.39</v>
+        <v>90.63</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>680</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0416</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
@@ -1742,42 +1809,42 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.057</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0517</v>
+        <v>0</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>10.02</v>
+        <v>14.18</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>23.7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1786,20 +1853,20 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>15.01</v>
+        <v>15.53</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>14.34</v>
+        <v>15.88</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>-0.0446</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0267</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -1808,60 +1875,60 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.038</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O10" s="6" t="n">
         <v>11.78</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>11.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>28.9</v>
+        <v>694.39</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>28.16</v>
+        <v>680</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J11" s="7" t="n">
-        <v>-0.0256</v>
+        <v>5</v>
+      </c>
+      <c r="J11" s="9" t="n">
+        <v>-0.0207</v>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
@@ -1874,42 +1941,42 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0</v>
+        <v>0.0254</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0517</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>12.9</v>
+        <v>10.02</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>32.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1918,16 +1985,16 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>70.64</v>
+        <v>15.01</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>69</v>
+        <v>14.34</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="7" t="n">
-        <v>-0.0232</v>
+      <c r="J12" s="9" t="n">
+        <v>-0.0446</v>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
@@ -1940,93 +2007,93 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0127</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0466</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>13.3</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>182.46</v>
+        <v>28.9</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>198.78</v>
+        <v>28.16</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+        <v>-0.0256</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0436</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>23.45</v>
+        <v>12.9</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>12.1</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
@@ -2036,63 +2103,63 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>14.05</v>
+        <v>70.64</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>13.25</v>
+        <v>69</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>-0.0567</v>
+        <v>5</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0178</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0331</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>14.88</v>
+        <v>24.18</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>35.5</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2102,96 +2169,96 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>14.51</v>
+        <v>198.78</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.106</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0036</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>20.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C16" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>32.56</v>
+        <v>14.05</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>30.73</v>
+        <v>13.25</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J16" s="7" t="n">
-        <v>-0.0563</v>
+        <v>2</v>
+      </c>
+      <c r="J16" s="9" t="n">
+        <v>-0.0567</v>
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
@@ -2204,88 +2271,88 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0036</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.079</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>15.98</v>
+        <v>14.88</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>43.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>-0.0478</v>
+        <v>7</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>-0.0089</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>13.05</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
@@ -2300,12 +2367,12 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2314,16 +2381,16 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J18" s="7" t="n">
-        <v>-0.0478</v>
+      <c r="J18" s="9" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
@@ -2336,22 +2403,22 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>12.93</v>
+        <v>15.98</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2366,12 +2433,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2380,16 +2447,16 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J19" s="7" t="n">
-        <v>-0.0563</v>
+      <c r="J19" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
@@ -2402,37 +2469,37 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>12.53</v>
+        <v>13.05</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
@@ -2446,64 +2513,64 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0478</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>32.16</v>
+        <v>12.93</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2512,44 +2579,44 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K21" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0563</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>30.86</v>
+        <v>12.53</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2564,12 +2631,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2578,16 +2645,16 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>27.31</v>
+        <v>43.19</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>27.86</v>
+        <v>43.88</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J22" s="9" t="n">
-        <v>0.0201</v>
+      <c r="J22" s="7" t="n">
+        <v>0.016</v>
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
@@ -2600,22 +2667,22 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0188</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0016</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>26.27</v>
+        <v>32.16</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>23.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2630,12 +2697,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2644,16 +2711,16 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>37.25</v>
+        <v>137.37</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>38.14</v>
+        <v>143</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J23" s="9" t="n">
-        <v>0.0239</v>
+      <c r="J23" s="7" t="n">
+        <v>0.04099999999999999</v>
       </c>
       <c r="K23" s="11" t="inlineStr">
         <is>
@@ -2666,22 +2733,22 @@
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0432</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.002</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>23.8</v>
+        <v>30.86</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>27.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2696,12 +2763,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2710,20 +2777,20 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>105.01</v>
+        <v>27.31</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>105</v>
+        <v>27.86</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K24" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0201</v>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2732,22 +2799,22 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0392</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0114</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>10.01</v>
+        <v>26.27</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>17.6</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2757,39 +2824,39 @@
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>26.25</v>
+        <v>37.25</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>25.64</v>
+        <v>38.14</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K25" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>0.0239</v>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2798,22 +2865,22 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0379</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0212</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>16.26</v>
+        <v>23.8</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2823,39 +2890,39 @@
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>10.7</v>
+        <v>105.01</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>10.73</v>
+        <v>105</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>-0.0001</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
@@ -2864,22 +2931,22 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0075</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.022</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>12.8</v>
+        <v>10.01</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2889,122 +2956,254 @@
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <v>-0.0568</v>
+        <v>4</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K27" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E28" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M28" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N28" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P28" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E29" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L29" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O29" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P29" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
+      <c r="B30" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C30" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D30" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E28" s="4" t="inlineStr">
+      <c r="E30" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
+      <c r="F30" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G28" s="5" t="n">
+      <c r="G30" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H28" s="5" t="n">
+      <c r="H30" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I28" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J28" s="7" t="n">
+      <c r="I30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K28" s="10" t="inlineStr">
+      <c r="K30" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L28" s="4" t="inlineStr">
+      <c r="L30" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M28" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N28" s="8" t="n">
+      <c r="M30" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N30" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O28" s="6" t="n">
+      <c r="O30" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P28" s="6" t="n">
+      <c r="P30" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3022,7 +3221,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E50"/>
+  <dimension ref="A1:E51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3039,7 +3238,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-15T02:02:45</t>
+          <t>محسوب في: 2026-05-18T02:02:30</t>
         </is>
       </c>
     </row>
@@ -3063,7 +3262,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6">
@@ -3073,7 +3272,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
@@ -3093,7 +3292,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9">
@@ -3104,7 +3303,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>36.0%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -3128,7 +3327,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.65%</t>
+          <t>-3.74%</t>
         </is>
       </c>
     </row>
@@ -3139,7 +3338,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.55</v>
+        <v>0.48</v>
       </c>
     </row>
     <row r="13">
@@ -3150,7 +3349,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-26.09%</t>
+          <t>-35.04%</t>
         </is>
       </c>
     </row>
@@ -3238,7 +3437,7 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>0</v>
@@ -3250,7 +3449,7 @@
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>-4.08%</t>
+          <t>-4.47%</t>
         </is>
       </c>
     </row>
@@ -3284,19 +3483,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>8</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>44.4%</t>
+          <t>42.1%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.27%</t>
+          <t>-0.43%</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3589,7 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>0</v>
@@ -3402,7 +3601,7 @@
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-4.09%</t>
+          <t>-4.35%</t>
         </is>
       </c>
     </row>
@@ -3613,19 +3812,42 @@
         </is>
       </c>
     </row>
-    <row r="45"/>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>اتصالات</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C45" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>-3.29%</t>
+        </is>
+      </c>
+    </row>
     <row r="46"/>
-    <row r="47">
-      <c r="A47" s="24" t="inlineStr">
+    <row r="47"/>
+    <row r="48">
+      <c r="A48" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="48"/>
     <row r="49"/>
-    <row r="50">
-      <c r="A50" s="21" t="inlineStr">
+    <row r="50"/>
+    <row r="51">
+      <c r="A51" s="21" t="inlineStr">
         <is>
           <t>2280: 0/3 = 0.0%</t>
         </is>
@@ -3646,7 +3868,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4610,6 +4832,88 @@
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>7040</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>اتصالات</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>-3.29%</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>-3.29%</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>-3.29%</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>1321</t>
+        </is>
+      </c>
+      <c r="B27" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
+        <is>
+          <t>-5.66%</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>-5.66%</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>-5.66%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-19_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -692,16 +692,16 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>15.84</v>
+        <v>16.15</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>3.33</v>
+        <v>5.35</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>6.33</v>
+        <v>6.98</v>
       </c>
       <c r="P4" s="8" t="n">
         <v>-0.33</v>
@@ -759,16 +759,16 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>128.9</v>
+        <v>128.6</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>0.58</v>
+        <v>0.34</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>1.12</v>
+        <v>2.06</v>
       </c>
       <c r="P5" s="8" t="n">
         <v>-1.69</v>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>14.25</v>
+        <v>14.16</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-2.66</v>
+        <v>-3.28</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0.55</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-3.21</v>
+        <v>-3.62</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,22 +849,22 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -873,39 +873,39 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>158.92</v>
+        <v>14.6</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>150.69</v>
+        <v>13.84</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>166.51</v>
+        <v>15.39</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>172.44</v>
+        <v>16.01</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3.46</v>
+        <v>3.63</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>24%</t>
+          <t>6%</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
         <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>154.1</v>
+        <v>14.55</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>-3.03</v>
+        <v>-0.34</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>0</v>
+        <v>4.45</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-3.41</v>
+        <v>-1.03</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,7 +916,7 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
@@ -926,53 +926,53 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>14.6</v>
+        <v>28.94</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>13.84</v>
+        <v>27.44</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>15.39</v>
+        <v>30.84</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>16.01</v>
+        <v>32.3</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>3.63</v>
+        <v>3</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>7%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>14.95</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>2.4</v>
+        <v>28.44</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>-1.73</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>4.45</v>
+        <v>0.48</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>0</v>
+        <v>-2.28</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,63 +983,63 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>28.94</v>
+        <v>11.35</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>27.44</v>
+        <v>10.76</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>30.84</v>
+        <v>12.01</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>32.3</v>
+        <v>12.51</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>3</v>
+        <v>16.05</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>28.6</v>
+        <v>11.18</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>-1.17</v>
+        <v>-1.5</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.48</v>
+        <v>3</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-2.28</v>
+        <v>-3.44</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1060,12 +1060,12 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
@@ -1074,39 +1074,39 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>11.35</v>
+        <v>230.06</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>10.76</v>
+        <v>220.32</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>12.01</v>
+        <v>238.88</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>12.51</v>
+        <v>245.84</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>16.05</v>
+        <v>12.77</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>11.33</v>
+        <v>225.7</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-0.18</v>
+        <v>-1.9</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-3.44</v>
+        <v>-2.2</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,7 +1117,7 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1127,53 +1127,53 @@
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>230.06</v>
+        <v>11.03</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>220.32</v>
+        <v>10.47</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>238.88</v>
+        <v>11.58</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>245.84</v>
+        <v>12.15</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>12.77</v>
+        <v>10.8</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L11" s="3" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>229.6</v>
-      </c>
-      <c r="N11" s="9" t="n">
-        <v>-0.2</v>
+        <v>11.03</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>-0</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0</v>
+        <v>0.27</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-2.03</v>
+        <v>-1.63</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1184,7 +1184,7 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1194,33 +1194,33 @@
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>11.03</v>
+        <v>32.97</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>10.47</v>
+        <v>31.39</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>11.58</v>
+        <v>34.55</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>12.15</v>
+        <v>36.13</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>10.8</v>
+        <v>7.94</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1228,19 +1228,19 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="N12" s="8" t="n">
-        <v>0</v>
+        <v>32.66</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>-0.9399999999999999</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>0</v>
+        <v>0.52</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>0</v>
+        <v>-1.67</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1251,22 +1251,22 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
@@ -1275,19 +1275,19 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>32.97</v>
+        <v>12.66</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>31.39</v>
+        <v>12.03</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>34.55</v>
+        <v>13.29</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>36.13</v>
+        <v>13.92</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>7.94</v>
+        <v>10.24</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>32.97</v>
+        <v>12.66</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P32"/>
+  <dimension ref="A1:P33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,27 +1428,27 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
@@ -1457,49 +1457,49 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>100.3</v>
+        <v>158.92</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>97</v>
+        <v>149.94</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0329</v>
+        <v>-0.0565</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0624</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>9.9</v>
+        <v>3.46</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>25.2</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
@@ -1509,63 +1509,63 @@
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>195.39</v>
+        <v>100.3</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>184.32</v>
+        <v>97</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>-0.0566</v>
+        <v>-0.0329</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.05429999999999999</v>
+        <v>0.006</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0634</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>8.51</v>
+        <v>9.9</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>43.7</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1575,7 +1575,7 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1585,68 +1585,68 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>32.56</v>
+        <v>195.39</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>32.9</v>
+        <v>184.32</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J6" s="7" t="n">
-        <v>0.0353</v>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>3</v>
+      </c>
+      <c r="J6" s="9" t="n">
+        <v>-0.0566</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.0663</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.0634</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>12.52</v>
+        <v>8.51</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>43.3</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C7" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1655,64 +1655,64 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>11.82</v>
+        <v>32.56</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>11.15</v>
+        <v>32.9</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.0663</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.0012</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>16.94</v>
+        <v>12.52</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>25.6</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -1721,16 +1721,16 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>45.31</v>
+        <v>11.82</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>43.14</v>
+        <v>11.15</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0563</v>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
@@ -1743,42 +1743,42 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0728</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>12.84</v>
+        <v>16.94</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>28.7</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1787,44 +1787,44 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>12.24</v>
+        <v>45.31</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>12.9</v>
+        <v>43.14</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J9" s="7" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>3</v>
+      </c>
+      <c r="J9" s="9" t="n">
+        <v>-0.0478</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0461</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.08</v>
+        <v>12.84</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>36.7</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1839,12 +1839,12 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1853,20 +1853,20 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>25.85</v>
+        <v>12.24</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>25.22</v>
+        <v>12.9</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J10" s="9" t="n">
-        <v>-0.0244</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J10" s="7" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
@@ -1875,22 +1875,22 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0155</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>14.35</v>
+        <v>16.08</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>26.1</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
@@ -1905,12 +1905,12 @@
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1919,20 +1919,20 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>90.63</v>
+        <v>25.85</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>25.22</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>0.0416</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+      <c r="J11" s="9" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1941,22 +1941,22 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>0</v>
+        <v>-0.0352</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>14.18</v>
+        <v>14.35</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>23</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1985,16 +1985,16 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>15.53</v>
+        <v>90.63</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>15.88</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>0.0267</v>
+        <v>0.0416</v>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
@@ -2007,22 +2007,22 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.038</v>
+        <v>0.057</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>19.9</v>
+        <v>23</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2037,12 +2037,12 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2051,20 +2051,20 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>694.39</v>
+        <v>15.53</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>680</v>
+        <v>15.88</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J13" s="9" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J13" s="7" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -2073,42 +2073,42 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.038</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0517</v>
+        <v>0</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>10.02</v>
+        <v>11.78</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>23.7</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2117,16 +2117,16 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>15.01</v>
+        <v>694.39</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>14.34</v>
+        <v>680</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J14" s="9" t="n">
-        <v>-0.0446</v>
+        <v>-0.0207</v>
       </c>
       <c r="K14" s="10" t="inlineStr">
         <is>
@@ -2139,27 +2139,27 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.0254</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0466</v>
+        <v>-0.0517</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>11.78</v>
+        <v>10.02</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>11.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -2169,30 +2169,30 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>28.9</v>
+        <v>15.01</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>28.16</v>
+        <v>14.34</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>-0.0256</v>
+        <v>-0.0446</v>
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
@@ -2205,37 +2205,37 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0</v>
+        <v>0.0127</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0466</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>12.9</v>
+        <v>11.78</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>32.8</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -2245,20 +2245,20 @@
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>70.64</v>
+        <v>28.9</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>69</v>
+        <v>28.16</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>-0.0232</v>
+        <v>-0.0256</v>
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
@@ -2271,22 +2271,22 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0178</v>
+        <v>0</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0436</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>24.18</v>
+        <v>12.9</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>13.3</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
@@ -2301,12 +2301,12 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2315,49 +2315,49 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>182.46</v>
+        <v>70.64</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>198.78</v>
+        <v>69</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J17" s="7" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+      <c r="J17" s="9" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0178</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0331</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>23.45</v>
+        <v>24.18</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>12.1</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
@@ -2367,63 +2367,63 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>14.05</v>
+        <v>182.46</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>13.25</v>
+        <v>198.78</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J18" s="9" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.106</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0036</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>14.88</v>
+        <v>23.45</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>35.5</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2447,110 +2447,110 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>14.64</v>
+        <v>14.05</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>14.51</v>
+        <v>13.25</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-0.0089</v>
+        <v>-0.0567</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0036</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.079</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>14.88</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>20.2</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>32.56</v>
+        <v>14.64</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>30.73</v>
+        <v>14.51</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0089</v>
       </c>
       <c r="K20" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0294</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>15.98</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>43.3</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
@@ -2565,12 +2565,12 @@
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2579,16 +2579,16 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0563</v>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
@@ -2601,22 +2601,22 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>13.05</v>
+        <v>15.98</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2673,7 +2673,7 @@
         <v>-0.0925</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>12.93</v>
+        <v>13.05</v>
       </c>
       <c r="P22" s="6" t="n">
         <v>28.7</v>
@@ -2682,7 +2682,7 @@
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,16 +2711,16 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0478</v>
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
@@ -2733,42 +2733,42 @@
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>12.53</v>
+        <v>12.93</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2777,44 +2777,44 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>43.19</v>
+        <v>32.56</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>43.88</v>
+        <v>30.73</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J24" s="7" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0608</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>32.16</v>
+        <v>12.53</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>13</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2843,16 +2843,16 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>137.37</v>
+        <v>43.19</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>143</v>
+        <v>43.88</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.04099999999999999</v>
+        <v>0.016</v>
       </c>
       <c r="K25" s="11" t="inlineStr">
         <is>
@@ -2865,22 +2865,22 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0188</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0016</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>30.86</v>
+        <v>32.16</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>22.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2895,7 +2895,7 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2909,16 +2909,16 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>27.31</v>
+        <v>137.37</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>27.86</v>
+        <v>143</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>0.0201</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K26" s="11" t="inlineStr">
         <is>
@@ -2931,22 +2931,22 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0432</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.002</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>26.27</v>
+        <v>30.86</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>23.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2961,12 +2961,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2975,16 +2975,16 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>37.25</v>
+        <v>27.31</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>38.14</v>
+        <v>27.86</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0239</v>
+        <v>0.0201</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
@@ -2997,22 +2997,22 @@
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0392</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0114</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>23.8</v>
+        <v>26.27</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>27.9</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -3041,20 +3041,20 @@
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>105.01</v>
+        <v>37.25</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>105</v>
+        <v>38.14</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J28" s="9" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K28" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J28" s="7" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -3063,22 +3063,22 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0379</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0212</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>10.01</v>
+        <v>23.8</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>17.6</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3088,35 +3088,35 @@
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>26.25</v>
+        <v>105.01</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>25.64</v>
+        <v>105</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>-0.0232</v>
+        <v>-0.0001</v>
       </c>
       <c r="K29" s="10" t="inlineStr">
         <is>
@@ -3129,22 +3129,22 @@
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0075</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.022</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>16.26</v>
+        <v>10.01</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>31.4</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -3173,20 +3173,20 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>10.7</v>
+        <v>26.25</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>10.73</v>
+        <v>25.64</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J30" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K30" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+      <c r="J30" s="9" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
@@ -3195,22 +3195,22 @@
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0011</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0316</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>12.8</v>
+        <v>16.26</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>14.8</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0006</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3220,63 +3220,63 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>8280</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>11.92</v>
+        <v>10.7</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>11.24</v>
+        <v>10.73</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="9" t="n">
-        <v>-0.0568</v>
-      </c>
-      <c r="K31" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>4</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0</v>
+        <v>0.0168</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.009300000000000001</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>12</v>
+        <v>12.8</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>33.5</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0008</t>
+          <t>T0007</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3291,30 +3291,30 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>26.89</v>
+        <v>11.92</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>25.73</v>
+        <v>11.24</v>
       </c>
       <c r="I32" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-0.0431</v>
+        <v>-0.0568</v>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
@@ -3330,12 +3330,78 @@
         <v>0</v>
       </c>
       <c r="N32" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O32" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P32" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>T0008</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>2050</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>26.89</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>25.73</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>-0.0431</v>
+      </c>
+      <c r="K33" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N33" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O32" s="6" t="n">
+      <c r="O33" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P32" s="6" t="n">
+      <c r="P33" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3370,7 +3436,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-18T05:54:24</t>
+          <t>محسوب في: 2026-05-19T02:02:57</t>
         </is>
       </c>
     </row>
@@ -3394,7 +3460,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
@@ -3424,7 +3490,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="9">
@@ -3435,7 +3501,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>34.5%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -3459,7 +3525,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-3.93%</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3536,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.49</v>
+        <v>0.46</v>
       </c>
     </row>
     <row r="13">
@@ -3481,7 +3547,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-37.14%</t>
+          <t>-42.79%</t>
         </is>
       </c>
     </row>
@@ -3615,19 +3681,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>42.9%</t>
+          <t>40.9%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.49%</t>
+          <t>-0.73%</t>
         </is>
       </c>
     </row>
@@ -3721,19 +3787,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>14.3%</t>
+          <t>12.5%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-3.23%</t>
+          <t>-3.53%</t>
         </is>
       </c>
     </row>
@@ -4007,7 +4073,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I28"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -5094,6 +5160,47 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" s="3" t="inlineStr">
+        <is>
+          <t>2110</t>
+        </is>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-20_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -692,13 +692,13 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>16.15</v>
+        <v>16.17</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>5.35</v>
+        <v>5.48</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>6.98</v>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>128.6</v>
+        <v>129.6</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>0.34</v>
+        <v>1.12</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>2.06</v>
@@ -826,19 +826,19 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>14.16</v>
+        <v>14.19</v>
       </c>
       <c r="N6" s="9" t="n">
-        <v>-3.28</v>
+        <v>-3.07</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>0.55</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-3.62</v>
+        <v>-4.3</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>14.55</v>
+        <v>14.22</v>
       </c>
       <c r="N7" s="9" t="n">
-        <v>-0.34</v>
+        <v>-2.6</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>4.45</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-1.03</v>
+        <v>-2.6</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,63 +916,63 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>28.94</v>
+        <v>11.35</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>27.44</v>
+        <v>10.76</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>30.84</v>
+        <v>12.01</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>32.3</v>
+        <v>12.51</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>3</v>
+        <v>16.05</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>7%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
         <v>3</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>28.44</v>
+        <v>11.2</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-1.73</v>
+        <v>-1.32</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.48</v>
+        <v>3</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.28</v>
+        <v>-3.44</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,7 +983,7 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -993,12 +993,12 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1007,39 +1007,39 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>11.35</v>
+        <v>230.06</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>10.76</v>
+        <v>220.32</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>12.01</v>
+        <v>238.88</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>12.51</v>
+        <v>245.84</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>16.05</v>
+        <v>12.77</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>50%</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>11.18</v>
+        <v>227.7</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>-1.5</v>
+        <v>-1.03</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>3</v>
+        <v>0.5</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-3.44</v>
+        <v>-2.2</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1060,53 +1060,53 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>230.06</v>
+        <v>32.97</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>220.32</v>
+        <v>31.39</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>238.88</v>
+        <v>34.55</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>245.84</v>
+        <v>36.13</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>12.77</v>
+        <v>7.94</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L10" s="3" t="n">
         <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>225.7</v>
+        <v>32.54</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-1.9</v>
+        <v>-1.3</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0.5</v>
+        <v>0.52</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-2.2</v>
+        <v>-2.88</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,43 +1117,43 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>11.03</v>
+        <v>12.66</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>10.47</v>
+        <v>12.03</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>11.58</v>
+        <v>13.29</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>12.15</v>
+        <v>13.92</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10.8</v>
+        <v>10.24</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1164,16 +1164,16 @@
         <v>1</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>11.03</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>-0</v>
+        <v>12.59</v>
+      </c>
+      <c r="N11" s="9" t="n">
+        <v>-0.55</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>0.27</v>
+        <v>1.11</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-1.63</v>
+        <v>-2.53</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1184,43 +1184,43 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>32.97</v>
+        <v>45.37</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>31.39</v>
+        <v>43.9</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>34.55</v>
+        <v>46.84</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>36.13</v>
+        <v>48.31</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>7.94</v>
+        <v>15.11</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1228,19 +1228,19 @@
         </is>
       </c>
       <c r="L12" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>32.66</v>
-      </c>
-      <c r="N12" s="9" t="n">
-        <v>-0.9399999999999999</v>
+        <v>45.37</v>
+      </c>
+      <c r="N12" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O12" s="8" t="n">
-        <v>0.52</v>
+        <v>0</v>
       </c>
       <c r="P12" s="8" t="n">
-        <v>-1.67</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="3" t="inlineStr">
         <is>
@@ -1251,43 +1251,43 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0040</t>
+          <t>T0042</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>4190</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>12.66</v>
+        <v>15.71</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>12.03</v>
+        <v>15.31</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>13.29</v>
+        <v>16.12</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>13.92</v>
+        <v>16.52</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>10.24</v>
+        <v>9.49</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>12.66</v>
+        <v>15.71</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P33"/>
+  <dimension ref="A1:P35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,22 +1428,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1453,129 +1453,129 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>158.92</v>
+        <v>28.94</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>149.94</v>
+        <v>28.7</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>4</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0565</v>
+        <v>-0.0083</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0</v>
+        <v>0.0048</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0624</v>
+        <v>-0.0256</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>3.46</v>
+        <v>3</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>14.4</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>100.3</v>
+        <v>11.03</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>97</v>
+        <v>10.42</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J5" s="9" t="n">
-        <v>-0.0329</v>
+        <v>-0.0555</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0063</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>9.9</v>
+        <v>10.8</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>25.2</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
@@ -1585,20 +1585,20 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>195.39</v>
+        <v>158.92</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>184.32</v>
+        <v>149.94</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J6" s="9" t="n">
-        <v>-0.0566</v>
+        <v>-0.0565</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
@@ -1611,22 +1611,22 @@
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.05429999999999999</v>
+        <v>0</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0634</v>
+        <v>-0.0624</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>8.51</v>
+        <v>3.46</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>43.7</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -1641,12 +1641,12 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
@@ -1655,20 +1655,20 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>32.56</v>
+        <v>100.3</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>32.9</v>
+        <v>97</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J7" s="7" t="n">
-        <v>0.0353</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+      <c r="J7" s="9" t="n">
+        <v>-0.0329</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
@@ -1677,60 +1677,60 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0663</v>
+        <v>0.006</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>12.52</v>
+        <v>9.9</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>43.3</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
+          <t>2026-05-13</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>11.82</v>
+        <v>195.39</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>11.15</v>
+        <v>184.32</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0566</v>
       </c>
       <c r="K8" s="10" t="inlineStr">
         <is>
@@ -1743,22 +1743,22 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.0634</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>16.94</v>
+        <v>8.51</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>25.6</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
@@ -1768,17 +1768,17 @@
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1787,64 +1787,64 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>43.14</v>
+        <v>32.9</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0</v>
+        <v>0.0663</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0012</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>12.84</v>
+        <v>12.52</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1853,64 +1853,64 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>12.24</v>
+        <v>11.82</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>12.9</v>
+        <v>11.15</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J10" s="7" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+        <v>1</v>
+      </c>
+      <c r="J10" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0728</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>16.08</v>
+        <v>16.94</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>36.7</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
@@ -1919,44 +1919,44 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>25.85</v>
+        <v>45.31</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>25.22</v>
+        <v>43.14</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J11" s="9" t="n">
-        <v>-0.0244</v>
+        <v>-0.0478</v>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M11" s="8" t="n">
         <v>0</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0461</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>14.35</v>
+        <v>12.84</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>26.1</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
@@ -1971,12 +1971,12 @@
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1985,16 +1985,16 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>90.63</v>
+        <v>12.24</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>12.9</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>0.0416</v>
+        <v>0.0609</v>
       </c>
       <c r="K12" s="11" t="inlineStr">
         <is>
@@ -2007,22 +2007,22 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.057</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>14.18</v>
+        <v>16.08</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>23</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2037,7 +2037,7 @@
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
@@ -2051,20 +2051,20 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>15.53</v>
+        <v>25.85</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>15.88</v>
+        <v>25.22</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J13" s="7" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>WIN_PARTIAL</t>
+      <c r="J13" s="9" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
@@ -2073,22 +2073,22 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>0</v>
+        <v>-0.0352</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>11.78</v>
+        <v>14.35</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>19.9</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2103,12 +2103,12 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2117,20 +2117,20 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>694.39</v>
+        <v>90.63</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>680</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I14" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J14" s="9" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K14" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J14" s="7" t="n">
+        <v>0.0416</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -2139,42 +2139,42 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.057</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0517</v>
+        <v>0</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>10.02</v>
+        <v>14.18</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>23.7</v>
+        <v>23</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2183,20 +2183,20 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>15.01</v>
+        <v>15.53</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>14.34</v>
+        <v>15.88</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J15" s="9" t="n">
-        <v>-0.0446</v>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J15" s="7" t="n">
+        <v>0.0267</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
+        <is>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
@@ -2205,60 +2205,60 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.038</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O15" s="6" t="n">
         <v>11.78</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>11.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>28.9</v>
+        <v>694.39</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>28.16</v>
+        <v>680</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>-0.0256</v>
+        <v>-0.0207</v>
       </c>
       <c r="K16" s="10" t="inlineStr">
         <is>
@@ -2271,42 +2271,42 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0</v>
+        <v>0.0254</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0436</v>
+        <v>-0.0517</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>12.9</v>
+        <v>10.02</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>32.8</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2315,16 +2315,16 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>70.64</v>
+        <v>15.01</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>69</v>
+        <v>14.34</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>-0.0232</v>
+        <v>-0.0446</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
@@ -2337,93 +2337,93 @@
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0127</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0466</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>13.3</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>182.46</v>
+        <v>28.9</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>198.78</v>
+        <v>28.16</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J18" s="7" t="n">
-        <v>0.08939999999999999</v>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
-        <is>
-          <t>WIN_T2</t>
+        <v>3</v>
+      </c>
+      <c r="J18" s="9" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.106</v>
+        <v>0</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0436</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>23.45</v>
+        <v>12.9</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>12.1</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
@@ -2433,63 +2433,63 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>14.05</v>
+        <v>70.64</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>13.25</v>
+        <v>69</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J19" s="9" t="n">
-        <v>-0.0567</v>
+        <v>-0.0232</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0178</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0331</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>14.88</v>
+        <v>24.18</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>35.5</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
@@ -2499,96 +2499,96 @@
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>14.64</v>
+        <v>182.46</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>14.51</v>
+        <v>198.78</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J20" s="9" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K20" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J20" s="7" t="n">
+        <v>0.08939999999999999</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.106</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0036</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>23.45</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>20.2</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C21" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>32.56</v>
+        <v>14.05</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>30.73</v>
+        <v>13.25</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0567</v>
       </c>
       <c r="K21" s="10" t="inlineStr">
         <is>
@@ -2601,88 +2601,88 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0036</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.079</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>15.98</v>
+        <v>14.88</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>43.3</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C22" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J22" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0089</v>
       </c>
       <c r="K22" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>13.05</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,16 +2711,16 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>45.31</v>
+        <v>32.56</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>43.14</v>
+        <v>30.73</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>-0.0478</v>
+        <v>-0.0563</v>
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
@@ -2733,22 +2733,22 @@
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0608</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>12.93</v>
+        <v>15.98</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>28.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2763,12 +2763,12 @@
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2777,16 +2777,16 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>32.56</v>
+        <v>45.31</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>30.73</v>
+        <v>43.14</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>1</v>
       </c>
       <c r="J24" s="9" t="n">
-        <v>-0.0563</v>
+        <v>-0.0478</v>
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
@@ -2799,37 +2799,37 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0925</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>12.53</v>
+        <v>13.05</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>43.3</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
@@ -2843,64 +2843,64 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J25" s="7" t="n">
-        <v>0.016</v>
-      </c>
-      <c r="K25" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J25" s="9" t="n">
+        <v>-0.0478</v>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>32.16</v>
+        <v>12.93</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2909,44 +2909,44 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>137.37</v>
+        <v>32.56</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>143</v>
+        <v>30.73</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J26" s="7" t="n">
-        <v>0.04099999999999999</v>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>1</v>
+      </c>
+      <c r="J26" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0432</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0608</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>30.86</v>
+        <v>12.53</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>22.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
@@ -2961,12 +2961,12 @@
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2975,16 +2975,16 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>27.31</v>
+        <v>43.19</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>27.86</v>
+        <v>43.88</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.0201</v>
+        <v>0.016</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
@@ -2997,22 +2997,22 @@
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0188</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0016</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>26.27</v>
+        <v>32.16</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>23.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
@@ -3027,12 +3027,12 @@
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -3041,16 +3041,16 @@
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>37.25</v>
+        <v>137.37</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>38.14</v>
+        <v>143</v>
       </c>
       <c r="I28" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>0.0239</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
@@ -3063,22 +3063,22 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0432</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.002</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>23.8</v>
+        <v>30.86</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>27.9</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
@@ -3093,12 +3093,12 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -3107,20 +3107,20 @@
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>105.01</v>
+        <v>27.31</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>105</v>
+        <v>27.86</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J29" s="9" t="n">
-        <v>-0.0001</v>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+      <c r="J29" s="7" t="n">
+        <v>0.0201</v>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
@@ -3129,22 +3129,22 @@
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0392</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0114</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>10.01</v>
+        <v>26.27</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>17.6</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3154,39 +3154,39 @@
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>26.25</v>
+        <v>37.25</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>25.64</v>
+        <v>38.14</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J30" s="9" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K30" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K30" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
@@ -3195,22 +3195,22 @@
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0379</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0212</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>16.26</v>
+        <v>23.8</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>31.4</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3220,39 +3220,39 @@
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>10.7</v>
+        <v>105.01</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>10.73</v>
+        <v>105</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J31" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K31" s="11" t="inlineStr">
-        <is>
-          <t>TIME_WIN</t>
+        <v>5</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -3261,22 +3261,22 @@
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0075</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.022</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>12.8</v>
+        <v>10.01</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>14.8</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0005</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3286,122 +3286,254 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>11.92</v>
+        <v>26.25</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>11.24</v>
+        <v>25.64</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-0.0568</v>
+        <v>-0.0232</v>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0</v>
+        <v>0.0011</v>
       </c>
       <c r="N32" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0316</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>12</v>
+        <v>16.26</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>33.5</v>
+        <v>31.4</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E33" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K33" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L33" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O33" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P33" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J34" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M34" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N34" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P34" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B33" s="3" t="inlineStr">
+      <c r="B35" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
+      <c r="C35" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D33" s="3" t="inlineStr">
+      <c r="D35" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E33" s="4" t="inlineStr">
+      <c r="E35" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F33" s="3" t="inlineStr">
+      <c r="F35" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G33" s="5" t="n">
+      <c r="G35" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H33" s="5" t="n">
+      <c r="H35" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="9" t="n">
+      <c r="I35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J35" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K33" s="10" t="inlineStr">
+      <c r="K35" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L33" s="4" t="inlineStr">
+      <c r="L35" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M33" s="8" t="n">
+      <c r="M35" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N33" s="8" t="n">
+      <c r="N35" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O33" s="6" t="n">
+      <c r="O35" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P33" s="6" t="n">
+      <c r="P35" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3419,7 +3551,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E52"/>
+  <dimension ref="A1:E53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -3436,7 +3568,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-19T02:02:57</t>
+          <t>محسوب في: 2026-05-20T02:02:30</t>
         </is>
       </c>
     </row>
@@ -3460,7 +3592,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>30</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6">
@@ -3490,7 +3622,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9">
@@ -3501,7 +3633,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>31.2%</t>
         </is>
       </c>
     </row>
@@ -3525,7 +3657,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.93%</t>
+          <t>-3.86%</t>
         </is>
       </c>
     </row>
@@ -3536,7 +3668,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.46</v>
+        <v>0.42</v>
       </c>
     </row>
     <row r="13">
@@ -3547,7 +3679,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-42.79%</t>
+          <t>-49.17%</t>
         </is>
       </c>
     </row>
@@ -3658,19 +3790,19 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>-2.12%</t>
+          <t>-1.79%</t>
         </is>
       </c>
     </row>
@@ -3704,7 +3836,7 @@
         </is>
       </c>
       <c r="B28" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C28" s="3" t="n">
         <v>0</v>
@@ -3716,7 +3848,7 @@
       </c>
       <c r="E28" s="17" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-4.05%</t>
         </is>
       </c>
     </row>
@@ -3787,19 +3919,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>12.5%</t>
+          <t>11.1%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-3.23%</t>
         </is>
       </c>
     </row>
@@ -4033,26 +4165,49 @@
         </is>
       </c>
     </row>
-    <row r="46"/>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>عقار</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C46" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" s="17" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>-5.55%</t>
+        </is>
+      </c>
+    </row>
     <row r="47"/>
-    <row r="48">
-      <c r="A48" s="24" t="inlineStr">
+    <row r="48"/>
+    <row r="49">
+      <c r="A49" s="24" t="inlineStr">
         <is>
           <t>⚠️ الأسهم المُتعِبة (Win Rate &lt; 30% مع 3+ صفقات)</t>
         </is>
       </c>
     </row>
-    <row r="49"/>
     <row r="50"/>
-    <row r="51">
-      <c r="A51" s="21" t="inlineStr">
-        <is>
-          <t>2370: 1/3 = 33.3%</t>
-        </is>
-      </c>
-    </row>
+    <row r="51"/>
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
+        <is>
+          <t>2370: 1/3 = 33.3%</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="21" t="inlineStr">
         <is>
           <t>2280: 0/3 = 0.0%</t>
         </is>
@@ -4073,7 +4228,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I29"/>
+  <dimension ref="A1:I30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4926,13 +5081,13 @@
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F23" s="3" t="inlineStr">
         <is>
@@ -4941,12 +5096,12 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-1.70%</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
@@ -5198,6 +5353,47 @@
       <c r="I29" s="3" t="inlineStr">
         <is>
           <t>-5.65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>4280</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>عقار</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>-5.55%</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>-5.55%</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>-5.55%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-21_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -82,12 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
@@ -162,18 +162,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -648,17 +648,17 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -672,39 +672,39 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>15.33</v>
+        <v>128.16</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>14.54</v>
+        <v>121.51</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>16.61</v>
+        <v>135.22</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>17.6</v>
+        <v>140.71</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>9.57</v>
+        <v>5.12</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>44%</t>
+          <t>38%</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
         <v>6</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>16.17</v>
+        <v>128</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>5.48</v>
+        <v>-0.12</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>6.98</v>
+        <v>2.06</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-0.33</v>
+        <v>-1.69</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -715,7 +715,7 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
@@ -725,7 +725,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -739,39 +739,39 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>128.16</v>
+        <v>14.64</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>121.51</v>
+        <v>13.88</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>135.22</v>
+        <v>15.47</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>140.71</v>
+        <v>16.12</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>5.12</v>
+        <v>3.78</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>41%</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>129.6</v>
+        <v>14.2</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>1.12</v>
+        <v>-3.01</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>2.06</v>
+        <v>0.55</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-1.69</v>
+        <v>-4.3</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -782,63 +782,63 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>14.64</v>
+        <v>11.35</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>13.88</v>
+        <v>10.76</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>15.47</v>
+        <v>12.01</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>16.12</v>
+        <v>12.51</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>3.78</v>
+        <v>16.05</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>68%</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>14.19</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>-3.07</v>
+        <v>10.9</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>-3.96</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>0.55</v>
+        <v>3</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-4.3</v>
+        <v>-4.85</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,63 +849,63 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>14.6</v>
+        <v>32.97</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>13.84</v>
+        <v>31.39</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>15.39</v>
+        <v>34.55</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>16.01</v>
+        <v>36.13</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>3.63</v>
+        <v>7.94</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
-          <t>6%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>14.22</v>
-      </c>
-      <c r="N7" s="9" t="n">
-        <v>-2.6</v>
+        <v>32.76</v>
+      </c>
+      <c r="N7" s="7" t="n">
+        <v>-0.64</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>4.45</v>
+        <v>1</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-2.6</v>
+        <v>-2.88</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,63 +916,63 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>11.35</v>
+        <v>12.66</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>10.76</v>
+        <v>12.03</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>12.01</v>
+        <v>13.29</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>12.51</v>
+        <v>13.92</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>16.05</v>
+        <v>10.24</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>11.2</v>
-      </c>
-      <c r="N8" s="9" t="n">
-        <v>-1.32</v>
+        <v>12.62</v>
+      </c>
+      <c r="N8" s="7" t="n">
+        <v>-0.32</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>3</v>
+        <v>1.11</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-3.44</v>
+        <v>-2.76</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1007,39 +1007,39 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>230.06</v>
+        <v>45.37</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>220.32</v>
+        <v>43.9</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>238.88</v>
+        <v>46.84</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>245.84</v>
+        <v>48.31</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>12.77</v>
+        <v>15.11</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
-          <t>50%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>227.7</v>
-      </c>
-      <c r="N9" s="9" t="n">
-        <v>-1.03</v>
+        <v>44.4</v>
+      </c>
+      <c r="N9" s="7" t="n">
+        <v>-2.14</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-2.2</v>
+        <v>-3.02</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,43 +1050,43 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0042</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4190</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>32.97</v>
+        <v>15.71</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>31.39</v>
+        <v>15.31</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>34.55</v>
+        <v>16.12</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>36.13</v>
+        <v>16.52</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>7.94</v>
+        <v>9.49</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1094,19 +1094,19 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>32.54</v>
+        <v>15.73</v>
       </c>
       <c r="N10" s="9" t="n">
-        <v>-1.3</v>
+        <v>0.13</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0.52</v>
+        <v>0.25</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-2.88</v>
+        <v>-1.46</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,43 +1117,43 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0040</t>
+          <t>T0043</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2270</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>12.66</v>
+        <v>224.35</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>12.03</v>
+        <v>213.89</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>13.29</v>
+        <v>234.81</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>13.92</v>
+        <v>245.27</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>10.24</v>
+        <v>14.29</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1161,19 +1161,19 @@
         </is>
       </c>
       <c r="L11" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>12.59</v>
-      </c>
-      <c r="N11" s="9" t="n">
-        <v>-0.55</v>
+        <v>224.35</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O11" s="8" t="n">
-        <v>1.11</v>
+        <v>0</v>
       </c>
       <c r="P11" s="8" t="n">
-        <v>-2.53</v>
+        <v>0</v>
       </c>
       <c r="Q11" s="3" t="inlineStr">
         <is>
@@ -1184,43 +1184,43 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0041</t>
+          <t>T0044</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>45.37</v>
+        <v>196.39</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>43.9</v>
+        <v>185.26</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>46.84</v>
+        <v>207.52</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>48.31</v>
+        <v>218.65</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>15.11</v>
+        <v>13.57</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>45.37</v>
+        <v>196.39</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1251,43 +1251,43 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0042</t>
+          <t>T0045</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>4190</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>15.71</v>
+        <v>87.52</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>15.31</v>
+        <v>83.53</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>16.12</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>16.52</v>
+        <v>95.5</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>9.49</v>
+        <v>10.05</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>15.71</v>
+        <v>87.52</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P35"/>
+  <dimension ref="A1:P38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,22 +1428,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1453,24 +1453,24 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>28.94</v>
+        <v>15.33</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>28.7</v>
+        <v>16.18</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J4" s="9" t="n">
-        <v>-0.0083</v>
+        <v>0.0554</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -1479,108 +1479,108 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0048</v>
+        <v>0.0698</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0256</v>
+        <v>-0.0033</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>3</v>
+        <v>9.57</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>28.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>11.03</v>
+        <v>14.6</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>10.42</v>
+        <v>14.22</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J5" s="9" t="n">
-        <v>-0.0555</v>
-      </c>
-      <c r="K5" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J5" s="7" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="K5" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.0063</v>
+        <v>0.0445</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.07980000000000001</v>
+        <v>-0.0322</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>10.8</v>
+        <v>3.63</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>32.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1589,18 +1589,18 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>158.92</v>
+        <v>230.06</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>149.94</v>
+        <v>219.22</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J6" s="9" t="n">
-        <v>-0.0565</v>
-      </c>
-      <c r="K6" s="10" t="inlineStr">
+      <c r="J6" s="7" t="n">
+        <v>-0.0471</v>
+      </c>
+      <c r="K6" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -1611,62 +1611,62 @@
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0624</v>
+        <v>-0.0559</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>3.46</v>
+        <v>12.77</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>14.4</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>100.3</v>
+        <v>28.94</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>97</v>
+        <v>28.7</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>-0.0329</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>-0.0083</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1677,62 +1677,62 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0048</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0256</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>9.9</v>
+        <v>3</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>25.2</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>195.39</v>
+        <v>11.03</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>184.32</v>
+        <v>10.42</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>-0.0566</v>
-      </c>
-      <c r="K8" s="10" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>-0.0555</v>
+      </c>
+      <c r="K8" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -1743,37 +1743,37 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.05429999999999999</v>
+        <v>0.0063</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0634</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>8.51</v>
+        <v>10.8</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>43.7</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1787,64 +1787,64 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>32.56</v>
+        <v>158.92</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>32.9</v>
+        <v>149.94</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>0.0353</v>
+        <v>-0.0565</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0663</v>
+        <v>0</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.0624</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>12.52</v>
+        <v>3.46</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>43.3</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C10" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1853,84 +1853,84 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>11.82</v>
+        <v>100.3</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>11.15</v>
+        <v>97</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J10" s="9" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J10" s="7" t="n">
+        <v>-0.0329</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>16.94</v>
+        <v>9.9</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>25.6</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>45.31</v>
+        <v>195.39</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>43.14</v>
+        <v>184.32</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K11" s="10" t="inlineStr">
+      <c r="J11" s="7" t="n">
+        <v>-0.0566</v>
+      </c>
+      <c r="K11" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -1941,42 +1941,42 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0634</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>12.84</v>
+        <v>8.51</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>28.7</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
@@ -1985,18 +1985,18 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>12.24</v>
+        <v>32.56</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>12.9</v>
+        <v>32.9</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J12" s="7" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
+      <c r="J12" s="9" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2007,42 +2007,42 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.0663</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0012</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>16.08</v>
+        <v>12.52</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>36.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2051,64 +2051,64 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>25.85</v>
+        <v>11.82</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>25.22</v>
+        <v>11.15</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J13" s="9" t="n">
-        <v>-0.0244</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>1</v>
+      </c>
+      <c r="J13" s="7" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0728</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>14.35</v>
+        <v>16.94</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>26.1</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2117,44 +2117,44 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>90.63</v>
+        <v>45.31</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>43.14</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>0.0416</v>
+        <v>-0.0478</v>
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>0</v>
+        <v>-0.0461</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>14.18</v>
+        <v>12.84</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>23</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
@@ -2169,12 +2169,12 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -2183,18 +2183,18 @@
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>15.53</v>
+        <v>12.24</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>15.88</v>
+        <v>12.9</v>
       </c>
       <c r="I15" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J15" s="7" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
+      <c r="J15" s="9" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2205,22 +2205,22 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.038</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>19.9</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -2235,12 +2235,12 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2249,18 +2249,18 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>694.39</v>
+        <v>25.85</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>680</v>
+        <v>25.22</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J16" s="9" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K16" s="10" t="inlineStr">
+      <c r="J16" s="7" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K16" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2271,42 +2271,42 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0254</v>
+        <v>0</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0517</v>
+        <v>-0.0352</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>10.02</v>
+        <v>14.35</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>23.7</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2315,20 +2315,20 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>15.01</v>
+        <v>90.63</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>14.34</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I17" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>-0.0446</v>
+        <v>0.0416</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
@@ -2337,64 +2337,64 @@
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.057</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>11.8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>28.9</v>
+        <v>15.53</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>28.16</v>
+        <v>15.88</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>-0.0256</v>
+        <v>0.0267</v>
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
@@ -2403,42 +2403,42 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0</v>
+        <v>0.038</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0436</v>
+        <v>0</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>12.9</v>
+        <v>11.78</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>32.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2447,18 +2447,18 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>70.64</v>
+        <v>694.39</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>69</v>
+        <v>680</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J19" s="9" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K19" s="10" t="inlineStr">
+      <c r="J19" s="7" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="K19" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2469,42 +2469,42 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0254</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0517</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>24.18</v>
+        <v>10.02</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>13.3</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2513,115 +2513,115 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>182.46</v>
+        <v>15.01</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>198.78</v>
+        <v>14.34</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>0.08939999999999999</v>
+        <v>-0.0446</v>
       </c>
       <c r="K20" s="11" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0127</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0466</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>23.45</v>
+        <v>11.78</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>14.05</v>
+        <v>28.9</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>13.25</v>
+        <v>28.16</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J21" s="9" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K21" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>3</v>
+      </c>
+      <c r="J21" s="7" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="K21" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.0036</v>
+        <v>0</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0436</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>14.88</v>
+        <v>12.9</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>35.5</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
@@ -2631,32 +2631,32 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>14.64</v>
+        <v>70.64</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>14.51</v>
+        <v>69</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J22" s="9" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J22" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2667,42 +2667,42 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0178</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0331</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>24.18</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>20.2</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C23" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,59 +2711,59 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>32.56</v>
+        <v>182.46</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>30.73</v>
+        <v>198.78</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>-0.0563</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.106</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0036</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>15.98</v>
+        <v>23.45</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>43.3</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C24" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
@@ -2773,22 +2773,22 @@
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>45.31</v>
+        <v>14.05</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>43.14</v>
+        <v>13.25</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J24" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K24" s="10" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J24" s="7" t="n">
+        <v>-0.0567</v>
+      </c>
+      <c r="K24" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2799,88 +2799,88 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.079</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>13.05</v>
+        <v>14.88</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>28.7</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C25" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J25" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K25" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>7</v>
+      </c>
+      <c r="J25" s="7" t="n">
+        <v>-0.0089</v>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>12.93</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2917,10 +2917,10 @@
       <c r="I26" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J26" s="9" t="n">
+      <c r="J26" s="7" t="n">
         <v>-0.0563</v>
       </c>
-      <c r="K26" s="10" t="inlineStr">
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2937,7 +2937,7 @@
         <v>-0.0608</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>12.53</v>
+        <v>15.98</v>
       </c>
       <c r="P26" s="6" t="n">
         <v>43.3</v>
@@ -2946,22 +2946,22 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
@@ -2975,64 +2975,64 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J27" s="7" t="n">
-        <v>0.016</v>
+        <v>-0.0478</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>32.16</v>
+        <v>13.05</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -3041,64 +3041,64 @@
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>137.37</v>
+        <v>45.31</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>143</v>
+        <v>43.14</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>0.04099999999999999</v>
+        <v>-0.0478</v>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0.0432</v>
+        <v>0</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0925</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>30.86</v>
+        <v>12.93</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>22.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -3107,44 +3107,44 @@
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>27.31</v>
+        <v>32.56</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>27.86</v>
+        <v>30.73</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>0.0201</v>
+        <v>-0.0563</v>
       </c>
       <c r="K29" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0608</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>26.27</v>
+        <v>12.53</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>23.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3159,12 +3159,12 @@
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -3173,18 +3173,18 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>37.25</v>
+        <v>43.19</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>38.14</v>
+        <v>43.88</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J30" s="7" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K30" s="11" t="inlineStr">
+      <c r="J30" s="9" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="K30" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3195,22 +3195,22 @@
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0188</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0016</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>23.8</v>
+        <v>32.16</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>27.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
@@ -3225,12 +3225,12 @@
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -3239,20 +3239,20 @@
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>105.01</v>
+        <v>137.37</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I31" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>-0.0001</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
@@ -3261,22 +3261,22 @@
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0432</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.002</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>10.01</v>
+        <v>30.86</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>17.6</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3286,39 +3286,39 @@
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>26.25</v>
+        <v>27.31</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>25.64</v>
+        <v>27.86</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-0.0232</v>
+        <v>0.0201</v>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
@@ -3327,22 +3327,22 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0392</v>
       </c>
       <c r="N32" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0114</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>16.26</v>
+        <v>26.27</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -3352,37 +3352,37 @@
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G33" s="5" t="n">
-        <v>10.7</v>
+        <v>37.25</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>10.73</v>
+        <v>38.14</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J33" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K33" s="11" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J33" s="9" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K33" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3393,22 +3393,22 @@
         </is>
       </c>
       <c r="M33" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0379</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>14.8</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3418,122 +3418,320 @@
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G34" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>11.24</v>
+        <v>105</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J34" s="9" t="n">
-        <v>-0.0568</v>
-      </c>
-      <c r="K34" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J34" s="7" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M34" s="8" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.022</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>33.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E35" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J35" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L35" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O35" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P35" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E36" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J36" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K36" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M36" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N36" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P36" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E37" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H37" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J37" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K37" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L37" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P37" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B35" s="3" t="inlineStr">
+      <c r="B38" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
+      <c r="C38" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D35" s="3" t="inlineStr">
+      <c r="D38" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E35" s="4" t="inlineStr">
+      <c r="E38" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F35" s="3" t="inlineStr">
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G35" s="5" t="n">
+      <c r="G38" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H35" s="5" t="n">
+      <c r="H38" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I35" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J35" s="9" t="n">
+      <c r="I38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J38" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K35" s="10" t="inlineStr">
+      <c r="K38" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L35" s="4" t="inlineStr">
+      <c r="L38" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M35" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N35" s="8" t="n">
+      <c r="M38" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N38" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O35" s="6" t="n">
+      <c r="O38" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P35" s="6" t="n">
+      <c r="P38" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3568,7 +3766,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-20T02:02:30</t>
+          <t>محسوب في: 2026-05-21T02:02:48</t>
         </is>
       </c>
     </row>
@@ -3592,7 +3790,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>32</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6">
@@ -3612,7 +3810,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8">
@@ -3622,7 +3820,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -3633,7 +3831,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>31.2%</t>
+          <t>31.4%</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3843,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>+3.58%</t>
+          <t>+3.76%</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3855,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.86%</t>
+          <t>-3.84%</t>
         </is>
       </c>
     </row>
@@ -3668,7 +3866,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.42</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="13">
@@ -3679,7 +3877,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-49.17%</t>
+          <t>-50.94%</t>
         </is>
       </c>
     </row>
@@ -3767,19 +3965,19 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C25" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>-4.47%</t>
+          <t>-2.47%</t>
         </is>
       </c>
     </row>
@@ -3813,19 +4011,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>9</v>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>40.9%</t>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>37.5%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.73%</t>
+          <t>-0.97%</t>
         </is>
       </c>
     </row>
@@ -3919,19 +4117,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C35" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>11.1%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-3.23%</t>
+          <t>-2.35%</t>
         </is>
       </c>
     </row>
@@ -3965,19 +4163,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D37" s="16" t="inlineStr">
-        <is>
-          <t>60.0%</t>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-0.74%</t>
+          <t>-1.05%</t>
         </is>
       </c>
     </row>
@@ -4126,7 +4324,7 @@
         </is>
       </c>
       <c r="B44" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C44" s="3" t="n">
         <v>0</v>
@@ -4138,7 +4336,7 @@
       </c>
       <c r="E44" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-3.39%</t>
         </is>
       </c>
     </row>
@@ -4228,7 +4426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I30"/>
+  <dimension ref="A1:I32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4662,7 +4860,7 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
@@ -4671,85 +4869,85 @@
         </is>
       </c>
       <c r="C13" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D13" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E13" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F13" s="17" t="inlineStr">
-        <is>
-          <t>33.3%</t>
+        <v>0</v>
+      </c>
+      <c r="F13" s="16" t="inlineStr">
+        <is>
+          <t>100.0%</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
         <is>
-          <t>-2.58%</t>
+          <t>+5.54%</t>
         </is>
       </c>
       <c r="H13" s="3" t="inlineStr">
         <is>
-          <t>+3.53%</t>
+          <t>+5.54%</t>
         </is>
       </c>
       <c r="I13" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>+5.54%</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D14" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>2</v>
+      </c>
+      <c r="F14" s="17" t="inlineStr">
+        <is>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-2.58%</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+3.53%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
@@ -4768,29 +4966,29 @@
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -4809,29 +5007,29 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -4850,29 +5048,29 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -4891,29 +5089,29 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -4932,29 +5130,29 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -4973,111 +5171,111 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D21" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E21" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F21" s="17" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="3" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="F22" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-4.78%</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-4.78%</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-4.78%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
@@ -5096,39 +5294,39 @@
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>-1.70%</t>
+          <t>-3.53%</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-2.60%</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-4.46%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D24" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E24" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
@@ -5137,29 +5335,29 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-1.70%</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-2.56%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
@@ -5178,29 +5376,29 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -5219,29 +5417,29 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -5260,29 +5458,29 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -5301,29 +5499,29 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -5342,58 +5540,140 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
+          <t>2110</t>
+        </is>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>-5.65%</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="3" t="inlineStr">
+        <is>
           <t>4280</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B31" s="4" t="inlineStr">
         <is>
           <t>عقار</t>
         </is>
       </c>
-      <c r="C30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D30" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="E30" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F30" s="3" t="inlineStr">
+      <c r="C31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>-5.55%</t>
         </is>
       </c>
-      <c r="H30" s="3" t="inlineStr">
+      <c r="H31" s="3" t="inlineStr">
         <is>
           <t>-5.55%</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
+      <c r="I31" s="3" t="inlineStr">
         <is>
           <t>-5.55%</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>7202</t>
+        </is>
+      </c>
+      <c r="B32" s="4" t="inlineStr">
+        <is>
+          <t>تقنية</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D32" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>-4.71%</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>-4.71%</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>-4.71%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-05-22_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -146,10 +146,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -648,63 +648,63 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>128.16</v>
+        <v>12.66</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>121.51</v>
+        <v>12.03</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>135.22</v>
+        <v>13.29</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>140.71</v>
+        <v>13.92</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>5.12</v>
+        <v>10.24</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>38%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>128</v>
+        <v>12.63</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-0.12</v>
+        <v>-0.24</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>2.06</v>
+        <v>1.11</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-1.69</v>
+        <v>-2.76</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
@@ -715,63 +715,63 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>14.64</v>
+        <v>45.37</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>13.88</v>
+        <v>43.9</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>15.47</v>
+        <v>46.84</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>16.12</v>
+        <v>48.31</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>3.78</v>
+        <v>15.11</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
-          <t>41%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>14.2</v>
+        <v>45</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>-3.01</v>
+        <v>-0.82</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>0.55</v>
+        <v>0</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-4.3</v>
+        <v>-3.02</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -782,63 +782,63 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0042</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>4190</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>11.35</v>
+        <v>15.71</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>10.76</v>
+        <v>15.31</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>12.01</v>
+        <v>16.12</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>12.51</v>
+        <v>16.52</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>16.05</v>
+        <v>9.49</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>68%</t>
+          <t>-</t>
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>10.9</v>
-      </c>
-      <c r="N6" s="7" t="n">
-        <v>-3.96</v>
+        <v>15.77</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>0.38</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>3</v>
+        <v>0.38</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-4.85</v>
+        <v>-1.46</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,43 +849,43 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0043</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2270</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>32.97</v>
+        <v>224.35</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>31.39</v>
+        <v>213.89</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>34.55</v>
+        <v>234.81</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>36.13</v>
+        <v>245.27</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>7.94</v>
+        <v>14.29</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>32.76</v>
+        <v>221.4</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>-0.64</v>
+        <v>-1.31</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>1</v>
+        <v>1.58</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-2.88</v>
+        <v>-1.31</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,22 +916,22 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0040</t>
+          <t>T0044</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
@@ -940,19 +940,19 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>12.66</v>
+        <v>196.39</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>12.03</v>
+        <v>185.26</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>13.29</v>
+        <v>207.52</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>13.92</v>
+        <v>218.65</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>10.24</v>
+        <v>13.57</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -960,19 +960,19 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>12.62</v>
+        <v>195.9</v>
       </c>
       <c r="N8" s="7" t="n">
-        <v>-0.32</v>
+        <v>-0.25</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>1.11</v>
+        <v>0.31</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-2.76</v>
+        <v>-1.22</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,22 +983,22 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0041</t>
+          <t>T0045</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
@@ -1007,19 +1007,19 @@
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>45.37</v>
+        <v>87.52</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>43.9</v>
+        <v>83.53</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>46.84</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>48.31</v>
+        <v>95.5</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>15.11</v>
+        <v>10.05</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1030,16 +1030,16 @@
         <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>44.4</v>
-      </c>
-      <c r="N9" s="7" t="n">
-        <v>-2.14</v>
+        <v>89.75</v>
+      </c>
+      <c r="N9" s="9" t="n">
+        <v>2.55</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>0</v>
+        <v>2.55</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-3.02</v>
+        <v>-3.22</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,43 +1050,43 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0042</t>
+          <t>T0046</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>4190</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>15.71</v>
+        <v>12.37</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>15.31</v>
+        <v>11.65</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>16.12</v>
+        <v>13.09</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>16.52</v>
+        <v>13.81</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>9.49</v>
+        <v>13.56</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1094,19 +1094,19 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>15.73</v>
-      </c>
-      <c r="N10" s="9" t="n">
-        <v>0.13</v>
+        <v>12.37</v>
+      </c>
+      <c r="N10" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="P10" s="8" t="n">
-        <v>-1.46</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
@@ -1117,22 +1117,22 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0043</t>
+          <t>T0047</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2270</t>
+          <t>4263</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1141,19 +1141,19 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>224.35</v>
+        <v>171.04</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>213.89</v>
+        <v>165.88</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>234.81</v>
+        <v>176.2</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>245.27</v>
+        <v>181.36</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>14.29</v>
+        <v>13.09</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>224.35</v>
+        <v>171.04</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1184,43 +1184,43 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0044</t>
+          <t>T0048</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>8313</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>196.39</v>
+        <v>151.3</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>185.26</v>
+        <v>144.55</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>207.52</v>
+        <v>158.05</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>218.65</v>
+        <v>164.8</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>13.57</v>
+        <v>13.08</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>196.39</v>
+        <v>151.3</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1251,43 +1251,43 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0045</t>
+          <t>T0049</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>8120</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>87.52</v>
+        <v>11.8</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>83.53</v>
+        <v>11.31</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>91.51000000000001</v>
+        <v>12.29</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>95.5</v>
+        <v>12.79</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>10.05</v>
+        <v>11.96</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>87.52</v>
+        <v>11.8</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P38"/>
+  <dimension ref="A1:P42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,22 +1428,22 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
@@ -1457,20 +1457,20 @@
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>15.33</v>
+        <v>128.16</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>16.18</v>
+        <v>127.3</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J4" s="9" t="n">
-        <v>0.0554</v>
+      <c r="J4" s="7" t="n">
+        <v>-0.0067</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
@@ -1479,62 +1479,62 @@
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0698</v>
+        <v>0.0206</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0033</v>
+        <v>-0.0169</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>9.57</v>
+        <v>5.12</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>47.4</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>14.6</v>
+        <v>14.64</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>14.22</v>
+        <v>14.3</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>-0.026</v>
-      </c>
-      <c r="K5" s="11" t="inlineStr">
+        <v>-0.0232</v>
+      </c>
+      <c r="K5" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1545,22 +1545,22 @@
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.0445</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0322</v>
+        <v>-0.043</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>3.63</v>
+        <v>3.78</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>16.8</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1589,59 +1589,59 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>230.06</v>
+        <v>11.35</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>219.22</v>
+        <v>10.97</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>-0.0471</v>
-      </c>
-      <c r="K6" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0335</v>
+      </c>
+      <c r="K6" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.005</v>
+        <v>0.03</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.0559</v>
+        <v>-0.04849999999999999</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>12.77</v>
+        <v>16.05</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>31.9</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1655,18 +1655,18 @@
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>28.94</v>
+        <v>32.97</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>28.7</v>
+        <v>32.12</v>
       </c>
       <c r="I7" s="3" t="n">
         <v>4</v>
       </c>
       <c r="J7" s="7" t="n">
-        <v>-0.0083</v>
-      </c>
-      <c r="K7" s="11" t="inlineStr">
+        <v>-0.0258</v>
+      </c>
+      <c r="K7" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1677,108 +1677,108 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0048</v>
+        <v>0.01</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0256</v>
+        <v>-0.0288</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>3</v>
+        <v>7.94</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>28.4</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>11.03</v>
+        <v>15.33</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>10.42</v>
+        <v>16.18</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J8" s="7" t="n">
-        <v>-0.0555</v>
+        <v>7</v>
+      </c>
+      <c r="J8" s="9" t="n">
+        <v>0.0554</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0063</v>
+        <v>0.0698</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.07980000000000001</v>
+        <v>-0.0033</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>10.8</v>
+        <v>9.57</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>32.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1787,64 +1787,64 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>158.92</v>
+        <v>14.6</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>149.94</v>
+        <v>14.22</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J9" s="7" t="n">
-        <v>-0.0565</v>
-      </c>
-      <c r="K9" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.026</v>
+      </c>
+      <c r="K9" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0</v>
+        <v>0.0445</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0624</v>
+        <v>-0.0322</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3.46</v>
+        <v>3.63</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>14.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
@@ -1853,59 +1853,59 @@
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>100.3</v>
+        <v>230.06</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>97</v>
+        <v>219.22</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J10" s="7" t="n">
-        <v>-0.0329</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>-0.0471</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.006</v>
+        <v>0.005</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0559</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>9.9</v>
+        <v>12.77</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>25.2</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1915,134 +1915,134 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>195.39</v>
+        <v>28.94</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>184.32</v>
+        <v>28.7</v>
       </c>
       <c r="I11" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J11" s="7" t="n">
+        <v>-0.0083</v>
+      </c>
+      <c r="K11" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L11" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>0.0048</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="O11" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>-0.0566</v>
-      </c>
-      <c r="K11" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>Stop Hit</t>
-        </is>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>0.05429999999999999</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>-0.0634</v>
-      </c>
-      <c r="O11" s="6" t="n">
-        <v>8.51</v>
-      </c>
       <c r="P11" s="6" t="n">
-        <v>43.7</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>32.56</v>
+        <v>11.03</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>32.9</v>
+        <v>10.42</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J12" s="9" t="n">
-        <v>0.0353</v>
+        <v>2</v>
+      </c>
+      <c r="J12" s="7" t="n">
+        <v>-0.0555</v>
       </c>
       <c r="K12" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0663</v>
+        <v>0.0063</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>12.52</v>
+        <v>10.8</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>43.3</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2051,18 +2051,18 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>11.82</v>
+        <v>158.92</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>11.15</v>
+        <v>149.94</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="J13" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
+        <v>-0.0565</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2073,22 +2073,22 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.0624</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>16.94</v>
+        <v>3.46</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>25.6</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
@@ -2098,17 +2098,17 @@
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
@@ -2117,130 +2117,130 @@
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>45.31</v>
+        <v>100.3</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>43.14</v>
+        <v>97</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K14" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0329</v>
+      </c>
+      <c r="K14" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>12.84</v>
+        <v>9.9</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>28.7</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>12.24</v>
+        <v>195.39</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>12.9</v>
+        <v>184.32</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J15" s="9" t="n">
-        <v>0.0609</v>
+        <v>3</v>
+      </c>
+      <c r="J15" s="7" t="n">
+        <v>-0.0566</v>
       </c>
       <c r="K15" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0634</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>16.08</v>
+        <v>8.51</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>36.7</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2249,20 +2249,20 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>25.85</v>
+        <v>32.56</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>25.22</v>
+        <v>32.9</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J16" s="7" t="n">
-        <v>-0.0244</v>
+      <c r="J16" s="9" t="n">
+        <v>0.0353</v>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
@@ -2271,42 +2271,42 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0</v>
+        <v>0.0663</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0012</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>14.35</v>
+        <v>12.52</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>26.1</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2315,64 +2315,64 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>90.63</v>
+        <v>11.82</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>11.15</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J17" s="9" t="n">
-        <v>0.0416</v>
+        <v>1</v>
+      </c>
+      <c r="J17" s="7" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K17" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.057</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>0</v>
+        <v>-0.0728</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>14.18</v>
+        <v>16.94</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>23</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -2381,44 +2381,44 @@
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>15.53</v>
+        <v>45.31</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>15.88</v>
+        <v>43.14</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J18" s="9" t="n">
-        <v>0.0267</v>
+        <v>3</v>
+      </c>
+      <c r="J18" s="7" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K18" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L18" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.038</v>
+        <v>0</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>0</v>
+        <v>-0.0461</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>11.78</v>
+        <v>12.84</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>19.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
@@ -2433,12 +2433,12 @@
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2447,20 +2447,20 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>694.39</v>
+        <v>12.24</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>680</v>
+        <v>12.9</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J19" s="7" t="n">
-        <v>-0.0207</v>
+      <c r="J19" s="9" t="n">
+        <v>0.0609</v>
       </c>
       <c r="K19" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
@@ -2469,42 +2469,42 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0254</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0517</v>
+        <v>-0.0155</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>10.02</v>
+        <v>16.08</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>23.7</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2513,18 +2513,18 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>15.01</v>
+        <v>25.85</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>14.34</v>
+        <v>25.22</v>
       </c>
       <c r="I20" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>-0.0446</v>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
+        <v>-0.0244</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2535,64 +2535,64 @@
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.0127</v>
+        <v>0</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0466</v>
+        <v>-0.0352</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>11.78</v>
+        <v>14.35</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>11.8</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>28.9</v>
+        <v>90.63</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>28.16</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J21" s="7" t="n">
-        <v>-0.0256</v>
+        <v>5</v>
+      </c>
+      <c r="J21" s="9" t="n">
+        <v>0.0416</v>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
@@ -2601,42 +2601,42 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0</v>
+        <v>0.057</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0436</v>
+        <v>0</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>12.9</v>
+        <v>14.18</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>32.8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2645,20 +2645,20 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>70.64</v>
+        <v>15.53</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>69</v>
+        <v>15.88</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J22" s="7" t="n">
-        <v>-0.0232</v>
+      <c r="J22" s="9" t="n">
+        <v>0.0267</v>
       </c>
       <c r="K22" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L22" s="4" t="inlineStr">
@@ -2667,42 +2667,42 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.038</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0331</v>
+        <v>0</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>24.18</v>
+        <v>11.78</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>13.3</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,44 +2711,44 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>182.46</v>
+        <v>694.39</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>198.78</v>
+        <v>680</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J23" s="9" t="n">
-        <v>0.08939999999999999</v>
+      <c r="J23" s="7" t="n">
+        <v>-0.0207</v>
       </c>
       <c r="K23" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0254</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0517</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>23.45</v>
+        <v>10.02</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>12.1</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -2758,103 +2758,103 @@
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>14.05</v>
+        <v>15.01</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>13.25</v>
+        <v>14.34</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K24" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0446</v>
+      </c>
+      <c r="K24" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0036</v>
+        <v>0.0127</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0466</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>14.88</v>
+        <v>11.78</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>35.5</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>14.64</v>
+        <v>28.9</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>14.51</v>
+        <v>28.16</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K25" s="11" t="inlineStr">
+        <v>-0.0256</v>
+      </c>
+      <c r="K25" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2865,37 +2865,37 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.0089</v>
+        <v>0</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0436</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>12.9</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>20.2</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C26" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
@@ -2909,64 +2909,64 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>32.56</v>
+        <v>70.64</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>30.73</v>
+        <v>69</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J26" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0232</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L26" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0178</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0331</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>15.98</v>
+        <v>24.18</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>43.3</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C27" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2975,59 +2975,59 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>45.31</v>
+        <v>182.46</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>43.14</v>
+        <v>198.78</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J27" s="7" t="n">
-        <v>-0.0478</v>
+        <v>5</v>
+      </c>
+      <c r="J27" s="9" t="n">
+        <v>0.08939999999999999</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0</v>
+        <v>0.106</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0036</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>13.05</v>
+        <v>23.45</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>28.7</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C28" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
@@ -3037,22 +3037,22 @@
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>45.31</v>
+        <v>14.05</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>43.14</v>
+        <v>13.25</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J28" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K28" s="11" t="inlineStr">
+        <v>-0.0567</v>
+      </c>
+      <c r="K28" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -3063,108 +3063,108 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.079</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>12.93</v>
+        <v>14.88</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>28.7</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C29" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>32.56</v>
+        <v>14.64</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>30.73</v>
+        <v>14.51</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J29" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K29" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0089</v>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L29" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0089</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0294</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>12.53</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>43.3</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -3173,64 +3173,64 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>43.19</v>
+        <v>32.56</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>43.88</v>
+        <v>30.73</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J30" s="9" t="n">
-        <v>0.016</v>
+        <v>1</v>
+      </c>
+      <c r="J30" s="7" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.0188</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0608</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>32.16</v>
+        <v>15.98</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>13</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
@@ -3239,64 +3239,64 @@
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>137.37</v>
+        <v>45.31</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>143</v>
+        <v>43.14</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J31" s="9" t="n">
-        <v>0.04099999999999999</v>
+        <v>1</v>
+      </c>
+      <c r="J31" s="7" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K31" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0.0432</v>
+        <v>0</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0925</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>30.86</v>
+        <v>13.05</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>22.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
@@ -3305,64 +3305,64 @@
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>27.31</v>
+        <v>45.31</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>27.86</v>
+        <v>43.14</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J32" s="9" t="n">
-        <v>0.0201</v>
+        <v>1</v>
+      </c>
+      <c r="J32" s="7" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K32" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0.0392</v>
+        <v>0</v>
       </c>
       <c r="N32" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0925</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>26.27</v>
+        <v>12.93</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>23.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C33" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -3371,44 +3371,44 @@
         </is>
       </c>
       <c r="G33" s="5" t="n">
-        <v>37.25</v>
+        <v>32.56</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>38.14</v>
+        <v>30.73</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J33" s="9" t="n">
-        <v>0.0239</v>
+        <v>1</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K33" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M33" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0608</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>23.8</v>
+        <v>12.53</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>27.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3423,12 +3423,12 @@
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F34" s="3" t="inlineStr">
@@ -3437,20 +3437,20 @@
         </is>
       </c>
       <c r="G34" s="5" t="n">
-        <v>105.01</v>
+        <v>43.19</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>105</v>
+        <v>43.88</v>
       </c>
       <c r="I34" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J34" s="7" t="n">
-        <v>-0.0001</v>
+      <c r="J34" s="9" t="n">
+        <v>0.016</v>
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
@@ -3459,22 +3459,22 @@
         </is>
       </c>
       <c r="M34" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0188</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.0016</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>10.01</v>
+        <v>32.16</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>17.6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
@@ -3484,39 +3484,39 @@
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G35" s="5" t="n">
-        <v>26.25</v>
+        <v>137.37</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>25.64</v>
+        <v>143</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J35" s="7" t="n">
-        <v>-0.0232</v>
+        <v>5</v>
+      </c>
+      <c r="J35" s="9" t="n">
+        <v>0.04099999999999999</v>
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
@@ -3525,22 +3525,22 @@
         </is>
       </c>
       <c r="M35" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0432</v>
       </c>
       <c r="N35" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.002</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>16.26</v>
+        <v>30.86</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>31.4</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -3550,12 +3550,12 @@
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
@@ -3565,22 +3565,22 @@
       </c>
       <c r="F36" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G36" s="5" t="n">
-        <v>10.7</v>
+        <v>27.31</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>10.73</v>
+        <v>27.86</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K36" s="10" t="inlineStr">
+        <v>0.0201</v>
+      </c>
+      <c r="K36" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3591,22 +3591,22 @@
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0392</v>
       </c>
       <c r="N36" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0114</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>12.8</v>
+        <v>26.27</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>14.8</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -3616,122 +3616,386 @@
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G37" s="5" t="n">
-        <v>11.92</v>
+        <v>37.25</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>11.24</v>
+        <v>38.14</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J37" s="7" t="n">
-        <v>-0.0568</v>
+        <v>5</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>0.0239</v>
       </c>
       <c r="K37" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M37" s="8" t="n">
-        <v>0</v>
+        <v>0.0379</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.0212</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>12</v>
+        <v>23.8</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>33.5</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
+          <t>T0009</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-11</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>4016</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>رعاية صحية</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>breakout</t>
+        </is>
+      </c>
+      <c r="G38" s="5" t="n">
+        <v>105.01</v>
+      </c>
+      <c r="H38" s="5" t="n">
+        <v>105</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="J38" s="7" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K38" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M38" s="8" t="n">
+        <v>0.0075</v>
+      </c>
+      <c r="N38" s="8" t="n">
+        <v>-0.022</v>
+      </c>
+      <c r="O38" s="6" t="n">
+        <v>10.01</v>
+      </c>
+      <c r="P38" s="6" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C39" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E39" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H39" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J39" s="7" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K39" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L39" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O39" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P39" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E40" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G40" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H40" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J40" s="9" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L40" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M40" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N40" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P40" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C41" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E41" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H41" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J41" s="7" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K41" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L41" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N41" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P41" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
+      <c r="B42" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C42" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D42" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E38" s="4" t="inlineStr">
+      <c r="E42" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
+      <c r="F42" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G38" s="5" t="n">
+      <c r="G42" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H38" s="5" t="n">
+      <c r="H42" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I38" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J38" s="7" t="n">
+      <c r="I42" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J42" s="7" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K38" s="11" t="inlineStr">
+      <c r="K42" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L38" s="4" t="inlineStr">
+      <c r="L42" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M38" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N38" s="8" t="n">
+      <c r="M42" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N42" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O38" s="6" t="n">
+      <c r="O42" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P38" s="6" t="n">
+      <c r="P42" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -3766,7 +4030,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-21T02:02:48</t>
+          <t>محسوب في: 2026-05-22T02:02:50</t>
         </is>
       </c>
     </row>
@@ -3790,7 +4054,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>35</v>
+        <v>39</v>
       </c>
     </row>
     <row r="6">
@@ -3820,7 +4084,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -3831,7 +4095,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>31.4%</t>
+          <t>28.2%</t>
         </is>
       </c>
     </row>
@@ -3855,7 +4119,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.84%</t>
+          <t>-3.61%</t>
         </is>
       </c>
     </row>
@@ -3866,7 +4130,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.45</v>
+        <v>0.41</v>
       </c>
     </row>
     <row r="13">
@@ -3877,7 +4141,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-50.94%</t>
+          <t>-59.86%</t>
         </is>
       </c>
     </row>
@@ -3965,19 +4229,19 @@
         </is>
       </c>
       <c r="B25" s="3" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C25" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D25" s="17" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="E25" s="17" t="inlineStr">
         <is>
-          <t>-2.47%</t>
+          <t>-2.19%</t>
         </is>
       </c>
     </row>
@@ -3988,19 +4252,19 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C26" s="3" t="n">
         <v>1</v>
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>25.0%</t>
+          <t>20.0%</t>
         </is>
       </c>
       <c r="E26" s="17" t="inlineStr">
         <is>
-          <t>-1.79%</t>
+          <t>-1.95%</t>
         </is>
       </c>
     </row>
@@ -4011,19 +4275,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>9</v>
       </c>
       <c r="D27" s="17" t="inlineStr">
         <is>
-          <t>37.5%</t>
+          <t>36.0%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.97%</t>
+          <t>-1.07%</t>
         </is>
       </c>
     </row>
@@ -4117,19 +4381,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>15.4%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-2.35%</t>
+          <t>-2.24%</t>
         </is>
       </c>
     </row>
@@ -4163,19 +4427,19 @@
         </is>
       </c>
       <c r="B37" s="3" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="C37" s="3" t="n">
         <v>3</v>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>50.0%</t>
+          <t>42.9%</t>
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr">
         <is>
-          <t>-1.05%</t>
+          <t>-1.38%</t>
         </is>
       </c>
     </row>
@@ -4400,7 +4664,7 @@
     <row r="52">
       <c r="A52" s="21" t="inlineStr">
         <is>
-          <t>2370: 1/3 = 33.3%</t>
+          <t>2370: 1/4 = 25.0%</t>
         </is>
       </c>
     </row>
@@ -4426,7 +4690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I32"/>
+  <dimension ref="A1:I35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -4910,17 +5174,17 @@
         </is>
       </c>
       <c r="C14" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="D14" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
@@ -5674,6 +5938,129 @@
       <c r="I32" s="3" t="inlineStr">
         <is>
           <t>-4.71%</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
+        <is>
+          <t>2223</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D33" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G33" s="3" t="inlineStr">
+        <is>
+          <t>-0.67%</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>-0.67%</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>-0.67%</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>2250</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D34" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>-2.32%</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
+        <is>
+          <t>8180</t>
+        </is>
+      </c>
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D35" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G35" s="3" t="inlineStr">
+        <is>
+          <t>-3.35%</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>-3.35%</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>-3.35%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-06-01_11:52
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -82,12 +82,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
     <fill>
@@ -162,18 +162,18 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -648,43 +648,43 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0040</t>
+          <t>T0042</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>4190</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>12.66</v>
+        <v>15.71</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>12.03</v>
+        <v>15.31</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>13.29</v>
+        <v>16.12</v>
       </c>
       <c r="I4" s="5" t="n">
-        <v>13.92</v>
+        <v>16.52</v>
       </c>
       <c r="J4" s="6" t="n">
-        <v>10.24</v>
+        <v>9.49</v>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
@@ -695,37 +695,37 @@
         <v>3</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>12.63</v>
+        <v>16.13</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>-0.24</v>
+        <v>2.67</v>
       </c>
       <c r="O4" s="8" t="n">
-        <v>1.11</v>
+        <v>2.8</v>
       </c>
       <c r="P4" s="8" t="n">
-        <v>-2.76</v>
+        <v>-1.46</v>
       </c>
       <c r="Q4" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0041</t>
+          <t>T0043</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2270</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -739,19 +739,19 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>45.37</v>
+        <v>224.35</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>43.9</v>
+        <v>213.89</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>46.84</v>
+        <v>234.81</v>
       </c>
       <c r="I5" s="5" t="n">
-        <v>48.31</v>
+        <v>245.27</v>
       </c>
       <c r="J5" s="6" t="n">
-        <v>15.11</v>
+        <v>14.29</v>
       </c>
       <c r="K5" s="3" t="inlineStr">
         <is>
@@ -762,16 +762,16 @@
         <v>2</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>45</v>
+        <v>226.2</v>
       </c>
       <c r="N5" s="7" t="n">
-        <v>-0.82</v>
+        <v>0.82</v>
       </c>
       <c r="O5" s="8" t="n">
-        <v>0</v>
+        <v>1.58</v>
       </c>
       <c r="P5" s="8" t="n">
-        <v>-3.02</v>
+        <v>-1.31</v>
       </c>
       <c r="Q5" s="3" t="inlineStr">
         <is>
@@ -782,43 +782,43 @@
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0042</t>
+          <t>T0044</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>4190</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>15.71</v>
+        <v>196.39</v>
       </c>
       <c r="G6" s="5" t="n">
-        <v>15.31</v>
+        <v>185.26</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>16.12</v>
+        <v>207.52</v>
       </c>
       <c r="I6" s="5" t="n">
-        <v>16.52</v>
+        <v>218.65</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>9.49</v>
+        <v>13.57</v>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
@@ -829,16 +829,16 @@
         <v>2</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>15.77</v>
-      </c>
-      <c r="N6" s="9" t="n">
-        <v>0.38</v>
+        <v>197.5</v>
+      </c>
+      <c r="N6" s="7" t="n">
+        <v>0.57</v>
       </c>
       <c r="O6" s="8" t="n">
-        <v>0.38</v>
+        <v>4.64</v>
       </c>
       <c r="P6" s="8" t="n">
-        <v>-1.46</v>
+        <v>-1.22</v>
       </c>
       <c r="Q6" s="3" t="inlineStr">
         <is>
@@ -849,7 +849,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0043</t>
+          <t>T0045</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
@@ -859,12 +859,12 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2270</t>
+          <t>4100</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr">
@@ -873,19 +873,19 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>224.35</v>
+        <v>87.52</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>213.89</v>
+        <v>83.53</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>234.81</v>
+        <v>91.51000000000001</v>
       </c>
       <c r="I7" s="5" t="n">
-        <v>245.27</v>
+        <v>95.5</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>14.29</v>
+        <v>10.05</v>
       </c>
       <c r="K7" s="3" t="inlineStr">
         <is>
@@ -893,19 +893,19 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>221.4</v>
+        <v>89.59999999999999</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>-1.31</v>
+        <v>2.38</v>
       </c>
       <c r="O7" s="8" t="n">
-        <v>1.58</v>
+        <v>3.52</v>
       </c>
       <c r="P7" s="8" t="n">
-        <v>-1.31</v>
+        <v>-3.22</v>
       </c>
       <c r="Q7" s="3" t="inlineStr">
         <is>
@@ -916,43 +916,43 @@
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0044</t>
+          <t>T0047</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>4263</t>
         </is>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>196.39</v>
+        <v>171.04</v>
       </c>
       <c r="G8" s="5" t="n">
-        <v>185.26</v>
+        <v>165.88</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>207.52</v>
+        <v>176.2</v>
       </c>
       <c r="I8" s="5" t="n">
-        <v>218.65</v>
+        <v>181.36</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>13.57</v>
+        <v>13.09</v>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
@@ -963,16 +963,16 @@
         <v>1</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>195.9</v>
-      </c>
-      <c r="N8" s="7" t="n">
-        <v>-0.25</v>
+        <v>170</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>-0.61</v>
       </c>
       <c r="O8" s="8" t="n">
-        <v>0.31</v>
+        <v>0.44</v>
       </c>
       <c r="P8" s="8" t="n">
-        <v>-1.22</v>
+        <v>-0.9</v>
       </c>
       <c r="Q8" s="3" t="inlineStr">
         <is>
@@ -983,43 +983,43 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0045</t>
+          <t>T0048</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>4100</t>
+          <t>8313</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>87.52</v>
+        <v>151.3</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>83.53</v>
+        <v>144.55</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>91.51000000000001</v>
+        <v>158.05</v>
       </c>
       <c r="I9" s="5" t="n">
-        <v>95.5</v>
+        <v>164.8</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>10.05</v>
+        <v>13.08</v>
       </c>
       <c r="K9" s="3" t="inlineStr">
         <is>
@@ -1030,16 +1030,16 @@
         <v>1</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>89.75</v>
+        <v>149.9</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>2.55</v>
+        <v>-0.93</v>
       </c>
       <c r="O9" s="8" t="n">
-        <v>2.55</v>
+        <v>3.04</v>
       </c>
       <c r="P9" s="8" t="n">
-        <v>-3.22</v>
+        <v>-1.12</v>
       </c>
       <c r="Q9" s="3" t="inlineStr">
         <is>
@@ -1050,7 +1050,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0046</t>
+          <t>T0049</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1060,33 +1060,33 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>8120</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>12.37</v>
+        <v>11.8</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>11.65</v>
+        <v>11.31</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>13.09</v>
+        <v>12.29</v>
       </c>
       <c r="I10" s="5" t="n">
-        <v>13.81</v>
+        <v>12.79</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>13.56</v>
+        <v>11.96</v>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
@@ -1094,45 +1094,45 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>12.37</v>
-      </c>
-      <c r="N10" s="8" t="n">
-        <v>0</v>
+        <v>12.19</v>
+      </c>
+      <c r="N10" s="7" t="n">
+        <v>3.31</v>
       </c>
       <c r="O10" s="8" t="n">
-        <v>0</v>
+        <v>5.85</v>
       </c>
       <c r="P10" s="8" t="n">
         <v>0</v>
       </c>
       <c r="Q10" s="3" t="inlineStr">
         <is>
-          <t>🟢 Active</t>
+          <t>🟡 Partial</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0047</t>
+          <t>T0050</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>4263</t>
+          <t>2340</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr">
@@ -1141,19 +1141,19 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>171.04</v>
+        <v>10.83</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>165.88</v>
+        <v>10.54</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>176.2</v>
+        <v>11.12</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>181.36</v>
+        <v>11.41</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>13.09</v>
+        <v>12.05</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>171.04</v>
+        <v>10.83</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1184,43 +1184,43 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0048</t>
+          <t>T0051</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>8313</t>
+          <t>4061</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F12" s="5" t="n">
-        <v>151.3</v>
+        <v>11.31</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>144.55</v>
+        <v>10.98</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>158.05</v>
+        <v>11.64</v>
       </c>
       <c r="I12" s="5" t="n">
-        <v>164.8</v>
+        <v>11.97</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>13.08</v>
+        <v>10.67</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1231,7 +1231,7 @@
         <v>0</v>
       </c>
       <c r="M12" s="5" t="n">
-        <v>151.3</v>
+        <v>11.31</v>
       </c>
       <c r="N12" s="8" t="n">
         <v>0</v>
@@ -1251,43 +1251,43 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0049</t>
+          <t>T0052</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>8120</t>
+          <t>4170</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>11.8</v>
+        <v>16.6</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>11.31</v>
+        <v>16.06</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>12.29</v>
+        <v>17.14</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>12.79</v>
+        <v>17.68</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>11.96</v>
+        <v>10.43</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>11.8</v>
+        <v>16.6</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P42"/>
+  <dimension ref="A1:P45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,159 +1428,159 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>128.16</v>
+        <v>12.66</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>127.3</v>
+        <v>13.91</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="J4" s="7" t="n">
-        <v>-0.0067</v>
+        <v>0.0984</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.0206</v>
+        <v>0.2062</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0169</v>
+        <v>-0.0276</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>5.12</v>
+        <v>10.24</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>35.2</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>14.64</v>
+        <v>45.37</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>14.3</v>
+        <v>48.26</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="J5" s="7" t="n">
-        <v>-0.0232</v>
+        <v>0.06370000000000001</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.102</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.043</v>
+        <v>-0.0302</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>3.78</v>
+        <v>15.11</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>15.7</v>
+        <v>26.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0046</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1589,49 +1589,49 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>11.35</v>
+        <v>12.37</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>10.97</v>
+        <v>13.8</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J6" s="7" t="n">
-        <v>-0.0335</v>
+        <v>0.1153</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.03</v>
+        <v>0.207</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>-0.04849999999999999</v>
+        <v>0</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>16.05</v>
+        <v>13.56</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>36.6</v>
+        <v>28</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
@@ -1641,7 +1641,7 @@
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
@@ -1651,22 +1651,22 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>32.97</v>
+        <v>128.16</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>32.12</v>
+        <v>127.3</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J7" s="7" t="n">
-        <v>-0.0258</v>
-      </c>
-      <c r="K7" s="10" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="J7" s="9" t="n">
+        <v>-0.0067</v>
+      </c>
+      <c r="K7" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1677,37 +1677,37 @@
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.01</v>
+        <v>0.0206</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0288</v>
+        <v>-0.0169</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>7.94</v>
+        <v>5.12</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>45.4</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
@@ -1721,20 +1721,20 @@
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>15.33</v>
+        <v>14.64</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>16.18</v>
+        <v>14.3</v>
       </c>
       <c r="I8" s="3" t="n">
         <v>7</v>
       </c>
       <c r="J8" s="9" t="n">
-        <v>0.0554</v>
+        <v>-0.0232</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
@@ -1743,37 +1743,37 @@
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.0698</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.0033</v>
+        <v>-0.043</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>9.57</v>
+        <v>3.78</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>47.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
@@ -1787,18 +1787,18 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>14.6</v>
+        <v>11.35</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>14.22</v>
+        <v>10.97</v>
       </c>
       <c r="I9" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J9" s="7" t="n">
-        <v>-0.026</v>
-      </c>
-      <c r="K9" s="10" t="inlineStr">
+      <c r="J9" s="9" t="n">
+        <v>-0.0335</v>
+      </c>
+      <c r="K9" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1809,22 +1809,22 @@
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.0445</v>
+        <v>0.03</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.0322</v>
+        <v>-0.04849999999999999</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>3.63</v>
+        <v>16.05</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>16.8</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
@@ -1834,78 +1834,78 @@
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>230.06</v>
+        <v>32.97</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>219.22</v>
+        <v>32.12</v>
       </c>
       <c r="I10" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J10" s="7" t="n">
-        <v>-0.0471</v>
-      </c>
-      <c r="K10" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+      <c r="J10" s="9" t="n">
+        <v>-0.0258</v>
+      </c>
+      <c r="K10" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L10" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0559</v>
+        <v>-0.0288</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>12.77</v>
+        <v>7.94</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>31.9</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1915,24 +1915,24 @@
       </c>
       <c r="F11" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>28.94</v>
+        <v>15.33</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>28.7</v>
+        <v>16.18</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J11" s="7" t="n">
-        <v>-0.0083</v>
+        <v>0.0554</v>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1941,108 +1941,108 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0048</v>
+        <v>0.0698</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0256</v>
+        <v>-0.0033</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>3</v>
+        <v>9.57</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>28.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>11.03</v>
+        <v>14.6</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>10.42</v>
+        <v>14.22</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J12" s="7" t="n">
-        <v>-0.0555</v>
-      </c>
-      <c r="K12" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J12" s="9" t="n">
+        <v>-0.026</v>
+      </c>
+      <c r="K12" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L12" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0063</v>
+        <v>0.0445</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.07980000000000001</v>
+        <v>-0.0322</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>10.8</v>
+        <v>3.63</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>32.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
@@ -2051,18 +2051,18 @@
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>158.92</v>
+        <v>230.06</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>149.94</v>
+        <v>219.22</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>4</v>
       </c>
-      <c r="J13" s="7" t="n">
-        <v>-0.0565</v>
-      </c>
-      <c r="K13" s="10" t="inlineStr">
+      <c r="J13" s="9" t="n">
+        <v>-0.0471</v>
+      </c>
+      <c r="K13" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2073,62 +2073,62 @@
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0624</v>
+        <v>-0.0559</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>3.46</v>
+        <v>12.77</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>14.4</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>100.3</v>
+        <v>28.94</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>97</v>
+        <v>28.7</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J14" s="7" t="n">
-        <v>-0.0329</v>
-      </c>
-      <c r="K14" s="10" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="J14" s="9" t="n">
+        <v>-0.0083</v>
+      </c>
+      <c r="K14" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2139,62 +2139,62 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0048</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0256</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>9.9</v>
+        <v>3</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>25.2</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>195.39</v>
+        <v>11.03</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>184.32</v>
+        <v>10.42</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J15" s="7" t="n">
-        <v>-0.0566</v>
-      </c>
-      <c r="K15" s="10" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J15" s="9" t="n">
+        <v>-0.0555</v>
+      </c>
+      <c r="K15" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2205,37 +2205,37 @@
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.05429999999999999</v>
+        <v>0.0063</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.0634</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>8.51</v>
+        <v>10.8</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>43.7</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
@@ -2249,64 +2249,64 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>32.56</v>
+        <v>158.92</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>32.9</v>
+        <v>149.94</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>0.0353</v>
+        <v>-0.0565</v>
       </c>
       <c r="K16" s="11" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L16" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0.0663</v>
+        <v>0</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.0624</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>12.52</v>
+        <v>3.46</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>43.3</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
@@ -2315,84 +2315,84 @@
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>11.82</v>
+        <v>100.3</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>11.15</v>
+        <v>97</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J17" s="7" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K17" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J17" s="9" t="n">
+        <v>-0.0329</v>
+      </c>
+      <c r="K17" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L17" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>16.94</v>
+        <v>9.9</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>25.6</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>45.31</v>
+        <v>195.39</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>43.14</v>
+        <v>184.32</v>
       </c>
       <c r="I18" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="J18" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K18" s="10" t="inlineStr">
+      <c r="J18" s="9" t="n">
+        <v>-0.0566</v>
+      </c>
+      <c r="K18" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2403,42 +2403,42 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0634</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>12.84</v>
+        <v>8.51</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>28.7</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F19" s="3" t="inlineStr">
@@ -2447,18 +2447,18 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>12.24</v>
+        <v>32.56</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>12.9</v>
+        <v>32.9</v>
       </c>
       <c r="I19" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J19" s="9" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K19" s="11" t="inlineStr">
+      <c r="J19" s="7" t="n">
+        <v>0.0353</v>
+      </c>
+      <c r="K19" s="10" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2469,42 +2469,42 @@
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.0663</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0012</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>16.08</v>
+        <v>12.52</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>36.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2513,64 +2513,64 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>25.85</v>
+        <v>11.82</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>25.22</v>
+        <v>11.15</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J20" s="7" t="n">
-        <v>-0.0244</v>
-      </c>
-      <c r="K20" s="10" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>1</v>
+      </c>
+      <c r="J20" s="9" t="n">
+        <v>-0.0563</v>
+      </c>
+      <c r="K20" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0728</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>14.35</v>
+        <v>16.94</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>26.1</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
@@ -2579,44 +2579,44 @@
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>90.63</v>
+        <v>45.31</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>43.14</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>0.0416</v>
+        <v>-0.0478</v>
       </c>
       <c r="K21" s="11" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L21" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>0</v>
+        <v>-0.0461</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>14.18</v>
+        <v>12.84</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>23</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -2631,12 +2631,12 @@
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2645,18 +2645,18 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>15.53</v>
+        <v>12.24</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>15.88</v>
+        <v>12.9</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J22" s="9" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K22" s="11" t="inlineStr">
+      <c r="J22" s="7" t="n">
+        <v>0.0609</v>
+      </c>
+      <c r="K22" s="10" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2667,22 +2667,22 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.038</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>19.9</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
@@ -2697,12 +2697,12 @@
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,18 +2711,18 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>694.39</v>
+        <v>25.85</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>680</v>
+        <v>25.22</v>
       </c>
       <c r="I23" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J23" s="7" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K23" s="10" t="inlineStr">
+      <c r="J23" s="9" t="n">
+        <v>-0.0244</v>
+      </c>
+      <c r="K23" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2733,42 +2733,42 @@
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0.0254</v>
+        <v>0</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0517</v>
+        <v>-0.0352</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>10.02</v>
+        <v>14.35</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>23.7</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2777,20 +2777,20 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>15.01</v>
+        <v>90.63</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>14.34</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I24" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>-0.0446</v>
+        <v>0.0416</v>
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
@@ -2799,64 +2799,64 @@
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.057</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>11.8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C25" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>28.9</v>
+        <v>15.53</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>28.16</v>
+        <v>15.88</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>-0.0256</v>
+        <v>0.0267</v>
       </c>
       <c r="K25" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L25" s="4" t="inlineStr">
@@ -2865,42 +2865,42 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N25" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N25" s="8" t="n">
-        <v>-0.0436</v>
-      </c>
       <c r="O25" s="6" t="n">
-        <v>12.9</v>
+        <v>11.78</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>32.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2909,18 +2909,18 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>70.64</v>
+        <v>694.39</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>69</v>
+        <v>680</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J26" s="7" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K26" s="10" t="inlineStr">
+      <c r="J26" s="9" t="n">
+        <v>-0.0207</v>
+      </c>
+      <c r="K26" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2931,42 +2931,42 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0254</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0517</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>24.18</v>
+        <v>10.02</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>13.3</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2975,115 +2975,115 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>182.46</v>
+        <v>15.01</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>198.78</v>
+        <v>14.34</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J27" s="9" t="n">
-        <v>0.08939999999999999</v>
+        <v>-0.0446</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0127</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0466</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>23.45</v>
+        <v>11.78</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>14.05</v>
+        <v>28.9</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>13.25</v>
+        <v>28.16</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="J28" s="7" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K28" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>3</v>
+      </c>
+      <c r="J28" s="9" t="n">
+        <v>-0.0256</v>
+      </c>
+      <c r="K28" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M28" s="8" t="n">
-        <v>0.0036</v>
+        <v>0</v>
       </c>
       <c r="N28" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0436</v>
       </c>
       <c r="O28" s="6" t="n">
-        <v>14.88</v>
+        <v>12.9</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>35.5</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
@@ -3093,32 +3093,32 @@
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>14.64</v>
+        <v>70.64</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>14.51</v>
+        <v>69</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J29" s="7" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K29" s="10" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J29" s="9" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K29" s="11" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -3129,42 +3129,42 @@
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0178</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0331</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>24.18</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>20.2</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C30" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -3173,59 +3173,59 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>32.56</v>
+        <v>182.46</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>30.73</v>
+        <v>198.78</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J30" s="7" t="n">
-        <v>-0.0563</v>
+        <v>0.08939999999999999</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.106</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0036</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>15.98</v>
+        <v>23.45</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>43.3</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C31" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C31" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
@@ -3235,22 +3235,22 @@
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>45.31</v>
+        <v>14.05</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>43.14</v>
+        <v>13.25</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J31" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K31" s="10" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="J31" s="9" t="n">
+        <v>-0.0567</v>
+      </c>
+      <c r="K31" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -3261,88 +3261,88 @@
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.079</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>13.05</v>
+        <v>14.88</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>28.7</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C32" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J32" s="7" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K32" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>7</v>
+      </c>
+      <c r="J32" s="9" t="n">
+        <v>-0.0089</v>
+      </c>
+      <c r="K32" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L32" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N32" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>12.93</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
@@ -3379,10 +3379,10 @@
       <c r="I33" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J33" s="7" t="n">
+      <c r="J33" s="9" t="n">
         <v>-0.0563</v>
       </c>
-      <c r="K33" s="10" t="inlineStr">
+      <c r="K33" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -3399,7 +3399,7 @@
         <v>-0.0608</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>12.53</v>
+        <v>15.98</v>
       </c>
       <c r="P33" s="6" t="n">
         <v>43.3</v>
@@ -3408,22 +3408,22 @@
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -3437,64 +3437,64 @@
         </is>
       </c>
       <c r="G34" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>0.016</v>
+        <v>-0.0478</v>
       </c>
       <c r="K34" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L34" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M34" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>32.16</v>
+        <v>13.05</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C35" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
@@ -3503,64 +3503,64 @@
         </is>
       </c>
       <c r="G35" s="5" t="n">
-        <v>137.37</v>
+        <v>45.31</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>143</v>
+        <v>43.14</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J35" s="9" t="n">
-        <v>0.04099999999999999</v>
+        <v>-0.0478</v>
       </c>
       <c r="K35" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M35" s="8" t="n">
-        <v>0.0432</v>
+        <v>0</v>
       </c>
       <c r="N35" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0925</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>30.86</v>
+        <v>12.93</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>22.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D36" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F36" s="3" t="inlineStr">
@@ -3569,44 +3569,44 @@
         </is>
       </c>
       <c r="G36" s="5" t="n">
-        <v>27.31</v>
+        <v>32.56</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>27.86</v>
+        <v>30.73</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J36" s="9" t="n">
-        <v>0.0201</v>
+        <v>-0.0563</v>
       </c>
       <c r="K36" s="11" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L36" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M36" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N36" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0608</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>26.27</v>
+        <v>12.53</v>
       </c>
       <c r="P36" s="6" t="n">
-        <v>23.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
@@ -3621,12 +3621,12 @@
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F37" s="3" t="inlineStr">
@@ -3635,18 +3635,18 @@
         </is>
       </c>
       <c r="G37" s="5" t="n">
-        <v>37.25</v>
+        <v>43.19</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>38.14</v>
+        <v>43.88</v>
       </c>
       <c r="I37" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J37" s="9" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K37" s="11" t="inlineStr">
+      <c r="J37" s="7" t="n">
+        <v>0.016</v>
+      </c>
+      <c r="K37" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3657,22 +3657,22 @@
         </is>
       </c>
       <c r="M37" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0188</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0016</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>23.8</v>
+        <v>32.16</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>27.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
@@ -3687,12 +3687,12 @@
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -3701,20 +3701,20 @@
         </is>
       </c>
       <c r="G38" s="5" t="n">
-        <v>105.01</v>
+        <v>137.37</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I38" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J38" s="7" t="n">
-        <v>-0.0001</v>
+        <v>0.04099999999999999</v>
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
@@ -3723,22 +3723,22 @@
         </is>
       </c>
       <c r="M38" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0432</v>
       </c>
       <c r="N38" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.002</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>10.01</v>
+        <v>30.86</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>17.6</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
@@ -3748,39 +3748,39 @@
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>26.25</v>
+        <v>27.31</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>25.64</v>
+        <v>27.86</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J39" s="7" t="n">
-        <v>-0.0232</v>
+        <v>0.0201</v>
       </c>
       <c r="K39" s="10" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
@@ -3789,22 +3789,22 @@
         </is>
       </c>
       <c r="M39" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0392</v>
       </c>
       <c r="N39" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0114</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>16.26</v>
+        <v>26.27</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -3814,37 +3814,37 @@
       </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G40" s="5" t="n">
-        <v>10.7</v>
+        <v>37.25</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>10.73</v>
+        <v>38.14</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J40" s="9" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K40" s="11" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="J40" s="7" t="n">
+        <v>0.0239</v>
+      </c>
+      <c r="K40" s="10" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3855,22 +3855,22 @@
         </is>
       </c>
       <c r="M40" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0379</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>14.8</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3880,122 +3880,320 @@
       </c>
       <c r="C41" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G41" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>11.24</v>
+        <v>105</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J41" s="7" t="n">
-        <v>-0.0568</v>
-      </c>
-      <c r="K41" s="10" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>5</v>
+      </c>
+      <c r="J41" s="9" t="n">
+        <v>-0.0001</v>
+      </c>
+      <c r="K41" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M41" s="8" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.022</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>33.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E42" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G42" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H42" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J42" s="9" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L42" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M42" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N42" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O42" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P42" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C43" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E43" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G43" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H43" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J43" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K43" s="10" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L43" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M43" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N43" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O43" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P43" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E44" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G44" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H44" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J44" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K44" s="11" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L44" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M44" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N44" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O44" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P44" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
+      <c r="B45" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C45" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D45" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E42" s="4" t="inlineStr">
+      <c r="E45" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
+      <c r="F45" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G42" s="5" t="n">
+      <c r="G45" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H42" s="5" t="n">
+      <c r="H45" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I42" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J42" s="7" t="n">
+      <c r="I45" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J45" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K42" s="10" t="inlineStr">
+      <c r="K45" s="11" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L42" s="4" t="inlineStr">
+      <c r="L45" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M42" s="8" t="n">
+      <c r="M45" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N42" s="8" t="n">
+      <c r="N45" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O42" s="6" t="n">
+      <c r="O45" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P42" s="6" t="n">
+      <c r="P45" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -4030,7 +4228,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-05-22T02:02:50</t>
+          <t>محسوب في: 2026-06-01T11:52:44</t>
         </is>
       </c>
     </row>
@@ -4054,7 +4252,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>39</v>
+        <v>42</v>
       </c>
     </row>
     <row r="6">
@@ -4074,7 +4272,7 @@
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8">
@@ -4095,7 +4293,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>28.2%</t>
+          <t>33.3%</t>
         </is>
       </c>
     </row>
@@ -4107,7 +4305,7 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>+3.76%</t>
+          <t>+4.93%</t>
         </is>
       </c>
     </row>
@@ -4130,7 +4328,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.41</v>
+        <v>0.68</v>
       </c>
     </row>
     <row r="13">
@@ -4141,7 +4339,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-59.86%</t>
+          <t>-32.12%</t>
         </is>
       </c>
     </row>
@@ -4156,12 +4354,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2082 (2026-05-12)</t>
+          <t>4280 (2026-06-01)</t>
         </is>
       </c>
       <c r="B16" s="20" t="inlineStr">
         <is>
-          <t>+8.94%</t>
+          <t>+11.53%</t>
         </is>
       </c>
     </row>
@@ -4252,19 +4450,19 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C26" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D26" s="17" t="inlineStr">
         <is>
-          <t>20.0%</t>
-        </is>
-      </c>
-      <c r="E26" s="17" t="inlineStr">
-        <is>
-          <t>-1.95%</t>
+          <t>33.3%</t>
+        </is>
+      </c>
+      <c r="E26" s="16" t="inlineStr">
+        <is>
+          <t>+0.01%</t>
         </is>
       </c>
     </row>
@@ -4275,19 +4473,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C27" s="3" t="n">
-        <v>9</v>
-      </c>
-      <c r="D27" s="17" t="inlineStr">
-        <is>
-          <t>36.0%</t>
+        <v>11</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>40.7%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-1.07%</t>
+          <t>-0.32%</t>
         </is>
       </c>
     </row>
@@ -4404,19 +4602,19 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C36" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="C36" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="D36" s="3" t="inlineStr">
-        <is>
-          <t>50.0%</t>
+      <c r="D36" s="16" t="inlineStr">
+        <is>
+          <t>66.7%</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>+1.89%</t>
+          <t>+4.54%</t>
         </is>
       </c>
     </row>
@@ -4450,19 +4648,19 @@
         </is>
       </c>
       <c r="B38" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="C38" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D38" s="17" t="inlineStr">
         <is>
-          <t>20.0%</t>
+          <t>33.3%</t>
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr">
         <is>
-          <t>-3.68%</t>
+          <t>-2.01%</t>
         </is>
       </c>
     </row>
@@ -4634,19 +4832,19 @@
         </is>
       </c>
       <c r="B46" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C46" s="3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D46" s="17" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>1</v>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr">
         <is>
-          <t>-5.55%</t>
+          <t>+2.99%</t>
         </is>
       </c>
     </row>
@@ -4805,10 +5003,10 @@
         </is>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E5" s="3" t="n">
         <v>0</v>
@@ -4820,12 +5018,12 @@
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
-          <t>+1.60%</t>
+          <t>+3.99%</t>
         </is>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
-          <t>+1.60%</t>
+          <t>+6.37%</t>
         </is>
       </c>
       <c r="I5" s="3" t="inlineStr">
@@ -5010,10 +5208,10 @@
         </is>
       </c>
       <c r="C10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" s="3" t="n">
         <v>0</v>
@@ -5025,12 +5223,12 @@
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>+6.09%</t>
+          <t>+7.96%</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
         <is>
-          <t>+6.09%</t>
+          <t>+9.84%</t>
         </is>
       </c>
       <c r="I10" s="3" t="inlineStr">
@@ -5165,94 +5363,94 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="B14" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="C14" s="3" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D14" s="3" t="n">
         <v>1</v>
       </c>
       <c r="E14" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F14" s="17" t="inlineStr">
-        <is>
-          <t>25.0%</t>
+        <v>1</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>-2.58%</t>
+          <t>+2.99%</t>
         </is>
       </c>
       <c r="H14" s="3" t="inlineStr">
         <is>
-          <t>+3.53%</t>
+          <t>+11.53%</t>
         </is>
       </c>
       <c r="I14" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.55%</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D15" s="3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E15" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="F15" s="3" t="inlineStr">
-        <is>
-          <t>0.0%</t>
+        <v>3</v>
+      </c>
+      <c r="F15" s="17" t="inlineStr">
+        <is>
+          <t>25.0%</t>
         </is>
       </c>
       <c r="G15" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-2.58%</t>
         </is>
       </c>
       <c r="H15" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>+3.53%</t>
         </is>
       </c>
       <c r="I15" s="3" t="inlineStr">
         <is>
-          <t>-5.68%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>4040</t>
         </is>
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>نقل</t>
         </is>
       </c>
       <c r="C16" s="3" t="n">
@@ -5271,29 +5469,29 @@
       </c>
       <c r="G16" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="H16" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
       <c r="I16" s="3" t="inlineStr">
         <is>
-          <t>-4.31%</t>
+          <t>-5.68%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C17" s="3" t="n">
@@ -5312,29 +5510,29 @@
       </c>
       <c r="G17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="H17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
       <c r="I17" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-4.31%</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>4145</t>
         </is>
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
@@ -5353,29 +5551,29 @@
       </c>
       <c r="G18" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H18" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>-0.01%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="C19" s="3" t="n">
@@ -5394,29 +5592,29 @@
       </c>
       <c r="G19" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="H19" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
       <c r="I19" s="3" t="inlineStr">
         <is>
-          <t>-2.32%</t>
+          <t>-0.01%</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
@@ -5435,29 +5633,29 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="H20" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
       <c r="I20" s="3" t="inlineStr">
         <is>
-          <t>-5.67%</t>
+          <t>-2.32%</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C21" s="3" t="n">
@@ -5476,111 +5674,111 @@
       </c>
       <c r="G21" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="H21" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
       <c r="I21" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-5.67%</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D22" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E22" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="17" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="H22" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
       <c r="I22" s="3" t="inlineStr">
         <is>
-          <t>-4.78%</t>
+          <t>-0.89%</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="C23" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D23" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E23" s="3" t="n">
-        <v>2</v>
-      </c>
-      <c r="F23" s="3" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="F23" s="17" t="inlineStr">
         <is>
           <t>0.0%</t>
         </is>
       </c>
       <c r="G23" s="3" t="inlineStr">
         <is>
-          <t>-3.53%</t>
+          <t>-4.78%</t>
         </is>
       </c>
       <c r="H23" s="3" t="inlineStr">
         <is>
-          <t>-2.60%</t>
+          <t>-4.78%</t>
         </is>
       </c>
       <c r="I23" s="3" t="inlineStr">
         <is>
-          <t>-4.46%</t>
+          <t>-4.78%</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
@@ -5599,39 +5797,39 @@
       </c>
       <c r="G24" s="3" t="inlineStr">
         <is>
-          <t>-1.70%</t>
+          <t>-3.53%</t>
         </is>
       </c>
       <c r="H24" s="3" t="inlineStr">
         <is>
-          <t>-0.83%</t>
+          <t>-2.60%</t>
         </is>
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>-2.56%</t>
+          <t>-4.46%</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="B25" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="3" t="n">
         <v>0</v>
       </c>
       <c r="E25" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F25" s="3" t="inlineStr">
         <is>
@@ -5640,29 +5838,29 @@
       </c>
       <c r="G25" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-1.70%</t>
         </is>
       </c>
       <c r="H25" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-0.83%</t>
         </is>
       </c>
       <c r="I25" s="3" t="inlineStr">
         <is>
-          <t>-2.44%</t>
+          <t>-2.56%</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="B26" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
@@ -5681,29 +5879,29 @@
       </c>
       <c r="G26" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
       <c r="H26" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
       <c r="I26" s="3" t="inlineStr">
         <is>
-          <t>-2.07%</t>
+          <t>-2.44%</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="C27" s="3" t="n">
@@ -5722,29 +5920,29 @@
       </c>
       <c r="G27" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
       <c r="H27" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
       <c r="I27" s="3" t="inlineStr">
         <is>
-          <t>-3.29%</t>
+          <t>-2.07%</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="B28" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="C28" s="3" t="n">
@@ -5763,29 +5961,29 @@
       </c>
       <c r="G28" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="H28" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>-5.66%</t>
+          <t>-3.29%</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="B29" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C29" s="3" t="n">
@@ -5804,29 +6002,29 @@
       </c>
       <c r="G29" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
       <c r="H29" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
       <c r="I29" s="3" t="inlineStr">
         <is>
-          <t>-5.63%</t>
+          <t>-5.66%</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="B30" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="C30" s="3" t="n">
@@ -5845,29 +6043,29 @@
       </c>
       <c r="G30" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
       <c r="H30" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
       <c r="I30" s="3" t="inlineStr">
         <is>
-          <t>-5.65%</t>
+          <t>-5.63%</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="B31" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="C31" s="3" t="n">
@@ -5886,17 +6084,17 @@
       </c>
       <c r="G31" s="3" t="inlineStr">
         <is>
-          <t>-5.55%</t>
+          <t>-5.65%</t>
         </is>
       </c>
       <c r="H31" s="3" t="inlineStr">
         <is>
-          <t>-5.55%</t>
+          <t>-5.65%</t>
         </is>
       </c>
       <c r="I31" s="3" t="inlineStr">
         <is>
-          <t>-5.55%</t>
+          <t>-5.65%</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
📊 V9.2.1 daily run 2026-06-02_02:02
</commit_message>
<xml_diff>
--- a/paper_trades/latest.xlsx
+++ b/paper_trades/latest.xlsx
@@ -146,10 +146,10 @@
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -692,13 +692,13 @@
         </is>
       </c>
       <c r="L4" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M4" s="5" t="n">
-        <v>16.13</v>
+        <v>16.1</v>
       </c>
       <c r="N4" s="7" t="n">
-        <v>2.67</v>
+        <v>2.48</v>
       </c>
       <c r="O4" s="8" t="n">
         <v>2.8</v>
@@ -759,13 +759,13 @@
         </is>
       </c>
       <c r="L5" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M5" s="5" t="n">
-        <v>226.2</v>
-      </c>
-      <c r="N5" s="7" t="n">
-        <v>0.82</v>
+        <v>224.3</v>
+      </c>
+      <c r="N5" s="9" t="n">
+        <v>-0.02</v>
       </c>
       <c r="O5" s="8" t="n">
         <v>1.58</v>
@@ -826,13 +826,13 @@
         </is>
       </c>
       <c r="L6" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M6" s="5" t="n">
-        <v>197.5</v>
+        <v>199</v>
       </c>
       <c r="N6" s="7" t="n">
-        <v>0.57</v>
+        <v>1.33</v>
       </c>
       <c r="O6" s="8" t="n">
         <v>4.64</v>
@@ -893,13 +893,13 @@
         </is>
       </c>
       <c r="L7" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="M7" s="5" t="n">
-        <v>89.59999999999999</v>
+        <v>89.7</v>
       </c>
       <c r="N7" s="7" t="n">
-        <v>2.38</v>
+        <v>2.49</v>
       </c>
       <c r="O7" s="8" t="n">
         <v>3.52</v>
@@ -960,13 +960,13 @@
         </is>
       </c>
       <c r="L8" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M8" s="5" t="n">
-        <v>170</v>
+        <v>169.8</v>
       </c>
       <c r="N8" s="9" t="n">
-        <v>-0.61</v>
+        <v>-0.72</v>
       </c>
       <c r="O8" s="8" t="n">
         <v>0.44</v>
@@ -1027,13 +1027,13 @@
         </is>
       </c>
       <c r="L9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M9" s="5" t="n">
-        <v>149.9</v>
+        <v>150.6</v>
       </c>
       <c r="N9" s="9" t="n">
-        <v>-0.93</v>
+        <v>-0.46</v>
       </c>
       <c r="O9" s="8" t="n">
         <v>3.04</v>
@@ -1094,13 +1094,13 @@
         </is>
       </c>
       <c r="L10" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M10" s="5" t="n">
-        <v>12.19</v>
+        <v>12.22</v>
       </c>
       <c r="N10" s="7" t="n">
-        <v>3.31</v>
+        <v>3.56</v>
       </c>
       <c r="O10" s="8" t="n">
         <v>5.85</v>
@@ -1117,12 +1117,12 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0050</t>
+          <t>T0053</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
@@ -1141,19 +1141,19 @@
         </is>
       </c>
       <c r="F11" s="5" t="n">
-        <v>10.83</v>
+        <v>10.72</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>10.54</v>
+        <v>10.44</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>11.12</v>
+        <v>11.01</v>
       </c>
       <c r="I11" s="5" t="n">
-        <v>11.41</v>
+        <v>11.29</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>12.05</v>
+        <v>10.14</v>
       </c>
       <c r="K11" s="3" t="inlineStr">
         <is>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="M11" s="5" t="n">
-        <v>10.83</v>
+        <v>10.72</v>
       </c>
       <c r="N11" s="8" t="n">
         <v>0</v>
@@ -1184,12 +1184,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0051</t>
+          <t>T0054</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1220,7 +1220,7 @@
         <v>11.97</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>10.67</v>
+        <v>8.57</v>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
@@ -1251,12 +1251,12 @@
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0052</t>
+          <t>T0055</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="C13" s="3" t="inlineStr">
@@ -1275,19 +1275,19 @@
         </is>
       </c>
       <c r="F13" s="5" t="n">
-        <v>16.6</v>
+        <v>16.84</v>
       </c>
       <c r="G13" s="5" t="n">
-        <v>16.06</v>
+        <v>16.3</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>17.14</v>
+        <v>17.38</v>
       </c>
       <c r="I13" s="5" t="n">
-        <v>17.68</v>
+        <v>17.92</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>10.43</v>
+        <v>8.42</v>
       </c>
       <c r="K13" s="3" t="inlineStr">
         <is>
@@ -1298,7 +1298,7 @@
         <v>0</v>
       </c>
       <c r="M13" s="5" t="n">
-        <v>16.6</v>
+        <v>16.84</v>
       </c>
       <c r="N13" s="8" t="n">
         <v>0</v>
@@ -1329,7 +1329,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P45"/>
+  <dimension ref="A1:P48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -1428,93 +1428,93 @@
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>T0040</t>
+          <t>T0050</t>
         </is>
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2340</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G4" s="5" t="n">
-        <v>12.66</v>
+        <v>10.83</v>
       </c>
       <c r="H4" s="5" t="n">
-        <v>13.91</v>
+        <v>10.49</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J4" s="7" t="n">
-        <v>0.0984</v>
+        <v>1</v>
+      </c>
+      <c r="J4" s="9" t="n">
+        <v>-0.0316</v>
       </c>
       <c r="K4" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L4" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M4" s="8" t="n">
-        <v>0.2062</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="N4" s="8" t="n">
-        <v>-0.0276</v>
+        <v>-0.0434</v>
       </c>
       <c r="O4" s="6" t="n">
-        <v>10.24</v>
+        <v>12.05</v>
       </c>
       <c r="P4" s="6" t="n">
-        <v>39.1</v>
+        <v>17.9</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>T0041</t>
+          <t>T0051</t>
         </is>
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>4061</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
@@ -1523,64 +1523,64 @@
         </is>
       </c>
       <c r="G5" s="5" t="n">
-        <v>45.37</v>
+        <v>11.31</v>
       </c>
       <c r="H5" s="5" t="n">
-        <v>48.26</v>
+        <v>10.93</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J5" s="7" t="n">
-        <v>0.06370000000000001</v>
+        <v>1</v>
+      </c>
+      <c r="J5" s="9" t="n">
+        <v>-0.034</v>
       </c>
       <c r="K5" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L5" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M5" s="8" t="n">
-        <v>0.102</v>
+        <v>0</v>
       </c>
       <c r="N5" s="8" t="n">
-        <v>-0.0302</v>
+        <v>-0.08839999999999999</v>
       </c>
       <c r="O5" s="6" t="n">
-        <v>15.11</v>
+        <v>10.67</v>
       </c>
       <c r="P5" s="6" t="n">
-        <v>26.9</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>T0046</t>
+          <t>T0052</t>
         </is>
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>4170</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F6" s="3" t="inlineStr">
@@ -1589,196 +1589,196 @@
         </is>
       </c>
       <c r="G6" s="5" t="n">
-        <v>12.37</v>
+        <v>16.6</v>
       </c>
       <c r="H6" s="5" t="n">
-        <v>13.8</v>
+        <v>15.98</v>
       </c>
       <c r="I6" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="J6" s="7" t="n">
-        <v>0.1153</v>
+      <c r="J6" s="9" t="n">
+        <v>-0.0374</v>
       </c>
       <c r="K6" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L6" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M6" s="8" t="n">
-        <v>0.207</v>
+        <v>0.0392</v>
       </c>
       <c r="N6" s="8" t="n">
-        <v>0</v>
+        <v>-0.044</v>
       </c>
       <c r="O6" s="6" t="n">
-        <v>13.56</v>
+        <v>10.43</v>
       </c>
       <c r="P6" s="6" t="n">
-        <v>28</v>
+        <v>25.1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>T0030</t>
+          <t>T0040</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
         <is>
-          <t>2223</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E7" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G7" s="5" t="n">
-        <v>128.16</v>
+        <v>12.66</v>
       </c>
       <c r="H7" s="5" t="n">
-        <v>127.3</v>
+        <v>13.91</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>-0.0067</v>
+        <v>4</v>
+      </c>
+      <c r="J7" s="7" t="n">
+        <v>0.0984</v>
       </c>
       <c r="K7" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L7" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M7" s="8" t="n">
-        <v>0.0206</v>
+        <v>0.2062</v>
       </c>
       <c r="N7" s="8" t="n">
-        <v>-0.0169</v>
+        <v>-0.0276</v>
       </c>
       <c r="O7" s="6" t="n">
-        <v>5.12</v>
+        <v>10.24</v>
       </c>
       <c r="P7" s="6" t="n">
-        <v>35.2</v>
+        <v>39.1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
         <is>
-          <t>T0031</t>
+          <t>T0041</t>
         </is>
       </c>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G8" s="5" t="n">
-        <v>14.64</v>
+        <v>45.37</v>
       </c>
       <c r="H8" s="5" t="n">
-        <v>14.3</v>
+        <v>48.26</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>7</v>
-      </c>
-      <c r="J8" s="9" t="n">
-        <v>-0.0232</v>
+        <v>3</v>
+      </c>
+      <c r="J8" s="7" t="n">
+        <v>0.06370000000000001</v>
       </c>
       <c r="K8" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L8" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M8" s="8" t="n">
-        <v>0.005500000000000001</v>
+        <v>0.102</v>
       </c>
       <c r="N8" s="8" t="n">
-        <v>-0.043</v>
+        <v>-0.0302</v>
       </c>
       <c r="O8" s="6" t="n">
-        <v>3.78</v>
+        <v>15.11</v>
       </c>
       <c r="P8" s="6" t="n">
-        <v>15.7</v>
+        <v>26.9</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>T0036</t>
+          <t>T0046</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="C9" s="3" t="inlineStr">
         <is>
-          <t>2026-05-22</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>8180</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F9" s="3" t="inlineStr">
@@ -1787,49 +1787,49 @@
         </is>
       </c>
       <c r="G9" s="5" t="n">
-        <v>11.35</v>
+        <v>12.37</v>
       </c>
       <c r="H9" s="5" t="n">
-        <v>10.97</v>
+        <v>13.8</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J9" s="9" t="n">
-        <v>-0.0335</v>
+        <v>1</v>
+      </c>
+      <c r="J9" s="7" t="n">
+        <v>0.1153</v>
       </c>
       <c r="K9" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L9" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M9" s="8" t="n">
-        <v>0.03</v>
+        <v>0.207</v>
       </c>
       <c r="N9" s="8" t="n">
-        <v>-0.04849999999999999</v>
+        <v>0</v>
       </c>
       <c r="O9" s="6" t="n">
-        <v>16.05</v>
+        <v>13.56</v>
       </c>
       <c r="P9" s="6" t="n">
-        <v>36.6</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>T0039</t>
+          <t>T0030</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -1839,7 +1839,7 @@
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2223</t>
         </is>
       </c>
       <c r="E10" s="4" t="inlineStr">
@@ -1849,22 +1849,22 @@
       </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G10" s="5" t="n">
-        <v>32.97</v>
+        <v>128.16</v>
       </c>
       <c r="H10" s="5" t="n">
-        <v>32.12</v>
+        <v>127.3</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J10" s="9" t="n">
-        <v>-0.0258</v>
-      </c>
-      <c r="K10" s="11" t="inlineStr">
+        <v>-0.0067</v>
+      </c>
+      <c r="K10" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -1875,37 +1875,37 @@
         </is>
       </c>
       <c r="M10" s="8" t="n">
-        <v>0.01</v>
+        <v>0.0206</v>
       </c>
       <c r="N10" s="8" t="n">
-        <v>-0.0288</v>
+        <v>-0.0169</v>
       </c>
       <c r="O10" s="6" t="n">
-        <v>7.94</v>
+        <v>5.12</v>
       </c>
       <c r="P10" s="6" t="n">
-        <v>45.4</v>
+        <v>35.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>T0028</t>
+          <t>T0031</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C11" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>2380</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="E11" s="4" t="inlineStr">
@@ -1919,20 +1919,20 @@
         </is>
       </c>
       <c r="G11" s="5" t="n">
-        <v>15.33</v>
+        <v>14.64</v>
       </c>
       <c r="H11" s="5" t="n">
-        <v>16.18</v>
+        <v>14.3</v>
       </c>
       <c r="I11" s="3" t="n">
         <v>7</v>
       </c>
-      <c r="J11" s="7" t="n">
-        <v>0.0554</v>
+      <c r="J11" s="9" t="n">
+        <v>-0.0232</v>
       </c>
       <c r="K11" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L11" s="4" t="inlineStr">
@@ -1941,37 +1941,37 @@
         </is>
       </c>
       <c r="M11" s="8" t="n">
-        <v>0.0698</v>
+        <v>0.005500000000000001</v>
       </c>
       <c r="N11" s="8" t="n">
-        <v>-0.0033</v>
+        <v>-0.043</v>
       </c>
       <c r="O11" s="6" t="n">
-        <v>9.57</v>
+        <v>3.78</v>
       </c>
       <c r="P11" s="6" t="n">
-        <v>47.4</v>
+        <v>15.7</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>T0033</t>
+          <t>T0036</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>8180</t>
         </is>
       </c>
       <c r="E12" s="4" t="inlineStr">
@@ -1985,18 +1985,18 @@
         </is>
       </c>
       <c r="G12" s="5" t="n">
-        <v>14.6</v>
+        <v>11.35</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>14.22</v>
+        <v>10.97</v>
       </c>
       <c r="I12" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J12" s="9" t="n">
-        <v>-0.026</v>
-      </c>
-      <c r="K12" s="11" t="inlineStr">
+        <v>-0.0335</v>
+      </c>
+      <c r="K12" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2007,22 +2007,22 @@
         </is>
       </c>
       <c r="M12" s="8" t="n">
-        <v>0.0445</v>
+        <v>0.03</v>
       </c>
       <c r="N12" s="8" t="n">
-        <v>-0.0322</v>
+        <v>-0.04849999999999999</v>
       </c>
       <c r="O12" s="6" t="n">
-        <v>3.63</v>
+        <v>16.05</v>
       </c>
       <c r="P12" s="6" t="n">
-        <v>16.8</v>
+        <v>36.6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>T0037</t>
+          <t>T0039</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
@@ -2032,78 +2032,78 @@
       </c>
       <c r="C13" s="3" t="inlineStr">
         <is>
-          <t>2026-05-21</t>
+          <t>2026-05-22</t>
         </is>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>7202</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E13" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G13" s="5" t="n">
-        <v>230.06</v>
+        <v>32.97</v>
       </c>
       <c r="H13" s="5" t="n">
-        <v>219.22</v>
+        <v>32.12</v>
       </c>
       <c r="I13" s="3" t="n">
         <v>4</v>
       </c>
       <c r="J13" s="9" t="n">
-        <v>-0.0471</v>
-      </c>
-      <c r="K13" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0258</v>
+      </c>
+      <c r="K13" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L13" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M13" s="8" t="n">
-        <v>0.005</v>
+        <v>0.01</v>
       </c>
       <c r="N13" s="8" t="n">
-        <v>-0.0559</v>
+        <v>-0.0288</v>
       </c>
       <c r="O13" s="6" t="n">
-        <v>12.77</v>
+        <v>7.94</v>
       </c>
       <c r="P13" s="6" t="n">
-        <v>31.9</v>
+        <v>45.4</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>T0034</t>
+          <t>T0028</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>2380</t>
         </is>
       </c>
       <c r="E14" s="4" t="inlineStr">
@@ -2113,24 +2113,24 @@
       </c>
       <c r="F14" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G14" s="5" t="n">
-        <v>28.94</v>
+        <v>15.33</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>28.7</v>
+        <v>16.18</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J14" s="9" t="n">
-        <v>-0.0083</v>
+        <v>7</v>
+      </c>
+      <c r="J14" s="7" t="n">
+        <v>0.0554</v>
       </c>
       <c r="K14" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L14" s="4" t="inlineStr">
@@ -2139,108 +2139,108 @@
         </is>
       </c>
       <c r="M14" s="8" t="n">
-        <v>0.0048</v>
+        <v>0.0698</v>
       </c>
       <c r="N14" s="8" t="n">
-        <v>-0.0256</v>
+        <v>-0.0033</v>
       </c>
       <c r="O14" s="6" t="n">
-        <v>3</v>
+        <v>9.57</v>
       </c>
       <c r="P14" s="6" t="n">
-        <v>28.4</v>
+        <v>47.4</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>T0038</t>
+          <t>T0033</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
         <is>
-          <t>2026-05-20</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>4280</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E15" s="4" t="inlineStr">
         <is>
-          <t>عقار</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G15" s="5" t="n">
-        <v>11.03</v>
+        <v>14.6</v>
       </c>
       <c r="H15" s="5" t="n">
-        <v>10.42</v>
+        <v>14.22</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="J15" s="9" t="n">
-        <v>-0.0555</v>
-      </c>
-      <c r="K15" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.026</v>
+      </c>
+      <c r="K15" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L15" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M15" s="8" t="n">
-        <v>0.0063</v>
+        <v>0.0445</v>
       </c>
       <c r="N15" s="8" t="n">
-        <v>-0.07980000000000001</v>
+        <v>-0.0322</v>
       </c>
       <c r="O15" s="6" t="n">
-        <v>10.8</v>
+        <v>3.63</v>
       </c>
       <c r="P15" s="6" t="n">
-        <v>32.4</v>
+        <v>16.8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>T0032</t>
+          <t>T0037</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>2026-05-19</t>
+          <t>2026-05-21</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>2110</t>
+          <t>7202</t>
         </is>
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F16" s="3" t="inlineStr">
@@ -2249,18 +2249,18 @@
         </is>
       </c>
       <c r="G16" s="5" t="n">
-        <v>158.92</v>
+        <v>230.06</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>149.94</v>
+        <v>219.22</v>
       </c>
       <c r="I16" s="3" t="n">
         <v>4</v>
       </c>
       <c r="J16" s="9" t="n">
-        <v>-0.0565</v>
-      </c>
-      <c r="K16" s="11" t="inlineStr">
+        <v>-0.0471</v>
+      </c>
+      <c r="K16" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2271,62 +2271,62 @@
         </is>
       </c>
       <c r="M16" s="8" t="n">
-        <v>0</v>
+        <v>0.005</v>
       </c>
       <c r="N16" s="8" t="n">
-        <v>-0.0624</v>
+        <v>-0.0559</v>
       </c>
       <c r="O16" s="6" t="n">
-        <v>3.46</v>
+        <v>12.77</v>
       </c>
       <c r="P16" s="6" t="n">
-        <v>14.4</v>
+        <v>31.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>T0025</t>
+          <t>T0034</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="C17" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>7040</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E17" s="4" t="inlineStr">
         <is>
-          <t>اتصالات</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F17" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>support_bounce</t>
         </is>
       </c>
       <c r="G17" s="5" t="n">
-        <v>100.3</v>
+        <v>28.94</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>97</v>
+        <v>28.7</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J17" s="9" t="n">
-        <v>-0.0329</v>
-      </c>
-      <c r="K17" s="11" t="inlineStr">
+        <v>-0.0083</v>
+      </c>
+      <c r="K17" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2337,62 +2337,62 @@
         </is>
       </c>
       <c r="M17" s="8" t="n">
-        <v>0.006</v>
+        <v>0.0048</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>-0.04190000000000001</v>
+        <v>-0.0256</v>
       </c>
       <c r="O17" s="6" t="n">
-        <v>9.9</v>
+        <v>3</v>
       </c>
       <c r="P17" s="6" t="n">
-        <v>25.2</v>
+        <v>28.4</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>T0029</t>
+          <t>T0038</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-20</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>1321</t>
+          <t>4280</t>
         </is>
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>عقار</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G18" s="5" t="n">
-        <v>195.39</v>
+        <v>11.03</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>184.32</v>
+        <v>10.42</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>-0.0566</v>
-      </c>
-      <c r="K18" s="11" t="inlineStr">
+        <v>-0.0555</v>
+      </c>
+      <c r="K18" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2403,37 +2403,37 @@
         </is>
       </c>
       <c r="M18" s="8" t="n">
-        <v>0.05429999999999999</v>
+        <v>0.0063</v>
       </c>
       <c r="N18" s="8" t="n">
-        <v>-0.0634</v>
+        <v>-0.07980000000000001</v>
       </c>
       <c r="O18" s="6" t="n">
-        <v>8.51</v>
+        <v>10.8</v>
       </c>
       <c r="P18" s="6" t="n">
-        <v>43.7</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>T0027</t>
+          <t>T0032</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="C19" s="3" t="inlineStr">
         <is>
-          <t>2026-05-18</t>
+          <t>2026-05-19</t>
         </is>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2110</t>
         </is>
       </c>
       <c r="E19" s="4" t="inlineStr">
@@ -2447,64 +2447,64 @@
         </is>
       </c>
       <c r="G19" s="5" t="n">
-        <v>32.56</v>
+        <v>158.92</v>
       </c>
       <c r="H19" s="5" t="n">
-        <v>32.9</v>
+        <v>149.94</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J19" s="7" t="n">
-        <v>0.0353</v>
+        <v>4</v>
+      </c>
+      <c r="J19" s="9" t="n">
+        <v>-0.0565</v>
       </c>
       <c r="K19" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L19" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M19" s="8" t="n">
-        <v>0.0663</v>
+        <v>0</v>
       </c>
       <c r="N19" s="8" t="n">
-        <v>-0.0012</v>
+        <v>-0.0624</v>
       </c>
       <c r="O19" s="6" t="n">
-        <v>12.52</v>
+        <v>3.46</v>
       </c>
       <c r="P19" s="6" t="n">
-        <v>43.3</v>
+        <v>14.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>T0035</t>
+          <t>T0025</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
+          <t>2026-05-12</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
           <t>2026-05-18</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-18</t>
-        </is>
-      </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>8070</t>
+          <t>7040</t>
         </is>
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>اتصالات</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -2513,84 +2513,84 @@
         </is>
       </c>
       <c r="G20" s="5" t="n">
-        <v>11.82</v>
+        <v>100.3</v>
       </c>
       <c r="H20" s="5" t="n">
-        <v>11.15</v>
+        <v>97</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J20" s="9" t="n">
-        <v>-0.0563</v>
-      </c>
-      <c r="K20" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0329</v>
+      </c>
+      <c r="K20" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L20" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M20" s="8" t="n">
-        <v>0.008500000000000001</v>
+        <v>0.006</v>
       </c>
       <c r="N20" s="8" t="n">
-        <v>-0.0728</v>
+        <v>-0.04190000000000001</v>
       </c>
       <c r="O20" s="6" t="n">
-        <v>16.94</v>
+        <v>9.9</v>
       </c>
       <c r="P20" s="6" t="n">
-        <v>25.6</v>
+        <v>25.2</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>T0026</t>
+          <t>T0029</t>
         </is>
       </c>
       <c r="B21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="C21" s="3" t="inlineStr">
         <is>
-          <t>2026-05-15</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>1321</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F21" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G21" s="5" t="n">
-        <v>45.31</v>
+        <v>195.39</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>43.14</v>
+        <v>184.32</v>
       </c>
       <c r="I21" s="3" t="n">
         <v>3</v>
       </c>
       <c r="J21" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K21" s="11" t="inlineStr">
+        <v>-0.0566</v>
+      </c>
+      <c r="K21" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -2601,42 +2601,42 @@
         </is>
       </c>
       <c r="M21" s="8" t="n">
-        <v>0</v>
+        <v>0.05429999999999999</v>
       </c>
       <c r="N21" s="8" t="n">
-        <v>-0.0461</v>
+        <v>-0.0634</v>
       </c>
       <c r="O21" s="6" t="n">
-        <v>12.84</v>
+        <v>8.51</v>
       </c>
       <c r="P21" s="6" t="n">
-        <v>28.7</v>
+        <v>43.7</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>T0015</t>
+          <t>T0027</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>2130</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -2645,18 +2645,18 @@
         </is>
       </c>
       <c r="G22" s="5" t="n">
-        <v>12.24</v>
+        <v>32.56</v>
       </c>
       <c r="H22" s="5" t="n">
-        <v>12.9</v>
+        <v>32.9</v>
       </c>
       <c r="I22" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>0.0609</v>
-      </c>
-      <c r="K22" s="10" t="inlineStr">
+        <v>0.0353</v>
+      </c>
+      <c r="K22" s="11" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2667,42 +2667,42 @@
         </is>
       </c>
       <c r="M22" s="8" t="n">
-        <v>0.08740000000000001</v>
+        <v>0.0663</v>
       </c>
       <c r="N22" s="8" t="n">
-        <v>-0.0155</v>
+        <v>-0.0012</v>
       </c>
       <c r="O22" s="6" t="n">
-        <v>16.08</v>
+        <v>12.52</v>
       </c>
       <c r="P22" s="6" t="n">
-        <v>36.7</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>T0016</t>
+          <t>T0035</t>
         </is>
       </c>
       <c r="B23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="C23" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-18</t>
         </is>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>3080</t>
+          <t>8070</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -2711,64 +2711,64 @@
         </is>
       </c>
       <c r="G23" s="5" t="n">
-        <v>25.85</v>
+        <v>11.82</v>
       </c>
       <c r="H23" s="5" t="n">
-        <v>25.22</v>
+        <v>11.15</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="J23" s="9" t="n">
-        <v>-0.0244</v>
-      </c>
-      <c r="K23" s="11" t="inlineStr">
-        <is>
-          <t>TIME_LOSS</t>
+        <v>-0.0563</v>
+      </c>
+      <c r="K23" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L23" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M23" s="8" t="n">
-        <v>0</v>
+        <v>0.008500000000000001</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>-0.0352</v>
+        <v>-0.0728</v>
       </c>
       <c r="O23" s="6" t="n">
-        <v>14.35</v>
+        <v>16.94</v>
       </c>
       <c r="P23" s="6" t="n">
-        <v>26.1</v>
+        <v>25.6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>T0017</t>
+          <t>T0026</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>2026-05-14</t>
+          <t>2026-05-15</t>
         </is>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>1833</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>فنادق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F24" s="3" t="inlineStr">
@@ -2777,44 +2777,44 @@
         </is>
       </c>
       <c r="G24" s="5" t="n">
-        <v>90.63</v>
+        <v>45.31</v>
       </c>
       <c r="H24" s="5" t="n">
-        <v>94.40000000000001</v>
+        <v>43.14</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J24" s="7" t="n">
-        <v>0.0416</v>
+        <v>3</v>
+      </c>
+      <c r="J24" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K24" s="10" t="inlineStr">
         <is>
-          <t>WIN_PARTIAL</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L24" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M24" s="8" t="n">
-        <v>0.057</v>
+        <v>0</v>
       </c>
       <c r="N24" s="8" t="n">
-        <v>0</v>
+        <v>-0.0461</v>
       </c>
       <c r="O24" s="6" t="n">
-        <v>14.18</v>
+        <v>12.84</v>
       </c>
       <c r="P24" s="6" t="n">
-        <v>23</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>T0018</t>
+          <t>T0015</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
@@ -2829,12 +2829,12 @@
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>3060</t>
+          <t>2130</t>
         </is>
       </c>
       <c r="E25" s="4" t="inlineStr">
         <is>
-          <t>أسمنت</t>
+          <t>صناعية</t>
         </is>
       </c>
       <c r="F25" s="3" t="inlineStr">
@@ -2843,18 +2843,18 @@
         </is>
       </c>
       <c r="G25" s="5" t="n">
-        <v>15.53</v>
+        <v>12.24</v>
       </c>
       <c r="H25" s="5" t="n">
-        <v>15.88</v>
+        <v>12.9</v>
       </c>
       <c r="I25" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>0.0267</v>
-      </c>
-      <c r="K25" s="10" t="inlineStr">
+        <v>0.0609</v>
+      </c>
+      <c r="K25" s="11" t="inlineStr">
         <is>
           <t>WIN_PARTIAL</t>
         </is>
@@ -2865,22 +2865,22 @@
         </is>
       </c>
       <c r="M25" s="8" t="n">
-        <v>0.038</v>
+        <v>0.08740000000000001</v>
       </c>
       <c r="N25" s="8" t="n">
-        <v>0</v>
+        <v>-0.0155</v>
       </c>
       <c r="O25" s="6" t="n">
-        <v>11.78</v>
+        <v>16.08</v>
       </c>
       <c r="P25" s="6" t="n">
-        <v>19.9</v>
+        <v>36.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>T0019</t>
+          <t>T0016</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
@@ -2895,12 +2895,12 @@
       </c>
       <c r="D26" s="3" t="inlineStr">
         <is>
-          <t>7203</t>
+          <t>3080</t>
         </is>
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
-          <t>تقنية</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2909,18 +2909,18 @@
         </is>
       </c>
       <c r="G26" s="5" t="n">
-        <v>694.39</v>
+        <v>25.85</v>
       </c>
       <c r="H26" s="5" t="n">
-        <v>680</v>
+        <v>25.22</v>
       </c>
       <c r="I26" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J26" s="9" t="n">
-        <v>-0.0207</v>
-      </c>
-      <c r="K26" s="11" t="inlineStr">
+        <v>-0.0244</v>
+      </c>
+      <c r="K26" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -2931,42 +2931,42 @@
         </is>
       </c>
       <c r="M26" s="8" t="n">
-        <v>0.0254</v>
+        <v>0</v>
       </c>
       <c r="N26" s="8" t="n">
-        <v>-0.0517</v>
+        <v>-0.0352</v>
       </c>
       <c r="O26" s="6" t="n">
-        <v>10.02</v>
+        <v>14.35</v>
       </c>
       <c r="P26" s="6" t="n">
-        <v>23.7</v>
+        <v>26.1</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>T0014</t>
+          <t>T0017</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C27" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D27" s="3" t="inlineStr">
         <is>
-          <t>8030</t>
+          <t>1833</t>
         </is>
       </c>
       <c r="E27" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>فنادق</t>
         </is>
       </c>
       <c r="F27" s="3" t="inlineStr">
@@ -2975,20 +2975,20 @@
         </is>
       </c>
       <c r="G27" s="5" t="n">
-        <v>15.01</v>
+        <v>90.63</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>14.34</v>
+        <v>94.40000000000001</v>
       </c>
       <c r="I27" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J27" s="9" t="n">
-        <v>-0.0446</v>
+      <c r="J27" s="7" t="n">
+        <v>0.0416</v>
       </c>
       <c r="K27" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L27" s="4" t="inlineStr">
@@ -2997,64 +2997,64 @@
         </is>
       </c>
       <c r="M27" s="8" t="n">
-        <v>0.0127</v>
+        <v>0.057</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>-0.0466</v>
+        <v>0</v>
       </c>
       <c r="O27" s="6" t="n">
-        <v>11.78</v>
+        <v>14.18</v>
       </c>
       <c r="P27" s="6" t="n">
-        <v>11.8</v>
+        <v>23</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>T0022</t>
+          <t>T0018</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>2026-05-13</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D28" s="3" t="inlineStr">
         <is>
-          <t>2170</t>
+          <t>3060</t>
         </is>
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>أسمنت</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
         <is>
-          <t>mean_reversion</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G28" s="5" t="n">
-        <v>28.9</v>
+        <v>15.53</v>
       </c>
       <c r="H28" s="5" t="n">
-        <v>28.16</v>
+        <v>15.88</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>3</v>
-      </c>
-      <c r="J28" s="9" t="n">
-        <v>-0.0256</v>
+        <v>5</v>
+      </c>
+      <c r="J28" s="7" t="n">
+        <v>0.0267</v>
       </c>
       <c r="K28" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>WIN_PARTIAL</t>
         </is>
       </c>
       <c r="L28" s="4" t="inlineStr">
@@ -3063,42 +3063,42 @@
         </is>
       </c>
       <c r="M28" s="8" t="n">
+        <v>0.038</v>
+      </c>
+      <c r="N28" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N28" s="8" t="n">
-        <v>-0.0436</v>
-      </c>
       <c r="O28" s="6" t="n">
-        <v>12.9</v>
+        <v>11.78</v>
       </c>
       <c r="P28" s="6" t="n">
-        <v>32.8</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="3" t="inlineStr">
         <is>
-          <t>T0011</t>
+          <t>T0019</t>
         </is>
       </c>
       <c r="B29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="C29" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-14</t>
         </is>
       </c>
       <c r="D29" s="3" t="inlineStr">
         <is>
-          <t>2320</t>
+          <t>7203</t>
         </is>
       </c>
       <c r="E29" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>تقنية</t>
         </is>
       </c>
       <c r="F29" s="3" t="inlineStr">
@@ -3107,18 +3107,18 @@
         </is>
       </c>
       <c r="G29" s="5" t="n">
-        <v>70.64</v>
+        <v>694.39</v>
       </c>
       <c r="H29" s="5" t="n">
-        <v>69</v>
+        <v>680</v>
       </c>
       <c r="I29" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>-0.0232</v>
-      </c>
-      <c r="K29" s="11" t="inlineStr">
+        <v>-0.0207</v>
+      </c>
+      <c r="K29" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -3129,42 +3129,42 @@
         </is>
       </c>
       <c r="M29" s="8" t="n">
-        <v>0.0178</v>
+        <v>0.0254</v>
       </c>
       <c r="N29" s="8" t="n">
-        <v>-0.0331</v>
+        <v>-0.0517</v>
       </c>
       <c r="O29" s="6" t="n">
-        <v>24.18</v>
+        <v>10.02</v>
       </c>
       <c r="P29" s="6" t="n">
-        <v>13.3</v>
+        <v>23.7</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="3" t="inlineStr">
         <is>
-          <t>T0012</t>
+          <t>T0014</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-10</t>
         </is>
       </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D30" s="3" t="inlineStr">
         <is>
-          <t>2082</t>
+          <t>8030</t>
         </is>
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F30" s="3" t="inlineStr">
@@ -3173,115 +3173,115 @@
         </is>
       </c>
       <c r="G30" s="5" t="n">
-        <v>182.46</v>
+        <v>15.01</v>
       </c>
       <c r="H30" s="5" t="n">
-        <v>198.78</v>
+        <v>14.34</v>
       </c>
       <c r="I30" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J30" s="7" t="n">
-        <v>0.08939999999999999</v>
+      <c r="J30" s="9" t="n">
+        <v>-0.0446</v>
       </c>
       <c r="K30" s="10" t="inlineStr">
         <is>
-          <t>WIN_T2</t>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L30" s="4" t="inlineStr">
         <is>
-          <t>Target2 Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M30" s="8" t="n">
-        <v>0.106</v>
+        <v>0.0127</v>
       </c>
       <c r="N30" s="8" t="n">
-        <v>-0.0036</v>
+        <v>-0.0466</v>
       </c>
       <c r="O30" s="6" t="n">
-        <v>23.45</v>
+        <v>11.78</v>
       </c>
       <c r="P30" s="6" t="n">
-        <v>12.1</v>
+        <v>11.8</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="3" t="inlineStr">
         <is>
-          <t>T0013</t>
+          <t>T0022</t>
         </is>
       </c>
       <c r="B31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C31" s="3" t="inlineStr">
         <is>
-          <t>2026-05-12</t>
+          <t>2026-05-13</t>
         </is>
       </c>
       <c r="D31" s="3" t="inlineStr">
         <is>
-          <t>6017</t>
+          <t>2170</t>
         </is>
       </c>
       <c r="E31" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F31" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>mean_reversion</t>
         </is>
       </c>
       <c r="G31" s="5" t="n">
-        <v>14.05</v>
+        <v>28.9</v>
       </c>
       <c r="H31" s="5" t="n">
-        <v>13.25</v>
+        <v>28.16</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="J31" s="9" t="n">
-        <v>-0.0567</v>
-      </c>
-      <c r="K31" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0256</v>
+      </c>
+      <c r="K31" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L31" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M31" s="8" t="n">
-        <v>0.0036</v>
+        <v>0</v>
       </c>
       <c r="N31" s="8" t="n">
-        <v>-0.079</v>
+        <v>-0.0436</v>
       </c>
       <c r="O31" s="6" t="n">
-        <v>14.88</v>
+        <v>12.9</v>
       </c>
       <c r="P31" s="6" t="n">
-        <v>35.5</v>
+        <v>32.8</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="3" t="inlineStr">
         <is>
-          <t>T0010</t>
+          <t>T0011</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-08</t>
         </is>
       </c>
       <c r="C32" s="3" t="inlineStr">
@@ -3291,32 +3291,32 @@
       </c>
       <c r="D32" s="3" t="inlineStr">
         <is>
-          <t>4020</t>
+          <t>2320</t>
         </is>
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
-          <t>تجزئة</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F32" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G32" s="5" t="n">
-        <v>14.64</v>
+        <v>70.64</v>
       </c>
       <c r="H32" s="5" t="n">
-        <v>14.51</v>
+        <v>69</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="J32" s="9" t="n">
-        <v>-0.0089</v>
-      </c>
-      <c r="K32" s="11" t="inlineStr">
+        <v>-0.0232</v>
+      </c>
+      <c r="K32" s="10" t="inlineStr">
         <is>
           <t>TIME_LOSS</t>
         </is>
@@ -3327,42 +3327,42 @@
         </is>
       </c>
       <c r="M32" s="8" t="n">
-        <v>0.0089</v>
+        <v>0.0178</v>
       </c>
       <c r="N32" s="8" t="n">
-        <v>-0.0294</v>
+        <v>-0.0331</v>
       </c>
       <c r="O32" s="6" t="n">
-        <v>9.619999999999999</v>
+        <v>24.18</v>
       </c>
       <c r="P32" s="6" t="n">
-        <v>20.2</v>
+        <v>13.3</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
-          <t>T0020</t>
+          <t>T0012</t>
         </is>
       </c>
       <c r="B33" s="3" t="inlineStr">
         <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="C33" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C33" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D33" s="3" t="inlineStr">
         <is>
-          <t>2370</t>
+          <t>2082</t>
         </is>
       </c>
       <c r="E33" s="4" t="inlineStr">
         <is>
-          <t>بتروكيماويات</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F33" s="3" t="inlineStr">
@@ -3371,59 +3371,59 @@
         </is>
       </c>
       <c r="G33" s="5" t="n">
-        <v>32.56</v>
+        <v>182.46</v>
       </c>
       <c r="H33" s="5" t="n">
-        <v>30.73</v>
+        <v>198.78</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J33" s="9" t="n">
-        <v>-0.0563</v>
+        <v>5</v>
+      </c>
+      <c r="J33" s="7" t="n">
+        <v>0.08939999999999999</v>
       </c>
       <c r="K33" s="11" t="inlineStr">
         <is>
-          <t>LOSS</t>
+          <t>WIN_T2</t>
         </is>
       </c>
       <c r="L33" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Target2 Hit</t>
         </is>
       </c>
       <c r="M33" s="8" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.106</v>
       </c>
       <c r="N33" s="8" t="n">
-        <v>-0.0608</v>
+        <v>-0.0036</v>
       </c>
       <c r="O33" s="6" t="n">
-        <v>15.98</v>
+        <v>23.45</v>
       </c>
       <c r="P33" s="6" t="n">
-        <v>43.3</v>
+        <v>12.1</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="3" t="inlineStr">
         <is>
-          <t>T0021</t>
+          <t>T0013</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
         <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C34" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D34" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>6017</t>
         </is>
       </c>
       <c r="E34" s="4" t="inlineStr">
@@ -3433,22 +3433,22 @@
       </c>
       <c r="F34" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G34" s="5" t="n">
-        <v>45.31</v>
+        <v>14.05</v>
       </c>
       <c r="H34" s="5" t="n">
-        <v>43.14</v>
+        <v>13.25</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J34" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K34" s="11" t="inlineStr">
+        <v>-0.0567</v>
+      </c>
+      <c r="K34" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -3459,88 +3459,88 @@
         </is>
       </c>
       <c r="M34" s="8" t="n">
-        <v>0</v>
+        <v>0.0036</v>
       </c>
       <c r="N34" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.079</v>
       </c>
       <c r="O34" s="6" t="n">
-        <v>13.05</v>
+        <v>14.88</v>
       </c>
       <c r="P34" s="6" t="n">
-        <v>28.7</v>
+        <v>35.5</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="3" t="inlineStr">
         <is>
-          <t>T0023</t>
+          <t>T0010</t>
         </is>
       </c>
       <c r="B35" s="3" t="inlineStr">
         <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C35" s="3" t="inlineStr">
+        <is>
           <t>2026-05-12</t>
         </is>
       </c>
-      <c r="C35" s="3" t="inlineStr">
-        <is>
-          <t>2026-05-12</t>
-        </is>
-      </c>
       <c r="D35" s="3" t="inlineStr">
         <is>
-          <t>2280</t>
+          <t>4020</t>
         </is>
       </c>
       <c r="E35" s="4" t="inlineStr">
         <is>
-          <t>زراعة وأغذية</t>
+          <t>تجزئة</t>
         </is>
       </c>
       <c r="F35" s="3" t="inlineStr">
         <is>
-          <t>breakout</t>
+          <t>default</t>
         </is>
       </c>
       <c r="G35" s="5" t="n">
-        <v>45.31</v>
+        <v>14.64</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>43.14</v>
+        <v>14.51</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="J35" s="9" t="n">
-        <v>-0.0478</v>
-      </c>
-      <c r="K35" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0089</v>
+      </c>
+      <c r="K35" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L35" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M35" s="8" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="N35" s="8" t="n">
-        <v>-0.0925</v>
+        <v>-0.0294</v>
       </c>
       <c r="O35" s="6" t="n">
-        <v>12.93</v>
+        <v>9.619999999999999</v>
       </c>
       <c r="P35" s="6" t="n">
-        <v>28.7</v>
+        <v>20.2</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="3" t="inlineStr">
         <is>
-          <t>T0024</t>
+          <t>T0020</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
@@ -3580,7 +3580,7 @@
       <c r="J36" s="9" t="n">
         <v>-0.0563</v>
       </c>
-      <c r="K36" s="11" t="inlineStr">
+      <c r="K36" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
@@ -3597,7 +3597,7 @@
         <v>-0.0608</v>
       </c>
       <c r="O36" s="6" t="n">
-        <v>12.53</v>
+        <v>15.98</v>
       </c>
       <c r="P36" s="6" t="n">
         <v>43.3</v>
@@ -3606,22 +3606,22 @@
     <row r="37">
       <c r="A37" s="3" t="inlineStr">
         <is>
-          <t>T0001</t>
+          <t>T0021</t>
         </is>
       </c>
       <c r="B37" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C37" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D37" s="3" t="inlineStr">
         <is>
-          <t>2285</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E37" s="4" t="inlineStr">
@@ -3635,64 +3635,64 @@
         </is>
       </c>
       <c r="G37" s="5" t="n">
-        <v>43.19</v>
+        <v>45.31</v>
       </c>
       <c r="H37" s="5" t="n">
-        <v>43.88</v>
+        <v>43.14</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J37" s="7" t="n">
-        <v>0.016</v>
+        <v>1</v>
+      </c>
+      <c r="J37" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K37" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L37" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M37" s="8" t="n">
-        <v>0.0188</v>
+        <v>0</v>
       </c>
       <c r="N37" s="8" t="n">
-        <v>-0.0016</v>
+        <v>-0.0925</v>
       </c>
       <c r="O37" s="6" t="n">
-        <v>32.16</v>
+        <v>13.05</v>
       </c>
       <c r="P37" s="6" t="n">
-        <v>13</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="3" t="inlineStr">
         <is>
-          <t>T0002</t>
+          <t>T0023</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D38" s="3" t="inlineStr">
         <is>
-          <t>8010</t>
+          <t>2280</t>
         </is>
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F38" s="3" t="inlineStr">
@@ -3701,64 +3701,64 @@
         </is>
       </c>
       <c r="G38" s="5" t="n">
-        <v>137.37</v>
+        <v>45.31</v>
       </c>
       <c r="H38" s="5" t="n">
-        <v>143</v>
+        <v>43.14</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J38" s="7" t="n">
-        <v>0.04099999999999999</v>
+        <v>1</v>
+      </c>
+      <c r="J38" s="9" t="n">
+        <v>-0.0478</v>
       </c>
       <c r="K38" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L38" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M38" s="8" t="n">
-        <v>0.0432</v>
+        <v>0</v>
       </c>
       <c r="N38" s="8" t="n">
-        <v>-0.002</v>
+        <v>-0.0925</v>
       </c>
       <c r="O38" s="6" t="n">
-        <v>30.86</v>
+        <v>12.93</v>
       </c>
       <c r="P38" s="6" t="n">
-        <v>22.9</v>
+        <v>28.7</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="3" t="inlineStr">
         <is>
-          <t>T0003</t>
+          <t>T0024</t>
         </is>
       </c>
       <c r="B39" s="3" t="inlineStr">
         <is>
-          <t>2026-05-07</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="C39" s="3" t="inlineStr">
         <is>
-          <t>2026-05-11</t>
+          <t>2026-05-12</t>
         </is>
       </c>
       <c r="D39" s="3" t="inlineStr">
         <is>
-          <t>8250</t>
+          <t>2370</t>
         </is>
       </c>
       <c r="E39" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>بتروكيماويات</t>
         </is>
       </c>
       <c r="F39" s="3" t="inlineStr">
@@ -3767,44 +3767,44 @@
         </is>
       </c>
       <c r="G39" s="5" t="n">
-        <v>27.31</v>
+        <v>32.56</v>
       </c>
       <c r="H39" s="5" t="n">
-        <v>27.86</v>
+        <v>30.73</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="J39" s="7" t="n">
-        <v>0.0201</v>
+        <v>1</v>
+      </c>
+      <c r="J39" s="9" t="n">
+        <v>-0.0563</v>
       </c>
       <c r="K39" s="10" t="inlineStr">
         <is>
-          <t>TIME_WIN</t>
+          <t>LOSS</t>
         </is>
       </c>
       <c r="L39" s="4" t="inlineStr">
         <is>
-          <t>Max Holding Days Reached</t>
+          <t>Stop Hit</t>
         </is>
       </c>
       <c r="M39" s="8" t="n">
-        <v>0.0392</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="N39" s="8" t="n">
-        <v>-0.0114</v>
+        <v>-0.0608</v>
       </c>
       <c r="O39" s="6" t="n">
-        <v>26.27</v>
+        <v>12.53</v>
       </c>
       <c r="P39" s="6" t="n">
-        <v>23.9</v>
+        <v>43.3</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="3" t="inlineStr">
         <is>
-          <t>T0004</t>
+          <t>T0001</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -3819,12 +3819,12 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>2083</t>
+          <t>2285</t>
         </is>
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
-          <t>مرافق</t>
+          <t>زراعة وأغذية</t>
         </is>
       </c>
       <c r="F40" s="3" t="inlineStr">
@@ -3833,18 +3833,18 @@
         </is>
       </c>
       <c r="G40" s="5" t="n">
-        <v>37.25</v>
+        <v>43.19</v>
       </c>
       <c r="H40" s="5" t="n">
-        <v>38.14</v>
+        <v>43.88</v>
       </c>
       <c r="I40" s="3" t="n">
         <v>5</v>
       </c>
       <c r="J40" s="7" t="n">
-        <v>0.0239</v>
-      </c>
-      <c r="K40" s="10" t="inlineStr">
+        <v>0.016</v>
+      </c>
+      <c r="K40" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -3855,22 +3855,22 @@
         </is>
       </c>
       <c r="M40" s="8" t="n">
-        <v>0.0379</v>
+        <v>0.0188</v>
       </c>
       <c r="N40" s="8" t="n">
-        <v>-0.0212</v>
+        <v>-0.0016</v>
       </c>
       <c r="O40" s="6" t="n">
-        <v>23.8</v>
+        <v>32.16</v>
       </c>
       <c r="P40" s="6" t="n">
-        <v>27.9</v>
+        <v>13</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">
         <is>
-          <t>T0009</t>
+          <t>T0002</t>
         </is>
       </c>
       <c r="B41" s="3" t="inlineStr">
@@ -3885,12 +3885,12 @@
       </c>
       <c r="D41" s="3" t="inlineStr">
         <is>
-          <t>4016</t>
+          <t>8010</t>
         </is>
       </c>
       <c r="E41" s="4" t="inlineStr">
         <is>
-          <t>رعاية صحية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F41" s="3" t="inlineStr">
@@ -3899,20 +3899,20 @@
         </is>
       </c>
       <c r="G41" s="5" t="n">
-        <v>105.01</v>
+        <v>137.37</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>105</v>
+        <v>143</v>
       </c>
       <c r="I41" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="J41" s="9" t="n">
-        <v>-0.0001</v>
+      <c r="J41" s="7" t="n">
+        <v>0.04099999999999999</v>
       </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L41" s="4" t="inlineStr">
@@ -3921,22 +3921,22 @@
         </is>
       </c>
       <c r="M41" s="8" t="n">
-        <v>0.0075</v>
+        <v>0.0432</v>
       </c>
       <c r="N41" s="8" t="n">
-        <v>-0.022</v>
+        <v>-0.002</v>
       </c>
       <c r="O41" s="6" t="n">
-        <v>10.01</v>
+        <v>30.86</v>
       </c>
       <c r="P41" s="6" t="n">
-        <v>17.6</v>
+        <v>22.9</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>T0005</t>
+          <t>T0003</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
@@ -3946,39 +3946,39 @@
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>4145</t>
+          <t>8250</t>
         </is>
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
-          <t>صناعية</t>
+          <t>تأمين</t>
         </is>
       </c>
       <c r="F42" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G42" s="5" t="n">
-        <v>26.25</v>
+        <v>27.31</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>25.64</v>
+        <v>27.86</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>4</v>
-      </c>
-      <c r="J42" s="9" t="n">
-        <v>-0.0232</v>
+        <v>5</v>
+      </c>
+      <c r="J42" s="7" t="n">
+        <v>0.0201</v>
       </c>
       <c r="K42" s="11" t="inlineStr">
         <is>
-          <t>TIME_LOSS</t>
+          <t>TIME_WIN</t>
         </is>
       </c>
       <c r="L42" s="4" t="inlineStr">
@@ -3987,22 +3987,22 @@
         </is>
       </c>
       <c r="M42" s="8" t="n">
-        <v>0.0011</v>
+        <v>0.0392</v>
       </c>
       <c r="N42" s="8" t="n">
-        <v>-0.0316</v>
+        <v>-0.0114</v>
       </c>
       <c r="O42" s="6" t="n">
-        <v>16.26</v>
+        <v>26.27</v>
       </c>
       <c r="P42" s="6" t="n">
-        <v>31.4</v>
+        <v>23.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="3" t="inlineStr">
         <is>
-          <t>T0006</t>
+          <t>T0004</t>
         </is>
       </c>
       <c r="B43" s="3" t="inlineStr">
@@ -4012,37 +4012,37 @@
       </c>
       <c r="C43" s="3" t="inlineStr">
         <is>
-          <t>2026-05-10</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D43" s="3" t="inlineStr">
         <is>
-          <t>8280</t>
+          <t>2083</t>
         </is>
       </c>
       <c r="E43" s="4" t="inlineStr">
         <is>
-          <t>تأمين</t>
+          <t>مرافق</t>
         </is>
       </c>
       <c r="F43" s="3" t="inlineStr">
         <is>
-          <t>support_bounce</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G43" s="5" t="n">
-        <v>10.7</v>
+        <v>37.25</v>
       </c>
       <c r="H43" s="5" t="n">
-        <v>10.73</v>
+        <v>38.14</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J43" s="7" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="K43" s="10" t="inlineStr">
+        <v>0.0239</v>
+      </c>
+      <c r="K43" s="11" t="inlineStr">
         <is>
           <t>TIME_WIN</t>
         </is>
@@ -4053,22 +4053,22 @@
         </is>
       </c>
       <c r="M43" s="8" t="n">
-        <v>0.0168</v>
+        <v>0.0379</v>
       </c>
       <c r="N43" s="8" t="n">
-        <v>-0.009300000000000001</v>
+        <v>-0.0212</v>
       </c>
       <c r="O43" s="6" t="n">
-        <v>12.8</v>
+        <v>23.8</v>
       </c>
       <c r="P43" s="6" t="n">
-        <v>14.8</v>
+        <v>27.9</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="3" t="inlineStr">
         <is>
-          <t>T0007</t>
+          <t>T0009</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -4078,122 +4078,320 @@
       </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
-          <t>2026-05-08</t>
+          <t>2026-05-11</t>
         </is>
       </c>
       <c r="D44" s="3" t="inlineStr">
         <is>
-          <t>4040</t>
+          <t>4016</t>
         </is>
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
-          <t>نقل</t>
+          <t>رعاية صحية</t>
         </is>
       </c>
       <c r="F44" s="3" t="inlineStr">
         <is>
-          <t>default</t>
+          <t>breakout</t>
         </is>
       </c>
       <c r="G44" s="5" t="n">
-        <v>11.92</v>
+        <v>105.01</v>
       </c>
       <c r="H44" s="5" t="n">
-        <v>11.24</v>
+        <v>105</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="J44" s="9" t="n">
-        <v>-0.0568</v>
-      </c>
-      <c r="K44" s="11" t="inlineStr">
-        <is>
-          <t>LOSS</t>
+        <v>-0.0001</v>
+      </c>
+      <c r="K44" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
         </is>
       </c>
       <c r="L44" s="4" t="inlineStr">
         <is>
-          <t>Stop Hit</t>
+          <t>Max Holding Days Reached</t>
         </is>
       </c>
       <c r="M44" s="8" t="n">
-        <v>0</v>
+        <v>0.0075</v>
       </c>
       <c r="N44" s="8" t="n">
-        <v>-0.1015</v>
+        <v>-0.022</v>
       </c>
       <c r="O44" s="6" t="n">
-        <v>12</v>
+        <v>10.01</v>
       </c>
       <c r="P44" s="6" t="n">
-        <v>33.5</v>
+        <v>17.6</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="3" t="inlineStr">
         <is>
+          <t>T0005</t>
+        </is>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C45" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>4145</t>
+        </is>
+      </c>
+      <c r="E45" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G45" s="5" t="n">
+        <v>26.25</v>
+      </c>
+      <c r="H45" s="5" t="n">
+        <v>25.64</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J45" s="9" t="n">
+        <v>-0.0232</v>
+      </c>
+      <c r="K45" s="10" t="inlineStr">
+        <is>
+          <t>TIME_LOSS</t>
+        </is>
+      </c>
+      <c r="L45" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M45" s="8" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="N45" s="8" t="n">
+        <v>-0.0316</v>
+      </c>
+      <c r="O45" s="6" t="n">
+        <v>16.26</v>
+      </c>
+      <c r="P45" s="6" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="3" t="inlineStr">
+        <is>
+          <t>T0006</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-10</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>8280</t>
+        </is>
+      </c>
+      <c r="E46" s="4" t="inlineStr">
+        <is>
+          <t>تأمين</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>support_bounce</t>
+        </is>
+      </c>
+      <c r="G46" s="5" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H46" s="5" t="n">
+        <v>10.73</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="J46" s="7" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="K46" s="11" t="inlineStr">
+        <is>
+          <t>TIME_WIN</t>
+        </is>
+      </c>
+      <c r="L46" s="4" t="inlineStr">
+        <is>
+          <t>Max Holding Days Reached</t>
+        </is>
+      </c>
+      <c r="M46" s="8" t="n">
+        <v>0.0168</v>
+      </c>
+      <c r="N46" s="8" t="n">
+        <v>-0.009300000000000001</v>
+      </c>
+      <c r="O46" s="6" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="P46" s="6" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>T0007</t>
+        </is>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-07</t>
+        </is>
+      </c>
+      <c r="C47" s="3" t="inlineStr">
+        <is>
+          <t>2026-05-08</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>4040</t>
+        </is>
+      </c>
+      <c r="E47" s="4" t="inlineStr">
+        <is>
+          <t>نقل</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>default</t>
+        </is>
+      </c>
+      <c r="G47" s="5" t="n">
+        <v>11.92</v>
+      </c>
+      <c r="H47" s="5" t="n">
+        <v>11.24</v>
+      </c>
+      <c r="I47" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J47" s="9" t="n">
+        <v>-0.0568</v>
+      </c>
+      <c r="K47" s="10" t="inlineStr">
+        <is>
+          <t>LOSS</t>
+        </is>
+      </c>
+      <c r="L47" s="4" t="inlineStr">
+        <is>
+          <t>Stop Hit</t>
+        </is>
+      </c>
+      <c r="M47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="N47" s="8" t="n">
+        <v>-0.1015</v>
+      </c>
+      <c r="O47" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="P47" s="6" t="n">
+        <v>33.5</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="3" t="inlineStr">
+        <is>
           <t>T0008</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B48" s="3" t="inlineStr">
         <is>
           <t>2026-05-07</t>
         </is>
       </c>
-      <c r="C45" s="3" t="inlineStr">
+      <c r="C48" s="3" t="inlineStr">
         <is>
           <t>2026-05-08</t>
         </is>
       </c>
-      <c r="D45" s="3" t="inlineStr">
+      <c r="D48" s="3" t="inlineStr">
         <is>
           <t>2050</t>
         </is>
       </c>
-      <c r="E45" s="4" t="inlineStr">
+      <c r="E48" s="4" t="inlineStr">
         <is>
           <t>بتروكيماويات</t>
         </is>
       </c>
-      <c r="F45" s="3" t="inlineStr">
+      <c r="F48" s="3" t="inlineStr">
         <is>
           <t>support_bounce</t>
         </is>
       </c>
-      <c r="G45" s="5" t="n">
+      <c r="G48" s="5" t="n">
         <v>26.89</v>
       </c>
-      <c r="H45" s="5" t="n">
+      <c r="H48" s="5" t="n">
         <v>25.73</v>
       </c>
-      <c r="I45" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="J45" s="9" t="n">
+      <c r="I48" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J48" s="9" t="n">
         <v>-0.0431</v>
       </c>
-      <c r="K45" s="11" t="inlineStr">
+      <c r="K48" s="10" t="inlineStr">
         <is>
           <t>LOSS</t>
         </is>
       </c>
-      <c r="L45" s="4" t="inlineStr">
+      <c r="L48" s="4" t="inlineStr">
         <is>
           <t>Stop Hit</t>
         </is>
       </c>
-      <c r="M45" s="8" t="n">
+      <c r="M48" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="8" t="n">
+      <c r="N48" s="8" t="n">
         <v>-0.08550000000000001</v>
       </c>
-      <c r="O45" s="6" t="n">
+      <c r="O48" s="6" t="n">
         <v>10.63</v>
       </c>
-      <c r="P45" s="6" t="n">
+      <c r="P48" s="6" t="n">
         <v>30.3</v>
       </c>
     </row>
@@ -4228,7 +4426,7 @@
     <row r="2">
       <c r="A2" s="13" t="inlineStr">
         <is>
-          <t>محسوب في: 2026-06-01T12:31:18</t>
+          <t>محسوب في: 2026-06-02T02:02:34</t>
         </is>
       </c>
     </row>
@@ -4252,7 +4450,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
     </row>
     <row r="6">
@@ -4282,7 +4480,7 @@
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9">
@@ -4293,7 +4491,7 @@
       </c>
       <c r="B9" s="16" t="inlineStr">
         <is>
-          <t>33.3%</t>
+          <t>31.1%</t>
         </is>
       </c>
     </row>
@@ -4317,7 +4515,7 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>-3.61%</t>
+          <t>-3.6%</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4526,7 @@
         </is>
       </c>
       <c r="B12" s="18" t="n">
-        <v>0.68</v>
+        <v>0.62</v>
       </c>
     </row>
     <row r="13">
@@ -4339,7 +4537,7 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>-32.12%</t>
+          <t>-42.42%</t>
         </is>
       </c>
     </row>
@@ -4473,19 +4671,19 @@
         </is>
       </c>
       <c r="B27" s="3" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C27" s="3" t="n">
         <v>11</v>
       </c>
-      <c r="D27" s="3" t="inlineStr">
-        <is>
-          <t>40.7%</t>
+      <c r="D27" s="17" t="inlineStr">
+        <is>
+          <t>36.7%</t>
         </is>
       </c>
       <c r="E27" s="17" t="inlineStr">
         <is>
-          <t>-0.32%</t>
+          <t>-0.63%</t>
         </is>
       </c>
     </row>
@@ -4579,19 +4777,19 @@
         </is>
       </c>
       <c r="B35" s="3" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C35" s="3" t="n">
         <v>2</v>
       </c>
       <c r="D35" s="17" t="inlineStr">
         <is>
-          <t>15.4%</t>
+          <t>14.3%</t>
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr">
         <is>
-          <t>-2.24%</t>
+          <t>-2.30%</t>
         </is>
       </c>
     </row>
@@ -4602,19 +4800,19 @@
         </is>
       </c>
       <c r="B36" s="3" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C36" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="D36" s="16" t="inlineStr">
-        <is>
-          <t>66.7%</t>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>50.0%</t>
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr">
         <is>
-          <t>+4.54%</t>
+          <t>+2.47%</t>
         </is>
       </c>
     </row>
@@ -4717,7 +4915,7 @@
         </is>
       </c>
       <c r="B41" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C41" s="3" t="n">
         <v>0</v>
@@ -4729,7 +4927,7 @@
       </c>
       <c r="E41" s="3" t="inlineStr">
         <is>
-          <t>-0.89%</t>
+          <t>-2.15%</t>
         </is>
       </c>
     </row>
@@ -4888,7 +5086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="35" customWidth="1" min="1" max="1"/>
@@ -6262,6 +6460,129 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" s="3" t="inlineStr">
+        <is>
+          <t>2340</t>
+        </is>
+      </c>
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>بتروكيماويات</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D36" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>-3.16%</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>-3.16%</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>-3.16%</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>4061</t>
+        </is>
+      </c>
+      <c r="B37" s="4" t="inlineStr">
+        <is>
+          <t>تجزئة</t>
+        </is>
+      </c>
+      <c r="C37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D37" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G37" s="3" t="inlineStr">
+        <is>
+          <t>-3.40%</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>-3.40%</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>-3.40%</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="3" t="inlineStr">
+        <is>
+          <t>4170</t>
+        </is>
+      </c>
+      <c r="B38" s="4" t="inlineStr">
+        <is>
+          <t>صناعية</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="D38" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>0.0%</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>-3.74%</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>-3.74%</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>-3.74%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:H1"/>

</xml_diff>